<commit_message>
Fixed packages's properties and constraints
</commit_message>
<xml_diff>
--- a/DW2022/Documentation/Design document.xlsx
+++ b/DW2022/Documentation/Design document.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Llewellyn\Desktop\DW2022_Repo\DW2022\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5D6F8B-2390-447E-8DD2-3F56B87736AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D034EEF9-CF3D-45F4-908E-EE8838FDFD87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" firstSheet="24" activeTab="29" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" firstSheet="22" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Added Updated Design Document
</commit_message>
<xml_diff>
--- a/DW2022/Documentation/Design document.xlsx
+++ b/DW2022/Documentation/Design document.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Llewellyn\Desktop\DW2022_Repo\DW2022\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D034EEF9-CF3D-45F4-908E-EE8838FDFD87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95CC4C66-9355-4515-A285-C3B67DAD7262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" firstSheet="22" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" firstSheet="15" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -25,24 +25,24 @@
     <sheet name="Source Files" sheetId="2" r:id="rId10"/>
     <sheet name="SF_MM_Stock_Take" sheetId="3" r:id="rId11"/>
     <sheet name="Stage1" sheetId="4" r:id="rId12"/>
-    <sheet name="S1_MM_Stock_Take" sheetId="31" r:id="rId13"/>
-    <sheet name="Stage2" sheetId="32" r:id="rId14"/>
-    <sheet name="S2_MM_Material_Group_Lookup" sheetId="33" r:id="rId15"/>
-    <sheet name="S2_MM_Material" sheetId="34" r:id="rId16"/>
-    <sheet name="S2_MM_Stock_Take" sheetId="36" r:id="rId17"/>
-    <sheet name="Process Metadata" sheetId="9" r:id="rId18"/>
-    <sheet name="SF_PW_Customer" sheetId="38" r:id="rId19"/>
-    <sheet name="SF_PW_Customer_Department" sheetId="43" r:id="rId20"/>
-    <sheet name="SF_PW_Customer_Department_Group" sheetId="44" r:id="rId21"/>
-    <sheet name="SF_PW_Employees" sheetId="46" r:id="rId22"/>
-    <sheet name="SF_PW_Employee_Timesheet" sheetId="47" r:id="rId23"/>
-    <sheet name="SF_PW_Internal_Projects" sheetId="50" r:id="rId24"/>
-    <sheet name="S1_PW_Customer" sheetId="40" r:id="rId25"/>
-    <sheet name="S1_PW_Customer_Department" sheetId="41" r:id="rId26"/>
-    <sheet name="S1_PW_Customer_Department_Group" sheetId="42" r:id="rId27"/>
-    <sheet name="S1_PW_Employees" sheetId="49" r:id="rId28"/>
-    <sheet name="S1_PW_Employee_Timesheet" sheetId="48" r:id="rId29"/>
-    <sheet name="S1_PW_Internal_Projects" sheetId="51" r:id="rId30"/>
+    <sheet name="S1_PW_Customer" sheetId="40" r:id="rId13"/>
+    <sheet name="S1_PW_Customer_Department" sheetId="41" r:id="rId14"/>
+    <sheet name="S1_PW_Employees" sheetId="49" r:id="rId15"/>
+    <sheet name="S1_PW_Internal_Projects" sheetId="51" r:id="rId16"/>
+    <sheet name="S1_PW_Employee_Timesheet" sheetId="48" r:id="rId17"/>
+    <sheet name="S1_PW_Customer_Department_Group" sheetId="42" r:id="rId18"/>
+    <sheet name="S1_MM_Stock_Take" sheetId="31" r:id="rId19"/>
+    <sheet name="Stage2" sheetId="32" r:id="rId20"/>
+    <sheet name="S2_MM_Material_Group_Lookup" sheetId="33" r:id="rId21"/>
+    <sheet name="S2_MM_Material" sheetId="34" r:id="rId22"/>
+    <sheet name="S2_MM_Stock_Take" sheetId="36" r:id="rId23"/>
+    <sheet name="Process Metadata" sheetId="9" r:id="rId24"/>
+    <sheet name="SF_PW_Customer" sheetId="38" r:id="rId25"/>
+    <sheet name="SF_PW_Customer_Department" sheetId="43" r:id="rId26"/>
+    <sheet name="SF_PW_Customer_Department_Group" sheetId="44" r:id="rId27"/>
+    <sheet name="SF_PW_Employees" sheetId="46" r:id="rId28"/>
+    <sheet name="SF_PW_Employee_Timesheet" sheetId="47" r:id="rId29"/>
+    <sheet name="SF_PW_Internal_Projects" sheetId="50" r:id="rId30"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId31"/>
@@ -51,13 +51,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Date records'!$A$2:$G$1100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Naming Conventions'!$A$28:$C$28</definedName>
     <definedName name="LU_DOW" localSheetId="3">#REF!</definedName>
-    <definedName name="LU_DOW" localSheetId="12">#REF!</definedName>
-    <definedName name="LU_DOW" localSheetId="15">#REF!</definedName>
-    <definedName name="LU_DOW" localSheetId="14">#REF!</definedName>
-    <definedName name="LU_DOW" localSheetId="16">#REF!</definedName>
+    <definedName name="LU_DOW" localSheetId="18">#REF!</definedName>
+    <definedName name="LU_DOW" localSheetId="21">#REF!</definedName>
+    <definedName name="LU_DOW" localSheetId="20">#REF!</definedName>
     <definedName name="LU_DOW" localSheetId="22">#REF!</definedName>
-    <definedName name="LU_DOW" localSheetId="21">#REF!</definedName>
-    <definedName name="LU_DOW" localSheetId="13">#REF!</definedName>
+    <definedName name="LU_DOW" localSheetId="28">#REF!</definedName>
+    <definedName name="LU_DOW" localSheetId="27">#REF!</definedName>
+    <definedName name="LU_DOW" localSheetId="19">#REF!</definedName>
     <definedName name="LU_DOW" localSheetId="8">#REF!</definedName>
     <definedName name="LU_DOW">#REF!</definedName>
     <definedName name="the_date">'[1]Calendar Day'!$A$31</definedName>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1786" uniqueCount="785">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1843" uniqueCount="808">
   <si>
     <t>Source Files</t>
   </si>
@@ -2283,15 +2283,15 @@
     <t>E_Hours</t>
   </si>
   <si>
+    <t>decimal(4,4)</t>
+  </si>
+  <si>
     <t>NULL VALUE Replacement</t>
   </si>
   <si>
     <t>Error if null: do not insert, write our error</t>
   </si>
   <si>
-    <t>*Unknown Week End Year</t>
-  </si>
-  <si>
     <t>nvarchar(7)</t>
   </si>
   <si>
@@ -2403,9 +2403,6 @@
     <t>IP_Request_Date</t>
   </si>
   <si>
-    <t>*Unknown Request Date</t>
-  </si>
-  <si>
     <t>IP_Customer_ID</t>
   </si>
   <si>
@@ -2436,21 +2433,12 @@
     <t>decimal(38,4)</t>
   </si>
   <si>
-    <t>*Unknown Labour Costs</t>
-  </si>
-  <si>
     <t>IP_Material_Costs</t>
   </si>
   <si>
-    <t>*Unknown Material Costs</t>
-  </si>
-  <si>
     <t>IP_Handling_Fee</t>
   </si>
   <si>
-    <t>*Unknown Handling Fee</t>
-  </si>
-  <si>
     <t>IP_Service_Billing_Number</t>
   </si>
   <si>
@@ -2461,6 +2449,87 @@
   </si>
   <si>
     <t>SF_PW_Internal_Projects</t>
+  </si>
+  <si>
+    <t>Customer.csv</t>
+  </si>
+  <si>
+    <t>Employees.csv</t>
+  </si>
+  <si>
+    <t>Customer_Department.csv</t>
+  </si>
+  <si>
+    <t>Customer_Department_Group.csv</t>
+  </si>
+  <si>
+    <t>Employee_Timesheet.csv</t>
+  </si>
+  <si>
+    <t>Internal_Projects.csv</t>
+  </si>
+  <si>
+    <t>Instrument Makers customer information worksheets (Excel)</t>
+  </si>
+  <si>
+    <t>Instrument Makers employees information worksheets (Excel)</t>
+  </si>
+  <si>
+    <t>Instrument Makers customer department information worksheets (Excel)</t>
+  </si>
+  <si>
+    <t>Instrument Makers employee timesheet information worksheets (Excel)</t>
+  </si>
+  <si>
+    <t>Instrument Makers customer department group information worksheets (Excel)</t>
+  </si>
+  <si>
+    <t>Instrument Makers internal projects worksheets (Excel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer information. </t>
+  </si>
+  <si>
+    <t>Customer department information</t>
+  </si>
+  <si>
+    <t>Customer department group information</t>
+  </si>
+  <si>
+    <t>Employees information</t>
+  </si>
+  <si>
+    <t>Employee timesheet information</t>
+  </si>
+  <si>
+    <t>Internal projects</t>
+  </si>
+  <si>
+    <t>Department of internal and external or private customers</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>IP</t>
+  </si>
+  <si>
+    <t>Department group of internal and external or private customers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employee information </t>
+  </si>
+  <si>
+    <t>Employee timesheet</t>
+  </si>
+  <si>
+    <t>Internal project information</t>
   </si>
 </sst>
 </file>
@@ -6740,7 +6809,7 @@
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
@@ -6783,7 +6852,7 @@
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C27" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.3">
@@ -6862,11 +6931,11 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="35.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.44140625" style="4" customWidth="1"/>
     <col min="4" max="4" width="63.5546875" style="3" customWidth="1"/>
     <col min="5" max="5" width="52.6640625" style="3" bestFit="1" customWidth="1"/>
@@ -6912,10 +6981,118 @@
         <v>162</v>
       </c>
     </row>
+    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>787</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>793</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>789</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>791</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>788</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>790</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>792</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
     <hyperlink ref="A3" location="SF_MM_Stock_Take!A1" display="SF_MM_Stock_Take" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="A4" location="SF_PW_Customer!A1" display="SF_PW_Customer" xr:uid="{03E53109-940E-43DA-87F1-274A8331958E}"/>
+    <hyperlink ref="A5" location="SF_PW_Customer_Department!A1" display="SF_PW_Customer_Department" xr:uid="{202DDCDB-F5B6-451B-A7DD-E51C91A20AD1}"/>
+    <hyperlink ref="A6" location="SF_PW_Customer_Department_Group!A1" display="SF_PW_Customer_Department_Group" xr:uid="{944A5AA1-F7BF-40EA-98B4-7ADF73C52AE8}"/>
+    <hyperlink ref="A7" location="SF_PW_Employees!A1" display="SF_PW_Employees" xr:uid="{65802583-25D6-49D5-9195-7C585BD9E016}"/>
+    <hyperlink ref="A8" location="SF_PW_Employee_Timesheet!A1" display="SF_PW_Employee_Timesheet" xr:uid="{3EFFFAD2-94E8-452A-87EA-6E34C50669A0}"/>
+    <hyperlink ref="A9" location="SF_PW_Internal_Projects!A1" display="SF_Internal_Projects" xr:uid="{35006256-C4B8-4453-A4E8-70A103E1368C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -7415,14 +7592,14 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.33203125" customWidth="1"/>
+    <col min="1" max="1" width="35.44140625" customWidth="1"/>
     <col min="2" max="2" width="69.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.88671875" customWidth="1"/>
     <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7521,179 +7698,1415 @@
         <v>651</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="142" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>674</v>
+      </c>
+      <c r="B12" t="s">
+        <v>799</v>
+      </c>
+      <c r="C12" t="s">
+        <v>274</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="F12" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="B13" t="s">
+        <v>804</v>
+      </c>
+      <c r="C13" t="s">
+        <v>274</v>
+      </c>
+      <c r="D13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="F13" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="B14" t="s">
+        <v>805</v>
+      </c>
+      <c r="C14" t="s">
+        <v>274</v>
+      </c>
+      <c r="D14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>700</v>
+      </c>
+      <c r="B15" t="s">
+        <v>806</v>
+      </c>
+      <c r="C15" t="s">
+        <v>274</v>
+      </c>
+      <c r="D15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="F15" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>779</v>
+      </c>
+      <c r="B16" t="s">
+        <v>807</v>
+      </c>
+      <c r="C16" t="s">
+        <v>274</v>
+      </c>
+      <c r="D16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="F16" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="142" t="s">
         <v>486</v>
       </c>
-      <c r="B13" s="142"/>
-      <c r="C13" s="142"/>
-      <c r="D13" s="142"/>
-      <c r="E13" s="142"/>
-      <c r="F13" s="142"/>
-    </row>
-    <row r="14" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
+      <c r="B18" s="142"/>
+      <c r="C18" s="142"/>
+      <c r="D18" s="142"/>
+      <c r="E18" s="142"/>
+      <c r="F18" s="142"/>
+    </row>
+    <row r="19" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B19" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="141" t="s">
+      <c r="C19" s="141" t="s">
         <v>471</v>
-      </c>
-      <c r="D14" s="141"/>
-      <c r="E14" s="141"/>
-      <c r="F14" s="12"/>
-    </row>
-    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>473</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="C15" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>474</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>535</v>
-      </c>
-      <c r="C16" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="143" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="143"/>
-      <c r="C18" s="143"/>
-      <c r="D18" s="143"/>
-      <c r="E18" s="143"/>
-      <c r="F18" s="143"/>
-    </row>
-    <row r="19" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="141" t="s">
-        <v>483</v>
       </c>
       <c r="D19" s="141"/>
       <c r="E19" s="141"/>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="12"/>
+    </row>
+    <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>473</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C20" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>474</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="C21" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="143" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="143"/>
+      <c r="C23" s="143"/>
+      <c r="D23" s="143"/>
+      <c r="E23" s="143"/>
+      <c r="F23" s="143"/>
+    </row>
+    <row r="24" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="141" t="s">
+        <v>483</v>
+      </c>
+      <c r="D24" s="141"/>
+      <c r="E24" s="141"/>
+      <c r="F24" s="8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B25" t="s">
         <v>33</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C25" t="s">
         <v>34</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+    <row r="26" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B26" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F26" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+    <row r="27" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B27" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F27" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="143" t="s">
+    <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="143" t="s">
         <v>469</v>
       </c>
-      <c r="B24" s="143"/>
-      <c r="C24" s="143"/>
-      <c r="D24" s="143"/>
-      <c r="E24" s="143"/>
-      <c r="F24" s="143"/>
-    </row>
-    <row r="25" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
+      <c r="B29" s="143"/>
+      <c r="C29" s="143"/>
+      <c r="D29" s="143"/>
+      <c r="E29" s="143"/>
+      <c r="F29" s="143"/>
+    </row>
+    <row r="30" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B30" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="141" t="s">
+      <c r="C30" s="141" t="s">
         <v>471</v>
       </c>
-      <c r="D25" s="141"/>
-      <c r="E25" s="141"/>
-      <c r="F25" s="8"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="D30" s="141"/>
+      <c r="E30" s="141"/>
+      <c r="F30" s="8"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B31" t="s">
         <v>470</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C31" t="s">
         <v>25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="C19:E19"/>
     <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="A29:F29"/>
     <mergeCell ref="A18:F18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A13:F13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
-    <hyperlink ref="A20" location="'Process Metadata'!A5" display="Import_Batch" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
-    <hyperlink ref="A21" location="'Process Metadata'!A16" display="Import_Batch_Process" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
-    <hyperlink ref="A22" location="'Process Metadata'!A25" display="Import_Batch_Process_Task" xr:uid="{00000000-0004-0000-0500-000003000000}"/>
+    <hyperlink ref="A25" location="'Process Metadata'!A5" display="Import_Batch" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
+    <hyperlink ref="A26" location="'Process Metadata'!A16" display="Import_Batch_Process" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
+    <hyperlink ref="A27" location="'Process Metadata'!A25" display="Import_Batch_Process_Task" xr:uid="{00000000-0004-0000-0500-000003000000}"/>
     <hyperlink ref="A10" location="S1_MM_Stock_Take!A1" display="S1_MM_Stock_Take!A1" xr:uid="{00000000-0004-0000-0500-000004000000}"/>
     <hyperlink ref="E10" location="SF_MM_Stock_Take!A1" display="SF_MM_Stock_Take" xr:uid="{00000000-0004-0000-0500-000005000000}"/>
-    <hyperlink ref="A26" location="'Process Metadata'!J5" display="V_IB_Latest" xr:uid="{00000000-0004-0000-0500-000006000000}"/>
+    <hyperlink ref="A31" location="'Process Metadata'!J5" display="V_IB_Latest" xr:uid="{00000000-0004-0000-0500-000006000000}"/>
+    <hyperlink ref="A12" location="S1_PW_Customer_Department!A1" display="S1_PW_Customer_Department" xr:uid="{7D25CD5C-119C-4698-9B1E-1A696EBBFB10}"/>
+    <hyperlink ref="A13" location="S1_PW_Customer_Department_Group!A1" display="S1_PW_Customer_Department_Group" xr:uid="{A617B09F-DC09-43F8-B46E-FDCB95814890}"/>
+    <hyperlink ref="A14" location="S1_PW_Employees!A1" display="S1_PW_Employees" xr:uid="{C1D0349A-5B61-4401-AE28-0E65E620A539}"/>
+    <hyperlink ref="A15" location="S1_PW_Employee_Timesheet!A1" display="S1_PW_Employee_Timesheet" xr:uid="{A5133407-A6AF-4A94-B8EC-31D643827EB2}"/>
+    <hyperlink ref="A16" location="S1_PW_Internal_Projects!A1" display="S1_PW_Internal_Projects" xr:uid="{569DF9AD-0178-44DC-A60B-CB5550C7E54E}"/>
+    <hyperlink ref="E12" location="SF_PW_Customer_Department!A1" display="SF_PW_Customer_Department" xr:uid="{B92CFB15-7D55-42B2-BB57-467A4E0C110E}"/>
+    <hyperlink ref="E13" location="SF_PW_Customer_Department_Group!A1" display="SF_PW_Customer_Department_Group" xr:uid="{57809120-193A-49A5-BDB9-C9EDA20AAA85}"/>
+    <hyperlink ref="E14" location="SF_PW_Employees!A1" display="SF_PW_Employees" xr:uid="{0E91F5A0-20A9-4E95-9A55-E0C8868FB127}"/>
+    <hyperlink ref="E15" location="SF_PW_Employee_Timesheet!A1" display="SF_PW_Employee_Timesheet" xr:uid="{CE52C8F4-C200-4F2B-A827-F5354AD98C00}"/>
+    <hyperlink ref="E16" location="SF_PW_Internal_Projects!A1" display="SF_Internal_Projects" xr:uid="{AC0BAF01-06A5-410C-A739-67113F97044D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7303D0-EAFB-485D-9ED0-6CB8F8BFE263}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="73.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="44.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="85"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C2" s="85"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="126" t="s">
+        <v>652</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D4" s="127" t="s">
+        <v>662</v>
+      </c>
+      <c r="E4" t="s">
+        <v>635</v>
+      </c>
+      <c r="F4" t="s">
+        <v>636</v>
+      </c>
+      <c r="G4" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="126" t="s">
+        <v>653</v>
+      </c>
+      <c r="B5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" t="s">
+        <v>135</v>
+      </c>
+      <c r="E5" t="s">
+        <v>669</v>
+      </c>
+      <c r="F5" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="126" t="s">
+        <v>654</v>
+      </c>
+      <c r="B6" t="s">
+        <v>660</v>
+      </c>
+      <c r="C6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D6" t="s">
+        <v>663</v>
+      </c>
+      <c r="E6" t="s">
+        <v>641</v>
+      </c>
+      <c r="F6" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="126" t="s">
+        <v>655</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>156</v>
+      </c>
+      <c r="D7" t="s">
+        <v>664</v>
+      </c>
+      <c r="E7" t="s">
+        <v>642</v>
+      </c>
+      <c r="F7" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="126" t="s">
+        <v>656</v>
+      </c>
+      <c r="B8" t="s">
+        <v>660</v>
+      </c>
+      <c r="C8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D8" t="s">
+        <v>665</v>
+      </c>
+      <c r="E8" s="126" t="s">
+        <v>643</v>
+      </c>
+      <c r="F8" s="126" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="126" t="s">
+        <v>657</v>
+      </c>
+      <c r="B9" t="s">
+        <v>660</v>
+      </c>
+      <c r="C9" t="s">
+        <v>156</v>
+      </c>
+      <c r="D9" t="s">
+        <v>666</v>
+      </c>
+      <c r="E9" s="126" t="s">
+        <v>670</v>
+      </c>
+      <c r="F9" s="126" t="s">
+        <v>665</v>
+      </c>
+      <c r="G9" s="126" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="126" t="s">
+        <v>658</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>156</v>
+      </c>
+      <c r="D10" t="s">
+        <v>667</v>
+      </c>
+      <c r="E10" s="126" t="s">
+        <v>644</v>
+      </c>
+      <c r="F10" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="126" t="s">
+        <v>659</v>
+      </c>
+      <c r="B11" t="s">
+        <v>661</v>
+      </c>
+      <c r="C11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D11" t="s">
+        <v>668</v>
+      </c>
+      <c r="E11" s="128">
+        <v>1200</v>
+      </c>
+      <c r="F11" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="126" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>156</v>
+      </c>
+      <c r="E12" s="85">
+        <v>1</v>
+      </c>
+      <c r="F12" s="85">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>673</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="19" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{7348AD42-28E1-48B7-8921-A82010335EB1}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F912F66-4428-47A9-8ADF-02B84F72CE81}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="85"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C2" s="85"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>684</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D4" t="s">
+        <v>662</v>
+      </c>
+      <c r="E4" t="s">
+        <v>638</v>
+      </c>
+      <c r="F4" t="s">
+        <v>681</v>
+      </c>
+      <c r="G4" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>685</v>
+      </c>
+      <c r="B5" t="s">
+        <v>687</v>
+      </c>
+      <c r="C5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" t="s">
+        <v>688</v>
+      </c>
+      <c r="E5" t="s">
+        <v>679</v>
+      </c>
+      <c r="F5" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>686</v>
+      </c>
+      <c r="B6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E6" t="s">
+        <v>680</v>
+      </c>
+      <c r="F6" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="126" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>156</v>
+      </c>
+      <c r="E7" s="85">
+        <v>1</v>
+      </c>
+      <c r="F7" s="85">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>673</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{8C3A7BBF-C04F-4B51-8B78-A0B63181F044}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5C07CAD-3831-4F85-9B1D-4C30D19E9E25}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="83.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="85"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C2" s="85"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>706</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" t="s">
+        <v>662</v>
+      </c>
+      <c r="E4" s="85" t="s">
+        <v>707</v>
+      </c>
+      <c r="F4" s="85" t="s">
+        <v>708</v>
+      </c>
+      <c r="G4" s="130" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>709</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" t="s">
+        <v>734</v>
+      </c>
+      <c r="E5" s="85" t="s">
+        <v>710</v>
+      </c>
+      <c r="F5" s="85" t="s">
+        <v>711</v>
+      </c>
+      <c r="G5" s="89"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>712</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" t="s">
+        <v>735</v>
+      </c>
+      <c r="E6" s="85" t="s">
+        <v>710</v>
+      </c>
+      <c r="F6" s="85" t="s">
+        <v>713</v>
+      </c>
+      <c r="G6" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>731</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="85" t="s">
+        <v>732</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="85">
+        <v>1</v>
+      </c>
+      <c r="F7" s="85">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="9"/>
+      <c r="C8" s="2"/>
+      <c r="E8" s="85"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="C9" s="2"/>
+      <c r="E9" s="85"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="9"/>
+      <c r="C10" s="2"/>
+      <c r="E10" s="85"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="9"/>
+      <c r="C11" s="2"/>
+      <c r="E11" s="85"/>
+      <c r="F11" s="85"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="9"/>
+      <c r="C12" s="85"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="85"/>
+      <c r="F12" s="85"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{DFFCEDC5-B5CD-4533-A52E-9F627F0A2FDF}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68F1906F-3F21-4ADD-B43B-A77686F8C5F2}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr defaultColWidth="23.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="55.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="139"/>
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="139"/>
+      <c r="I2" s="139"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="140" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="137" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="137" t="s">
+        <v>465</v>
+      </c>
+      <c r="D3" s="137" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="137" t="s">
+        <v>762</v>
+      </c>
+      <c r="F3" s="137" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="137" t="s">
+        <v>256</v>
+      </c>
+      <c r="H3" s="137" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="134" t="s">
+        <v>763</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" t="s">
+        <v>662</v>
+      </c>
+      <c r="F4" t="s">
+        <v>744</v>
+      </c>
+      <c r="G4" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="135" t="s">
+        <v>764</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="129">
+        <v>43872</v>
+      </c>
+      <c r="F5" s="129">
+        <v>43849</v>
+      </c>
+      <c r="G5" s="129">
+        <v>43853</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="135" t="s">
+        <v>765</v>
+      </c>
+      <c r="B6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
+        <v>135</v>
+      </c>
+      <c r="F6" t="s">
+        <v>758</v>
+      </c>
+      <c r="G6" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="135" t="s">
+        <v>766</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" t="s">
+        <v>767</v>
+      </c>
+      <c r="F7" t="s">
+        <v>748</v>
+      </c>
+      <c r="G7" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="135" t="s">
+        <v>768</v>
+      </c>
+      <c r="B8" t="s">
+        <v>769</v>
+      </c>
+      <c r="E8" t="s">
+        <v>770</v>
+      </c>
+      <c r="F8" t="s">
+        <v>759</v>
+      </c>
+      <c r="G8" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="135" t="s">
+        <v>771</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="135" t="s">
+        <v>773</v>
+      </c>
+      <c r="B10" t="s">
+        <v>774</v>
+      </c>
+      <c r="E10" t="s">
+        <v>326</v>
+      </c>
+      <c r="F10" s="85">
+        <v>12530</v>
+      </c>
+      <c r="G10" s="85">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="135" t="s">
+        <v>775</v>
+      </c>
+      <c r="B11" t="s">
+        <v>774</v>
+      </c>
+      <c r="E11" t="s">
+        <v>326</v>
+      </c>
+      <c r="F11" s="85">
+        <v>5360</v>
+      </c>
+      <c r="G11" s="85">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="135" t="s">
+        <v>776</v>
+      </c>
+      <c r="B12" t="s">
+        <v>774</v>
+      </c>
+      <c r="E12" t="s">
+        <v>326</v>
+      </c>
+      <c r="F12" s="85">
+        <v>1340</v>
+      </c>
+      <c r="G12" s="85">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="136" t="s">
+        <v>777</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="E13" t="s">
+        <v>778</v>
+      </c>
+      <c r="F13" s="85">
+        <v>5127095</v>
+      </c>
+      <c r="G13" s="85">
+        <v>4604041</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="139" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="85">
+        <v>1</v>
+      </c>
+      <c r="G14" s="85">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{70A1E038-0C96-4A41-9912-DEEE86C5416F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CBF657F-107F-4D04-A554-8C4B6A024335}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="85"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C2" s="85"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>714</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" t="s">
+        <v>662</v>
+      </c>
+      <c r="E4" s="85">
+        <v>2019</v>
+      </c>
+      <c r="F4" s="85">
+        <v>2019</v>
+      </c>
+      <c r="G4" s="130" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>715</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="85">
+        <v>0</v>
+      </c>
+      <c r="E5" s="85">
+        <v>36</v>
+      </c>
+      <c r="F5" s="85">
+        <v>47</v>
+      </c>
+      <c r="G5" s="89"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>716</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="129">
+        <v>43872</v>
+      </c>
+      <c r="E6" s="129">
+        <v>43714</v>
+      </c>
+      <c r="F6" s="129">
+        <v>43791</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>717</v>
+      </c>
+      <c r="B7" t="s">
+        <v>728</v>
+      </c>
+      <c r="C7" s="85"/>
+      <c r="D7" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="E7" t="s">
+        <v>719</v>
+      </c>
+      <c r="F7" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>721</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" t="s">
+        <v>730</v>
+      </c>
+      <c r="E8" t="s">
+        <v>722</v>
+      </c>
+      <c r="F8" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>724</v>
+      </c>
+      <c r="B9" t="s">
+        <v>725</v>
+      </c>
+      <c r="D9" s="85">
+        <v>0</v>
+      </c>
+      <c r="E9" s="85">
+        <v>0.5</v>
+      </c>
+      <c r="F9" s="85">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>731</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="85" t="s">
+        <v>732</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="85">
+        <v>1</v>
+      </c>
+      <c r="F10" s="85">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>733</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{61D2137B-2D94-4C63-851E-29BA389C2F89}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81DFFCD9-6E0D-46F7-A5D0-F21B460087EE}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="44.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="85"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C2" s="85"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>696</v>
+      </c>
+      <c r="B4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" t="s">
+        <v>662</v>
+      </c>
+      <c r="E4" t="s">
+        <v>680</v>
+      </c>
+      <c r="F4" t="s">
+        <v>683</v>
+      </c>
+      <c r="G4" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>697</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="127" t="s">
+        <v>662</v>
+      </c>
+      <c r="E5" t="s">
+        <v>692</v>
+      </c>
+      <c r="F5" t="s">
+        <v>694</v>
+      </c>
+      <c r="G5" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>698</v>
+      </c>
+      <c r="B6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="127" t="s">
+        <v>662</v>
+      </c>
+      <c r="E6" t="s">
+        <v>693</v>
+      </c>
+      <c r="F6" t="s">
+        <v>695</v>
+      </c>
+      <c r="G6" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="126" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="85">
+        <v>1</v>
+      </c>
+      <c r="F7" s="85">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>673</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{AB308857-2754-4349-AD90-AE62710AED13}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -8286,7 +9699,270 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:C35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" style="111" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="62.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="112" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="113" t="s">
+        <v>260</v>
+      </c>
+      <c r="C3" s="114" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="116" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" s="117" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="112" t="s">
+        <v>577</v>
+      </c>
+      <c r="B6" s="113" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" s="114" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="116" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="117" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="112" t="s">
+        <v>580</v>
+      </c>
+      <c r="B9" s="113" t="s">
+        <v>260</v>
+      </c>
+      <c r="C9" s="114" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="116" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="117" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="112" t="s">
+        <v>261</v>
+      </c>
+      <c r="B12" s="113" t="s">
+        <v>262</v>
+      </c>
+      <c r="C12" s="114" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="118" t="s">
+        <v>594</v>
+      </c>
+      <c r="C13" s="119" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="118" t="s">
+        <v>264</v>
+      </c>
+      <c r="C14" s="119" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="116" t="s">
+        <v>459</v>
+      </c>
+      <c r="C15" s="117" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="112" t="s">
+        <v>477</v>
+      </c>
+      <c r="B17" s="113" t="s">
+        <v>262</v>
+      </c>
+      <c r="C17" s="114" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="118" t="s">
+        <v>594</v>
+      </c>
+      <c r="C18" s="119" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="118" t="s">
+        <v>264</v>
+      </c>
+      <c r="C19" s="119" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="116" t="s">
+        <v>459</v>
+      </c>
+      <c r="C20" s="117" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="112" t="s">
+        <v>602</v>
+      </c>
+      <c r="B22" s="113" t="s">
+        <v>262</v>
+      </c>
+      <c r="C22" s="114" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="77" t="s">
+        <v>603</v>
+      </c>
+      <c r="B23" s="118" t="s">
+        <v>594</v>
+      </c>
+      <c r="C23" s="119" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="118" t="s">
+        <v>583</v>
+      </c>
+      <c r="C24" s="119" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="118" t="s">
+        <v>585</v>
+      </c>
+      <c r="C25" s="119" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="116" t="s">
+        <v>459</v>
+      </c>
+      <c r="C26" s="117" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="112" t="s">
+        <v>266</v>
+      </c>
+      <c r="B28" s="120" t="s">
+        <v>128</v>
+      </c>
+      <c r="C28" s="121" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="124" t="s">
+        <v>623</v>
+      </c>
+      <c r="C29" s="125" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="116" t="s">
+        <v>589</v>
+      </c>
+      <c r="C30" s="117" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="112" t="s">
+        <v>588</v>
+      </c>
+      <c r="B32" s="113" t="s">
+        <v>590</v>
+      </c>
+      <c r="C32" s="114" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="118" t="s">
+        <v>592</v>
+      </c>
+      <c r="C33" s="119" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="118" t="s">
+        <v>598</v>
+      </c>
+      <c r="C34" s="119" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="116" t="s">
+        <v>600</v>
+      </c>
+      <c r="C35" s="117" t="s">
+        <v>601</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -8582,7 +10258,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -8836,7 +10512,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -9206,7 +10882,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -9637,7 +11313,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -10128,7 +11804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F53ACD6D-1CA9-4DB0-842E-608E26D26789}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -10353,270 +12029,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
-  <dimension ref="A1:C35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" style="111" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="62.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="112" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="113" t="s">
-        <v>260</v>
-      </c>
-      <c r="C3" s="114" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="116" t="s">
-        <v>128</v>
-      </c>
-      <c r="C4" s="117" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="112" t="s">
-        <v>577</v>
-      </c>
-      <c r="B6" s="113" t="s">
-        <v>260</v>
-      </c>
-      <c r="C6" s="114" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="116" t="s">
-        <v>128</v>
-      </c>
-      <c r="C7" s="117" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="112" t="s">
-        <v>580</v>
-      </c>
-      <c r="B9" s="113" t="s">
-        <v>260</v>
-      </c>
-      <c r="C9" s="114" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="116" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" s="117" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="112" t="s">
-        <v>261</v>
-      </c>
-      <c r="B12" s="113" t="s">
-        <v>262</v>
-      </c>
-      <c r="C12" s="114" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="118" t="s">
-        <v>594</v>
-      </c>
-      <c r="C13" s="119" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="118" t="s">
-        <v>264</v>
-      </c>
-      <c r="C14" s="119" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="116" t="s">
-        <v>459</v>
-      </c>
-      <c r="C15" s="117" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="112" t="s">
-        <v>477</v>
-      </c>
-      <c r="B17" s="113" t="s">
-        <v>262</v>
-      </c>
-      <c r="C17" s="114" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="118" t="s">
-        <v>594</v>
-      </c>
-      <c r="C18" s="119" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="118" t="s">
-        <v>264</v>
-      </c>
-      <c r="C19" s="119" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="116" t="s">
-        <v>459</v>
-      </c>
-      <c r="C20" s="117" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="112" t="s">
-        <v>602</v>
-      </c>
-      <c r="B22" s="113" t="s">
-        <v>262</v>
-      </c>
-      <c r="C22" s="114" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="77" t="s">
-        <v>603</v>
-      </c>
-      <c r="B23" s="118" t="s">
-        <v>594</v>
-      </c>
-      <c r="C23" s="119" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="118" t="s">
-        <v>583</v>
-      </c>
-      <c r="C24" s="119" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="118" t="s">
-        <v>585</v>
-      </c>
-      <c r="C25" s="119" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="116" t="s">
-        <v>459</v>
-      </c>
-      <c r="C26" s="117" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="112" t="s">
-        <v>266</v>
-      </c>
-      <c r="B28" s="120" t="s">
-        <v>128</v>
-      </c>
-      <c r="C28" s="121" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="124" t="s">
-        <v>623</v>
-      </c>
-      <c r="C29" s="125" t="s">
-        <v>624</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="116" t="s">
-        <v>589</v>
-      </c>
-      <c r="C30" s="117" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="112" t="s">
-        <v>588</v>
-      </c>
-      <c r="B32" s="113" t="s">
-        <v>590</v>
-      </c>
-      <c r="C32" s="114" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="118" t="s">
-        <v>592</v>
-      </c>
-      <c r="C33" s="119" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" s="77" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="118" t="s">
-        <v>598</v>
-      </c>
-      <c r="C34" s="119" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="116" t="s">
-        <v>600</v>
-      </c>
-      <c r="C35" s="117" t="s">
-        <v>601</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33BE34B8-8218-4781-961D-6580DD97671B}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -10740,7 +12153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B558D092-5AD7-4F32-8C6F-DC10DA3F7A5D}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -10864,7 +12277,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{967457EE-6E3E-4E8A-8269-85B7705D1CFD}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -11019,7 +12432,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32B6B9E6-C074-45FB-88DC-1F378DA8C765}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -11190,7 +12603,7 @@
         <v>724</v>
       </c>
       <c r="B8" t="s">
-        <v>775</v>
+        <v>725</v>
       </c>
       <c r="E8" t="s">
         <v>346</v>
@@ -11208,1150 +12621,6 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{62B20555-F67B-4F27-B967-0C0ECDBD246E}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6F5B38-E122-44E0-98B8-6AC4250F1F30}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
-  <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" customWidth="1"/>
-    <col min="7" max="7" width="55.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="42.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="137" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="138" t="s">
-        <v>739</v>
-      </c>
-      <c r="C3" s="137" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="137" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="138" t="s">
-        <v>625</v>
-      </c>
-      <c r="F3" s="138" t="s">
-        <v>740</v>
-      </c>
-      <c r="G3" s="137" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="137" t="s">
-        <v>256</v>
-      </c>
-      <c r="I3" s="137" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="134" t="s">
-        <v>741</v>
-      </c>
-      <c r="B4" t="s">
-        <v>210</v>
-      </c>
-      <c r="D4" t="s">
-        <v>742</v>
-      </c>
-      <c r="E4" t="s">
-        <v>743</v>
-      </c>
-      <c r="F4" t="s">
-        <v>743</v>
-      </c>
-      <c r="G4" t="s">
-        <v>744</v>
-      </c>
-      <c r="H4" t="s">
-        <v>745</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="135" t="s">
-        <v>746</v>
-      </c>
-      <c r="B5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" t="s">
-        <v>743</v>
-      </c>
-      <c r="F5" t="s">
-        <v>742</v>
-      </c>
-      <c r="G5" s="129">
-        <v>43849</v>
-      </c>
-      <c r="H5" s="129">
-        <v>43853</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="135" t="s">
-        <v>627</v>
-      </c>
-      <c r="B6" t="s">
-        <v>210</v>
-      </c>
-      <c r="E6" t="s">
-        <v>743</v>
-      </c>
-      <c r="F6" t="s">
-        <v>743</v>
-      </c>
-      <c r="G6" t="s">
-        <v>758</v>
-      </c>
-      <c r="H6" t="s">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="135" t="s">
-        <v>747</v>
-      </c>
-      <c r="B7" t="s">
-        <v>211</v>
-      </c>
-      <c r="E7" t="s">
-        <v>742</v>
-      </c>
-      <c r="F7" t="s">
-        <v>742</v>
-      </c>
-      <c r="G7" t="s">
-        <v>748</v>
-      </c>
-      <c r="H7" t="s">
-        <v>749</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="135" t="s">
-        <v>750</v>
-      </c>
-      <c r="B8" t="s">
-        <v>751</v>
-      </c>
-      <c r="E8" t="s">
-        <v>743</v>
-      </c>
-      <c r="F8" t="s">
-        <v>742</v>
-      </c>
-      <c r="G8" t="s">
-        <v>759</v>
-      </c>
-      <c r="H8" t="s">
-        <v>761</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="135" t="s">
-        <v>752</v>
-      </c>
-      <c r="B9" t="s">
-        <v>211</v>
-      </c>
-      <c r="E9" t="s">
-        <v>742</v>
-      </c>
-      <c r="F9" t="s">
-        <v>742</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="135" t="s">
-        <v>753</v>
-      </c>
-      <c r="B10" t="s">
-        <v>754</v>
-      </c>
-      <c r="E10" t="s">
-        <v>742</v>
-      </c>
-      <c r="F10" t="s">
-        <v>742</v>
-      </c>
-      <c r="G10" s="85">
-        <v>12530</v>
-      </c>
-      <c r="H10" s="85">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="135" t="s">
-        <v>755</v>
-      </c>
-      <c r="B11" t="s">
-        <v>754</v>
-      </c>
-      <c r="E11" t="s">
-        <v>742</v>
-      </c>
-      <c r="F11" t="s">
-        <v>742</v>
-      </c>
-      <c r="G11" s="85">
-        <v>5360</v>
-      </c>
-      <c r="H11" s="85">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="135" t="s">
-        <v>756</v>
-      </c>
-      <c r="B12" t="s">
-        <v>754</v>
-      </c>
-      <c r="E12" t="s">
-        <v>742</v>
-      </c>
-      <c r="F12" t="s">
-        <v>742</v>
-      </c>
-      <c r="G12" s="85">
-        <v>1340</v>
-      </c>
-      <c r="H12" s="85">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="136" t="s">
-        <v>757</v>
-      </c>
-      <c r="B13" t="s">
-        <v>211</v>
-      </c>
-      <c r="E13" t="s">
-        <v>742</v>
-      </c>
-      <c r="F13" t="s">
-        <v>742</v>
-      </c>
-      <c r="G13" s="85">
-        <v>5127095</v>
-      </c>
-      <c r="H13" s="85">
-        <v>4604041</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="Index!A1" display="index" xr:uid="{517959C2-4AED-4317-8F4E-F3B3E9646D4B}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7303D0-EAFB-485D-9ED0-6CB8F8BFE263}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="73.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="44.44140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C2" s="85"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>495</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>725</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="126" t="s">
-        <v>652</v>
-      </c>
-      <c r="B4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" t="s">
-        <v>156</v>
-      </c>
-      <c r="D4" s="127" t="s">
-        <v>662</v>
-      </c>
-      <c r="E4" t="s">
-        <v>635</v>
-      </c>
-      <c r="F4" t="s">
-        <v>636</v>
-      </c>
-      <c r="G4" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="126" t="s">
-        <v>653</v>
-      </c>
-      <c r="B5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C5" t="s">
-        <v>156</v>
-      </c>
-      <c r="D5" t="s">
-        <v>135</v>
-      </c>
-      <c r="E5" t="s">
-        <v>669</v>
-      </c>
-      <c r="F5" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="126" t="s">
-        <v>654</v>
-      </c>
-      <c r="B6" t="s">
-        <v>660</v>
-      </c>
-      <c r="C6" t="s">
-        <v>156</v>
-      </c>
-      <c r="D6" t="s">
-        <v>663</v>
-      </c>
-      <c r="E6" t="s">
-        <v>641</v>
-      </c>
-      <c r="F6" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="126" t="s">
-        <v>655</v>
-      </c>
-      <c r="B7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>156</v>
-      </c>
-      <c r="D7" t="s">
-        <v>664</v>
-      </c>
-      <c r="E7" t="s">
-        <v>642</v>
-      </c>
-      <c r="F7" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="126" t="s">
-        <v>656</v>
-      </c>
-      <c r="B8" t="s">
-        <v>660</v>
-      </c>
-      <c r="C8" t="s">
-        <v>156</v>
-      </c>
-      <c r="D8" t="s">
-        <v>665</v>
-      </c>
-      <c r="E8" s="126" t="s">
-        <v>643</v>
-      </c>
-      <c r="F8" s="126" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="126" t="s">
-        <v>657</v>
-      </c>
-      <c r="B9" t="s">
-        <v>660</v>
-      </c>
-      <c r="C9" t="s">
-        <v>156</v>
-      </c>
-      <c r="D9" t="s">
-        <v>666</v>
-      </c>
-      <c r="E9" s="126" t="s">
-        <v>670</v>
-      </c>
-      <c r="F9" s="126" t="s">
-        <v>665</v>
-      </c>
-      <c r="G9" s="126" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="126" t="s">
-        <v>658</v>
-      </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>156</v>
-      </c>
-      <c r="D10" t="s">
-        <v>667</v>
-      </c>
-      <c r="E10" s="126" t="s">
-        <v>644</v>
-      </c>
-      <c r="F10" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="126" t="s">
-        <v>659</v>
-      </c>
-      <c r="B11" t="s">
-        <v>661</v>
-      </c>
-      <c r="C11" t="s">
-        <v>156</v>
-      </c>
-      <c r="D11" t="s">
-        <v>668</v>
-      </c>
-      <c r="E11" s="128">
-        <v>1200</v>
-      </c>
-      <c r="F11" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="126" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" t="s">
-        <v>156</v>
-      </c>
-      <c r="E12" s="85">
-        <v>1</v>
-      </c>
-      <c r="F12" s="85">
-        <v>1</v>
-      </c>
-      <c r="G12" t="s">
-        <v>673</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{7348AD42-28E1-48B7-8921-A82010335EB1}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F912F66-4428-47A9-8ADF-02B84F72CE81}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="44.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.88671875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C2" s="85"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>495</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>725</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>684</v>
-      </c>
-      <c r="B4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" t="s">
-        <v>156</v>
-      </c>
-      <c r="D4" t="s">
-        <v>662</v>
-      </c>
-      <c r="E4" t="s">
-        <v>638</v>
-      </c>
-      <c r="F4" t="s">
-        <v>681</v>
-      </c>
-      <c r="G4" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>685</v>
-      </c>
-      <c r="B5" t="s">
-        <v>687</v>
-      </c>
-      <c r="C5" t="s">
-        <v>156</v>
-      </c>
-      <c r="D5" t="s">
-        <v>688</v>
-      </c>
-      <c r="E5" t="s">
-        <v>679</v>
-      </c>
-      <c r="F5" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>686</v>
-      </c>
-      <c r="B6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" t="s">
-        <v>156</v>
-      </c>
-      <c r="D6" t="s">
-        <v>135</v>
-      </c>
-      <c r="E6" t="s">
-        <v>680</v>
-      </c>
-      <c r="F6" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="126" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>156</v>
-      </c>
-      <c r="E7" s="85">
-        <v>1</v>
-      </c>
-      <c r="F7" s="85">
-        <v>1</v>
-      </c>
-      <c r="G7" t="s">
-        <v>673</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{8C3A7BBF-C04F-4B51-8B78-A0B63181F044}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81DFFCD9-6E0D-46F7-A5D0-F21B460087EE}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="44.44140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C2" s="85"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>495</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>725</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>696</v>
-      </c>
-      <c r="B4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D4" t="s">
-        <v>662</v>
-      </c>
-      <c r="E4" t="s">
-        <v>680</v>
-      </c>
-      <c r="F4" t="s">
-        <v>683</v>
-      </c>
-      <c r="G4" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>697</v>
-      </c>
-      <c r="B5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="127" t="s">
-        <v>662</v>
-      </c>
-      <c r="E5" t="s">
-        <v>692</v>
-      </c>
-      <c r="F5" t="s">
-        <v>694</v>
-      </c>
-      <c r="G5" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>698</v>
-      </c>
-      <c r="B6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" s="127" t="s">
-        <v>662</v>
-      </c>
-      <c r="E6" t="s">
-        <v>693</v>
-      </c>
-      <c r="F6" t="s">
-        <v>695</v>
-      </c>
-      <c r="G6" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="126" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="85">
-        <v>1</v>
-      </c>
-      <c r="F7" s="85">
-        <v>1</v>
-      </c>
-      <c r="G7" t="s">
-        <v>673</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{AB308857-2754-4349-AD90-AE62710AED13}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5C07CAD-3831-4F85-9B1D-4C30D19E9E25}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="83.88671875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C2" s="85"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>495</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>725</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
-        <v>706</v>
-      </c>
-      <c r="B4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" t="s">
-        <v>662</v>
-      </c>
-      <c r="E4" s="85" t="s">
-        <v>707</v>
-      </c>
-      <c r="F4" s="85" t="s">
-        <v>708</v>
-      </c>
-      <c r="G4" s="130" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>709</v>
-      </c>
-      <c r="B5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" t="s">
-        <v>734</v>
-      </c>
-      <c r="E5" s="85" t="s">
-        <v>710</v>
-      </c>
-      <c r="F5" s="85" t="s">
-        <v>711</v>
-      </c>
-      <c r="G5" s="89"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
-        <v>712</v>
-      </c>
-      <c r="B6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="2"/>
-      <c r="D6" t="s">
-        <v>735</v>
-      </c>
-      <c r="E6" s="85" t="s">
-        <v>710</v>
-      </c>
-      <c r="F6" s="85" t="s">
-        <v>713</v>
-      </c>
-      <c r="G6" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>731</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="85" t="s">
-        <v>732</v>
-      </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="85">
-        <v>1</v>
-      </c>
-      <c r="F7" s="85">
-        <v>1</v>
-      </c>
-      <c r="G7" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="C8" s="2"/>
-      <c r="E8" s="85"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-      <c r="C9" s="2"/>
-      <c r="E9" s="85"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="C10" s="2"/>
-      <c r="E10" s="85"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
-      <c r="C11" s="2"/>
-      <c r="E11" s="85"/>
-      <c r="F11" s="85"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
-      <c r="C12" s="85"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="85"/>
-      <c r="F12" s="85"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{DFFCEDC5-B5CD-4533-A52E-9F627F0A2FDF}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CBF657F-107F-4D04-A554-8C4B6A024335}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C2" s="85"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>495</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>725</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
-        <v>714</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" t="s">
-        <v>662</v>
-      </c>
-      <c r="E4" s="85">
-        <v>2019</v>
-      </c>
-      <c r="F4" s="85">
-        <v>2019</v>
-      </c>
-      <c r="G4" s="130" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>715</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="85">
-        <v>0</v>
-      </c>
-      <c r="E5" s="85">
-        <v>36</v>
-      </c>
-      <c r="F5" s="85">
-        <v>47</v>
-      </c>
-      <c r="G5" s="89"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
-        <v>716</v>
-      </c>
-      <c r="B6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" s="2"/>
-      <c r="D6" t="s">
-        <v>727</v>
-      </c>
-      <c r="E6" s="129">
-        <v>43714</v>
-      </c>
-      <c r="F6" s="129">
-        <v>43791</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>717</v>
-      </c>
-      <c r="B7" t="s">
-        <v>728</v>
-      </c>
-      <c r="C7" s="85"/>
-      <c r="D7" s="2" t="s">
-        <v>729</v>
-      </c>
-      <c r="E7" t="s">
-        <v>719</v>
-      </c>
-      <c r="F7" t="s">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>721</v>
-      </c>
-      <c r="B8" t="s">
-        <v>61</v>
-      </c>
-      <c r="D8" t="s">
-        <v>730</v>
-      </c>
-      <c r="E8" t="s">
-        <v>722</v>
-      </c>
-      <c r="F8" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>724</v>
-      </c>
-      <c r="B9" t="s">
-        <v>775</v>
-      </c>
-      <c r="D9" s="85">
-        <v>0</v>
-      </c>
-      <c r="E9" s="85">
-        <v>0.5</v>
-      </c>
-      <c r="F9" s="85">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
-        <v>731</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="85" t="s">
-        <v>732</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="85">
-        <v>1</v>
-      </c>
-      <c r="F10" s="85">
-        <v>1</v>
-      </c>
-      <c r="G10" t="s">
-        <v>733</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{61D2137B-2D94-4C63-851E-29BA389C2F89}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12475,246 +12744,261 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68F1906F-3F21-4ADD-B43B-A77686F8C5F2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6F5B38-E122-44E0-98B8-6AC4250F1F30}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultColWidth="23.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="55.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="42.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>738</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="139"/>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="139"/>
-      <c r="I2" s="139"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="140" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="137" t="s">
-        <v>16</v>
+      <c r="A2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="137" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="138" t="s">
+        <v>739</v>
       </c>
       <c r="C3" s="137" t="s">
-        <v>465</v>
+        <v>7</v>
       </c>
       <c r="D3" s="137" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="137" t="s">
-        <v>762</v>
-      </c>
-      <c r="F3" s="137" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="138" t="s">
+        <v>625</v>
+      </c>
+      <c r="F3" s="138" t="s">
+        <v>740</v>
+      </c>
+      <c r="G3" s="137" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="137" t="s">
+      <c r="H3" s="137" t="s">
         <v>256</v>
       </c>
-      <c r="H3" s="137" t="s">
-        <v>257</v>
+      <c r="I3" s="137" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="134" t="s">
-        <v>763</v>
+        <v>741</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>210</v>
+      </c>
+      <c r="D4" t="s">
+        <v>742</v>
       </c>
       <c r="E4" t="s">
-        <v>662</v>
+        <v>743</v>
       </c>
       <c r="F4" t="s">
+        <v>743</v>
+      </c>
+      <c r="G4" t="s">
         <v>744</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>745</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="135" t="s">
-        <v>764</v>
+        <v>746</v>
       </c>
       <c r="B5" t="s">
         <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>765</v>
-      </c>
-      <c r="F5" s="129">
+        <v>743</v>
+      </c>
+      <c r="F5" t="s">
+        <v>742</v>
+      </c>
+      <c r="G5" s="129">
         <v>43849</v>
       </c>
-      <c r="G5" s="129">
+      <c r="H5" s="129">
         <v>43853</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="135" t="s">
-        <v>766</v>
+        <v>627</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>210</v>
       </c>
       <c r="E6" t="s">
-        <v>135</v>
+        <v>743</v>
       </c>
       <c r="F6" t="s">
+        <v>743</v>
+      </c>
+      <c r="G6" t="s">
         <v>758</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>760</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="135" t="s">
-        <v>767</v>
+        <v>747</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>211</v>
       </c>
       <c r="E7" t="s">
-        <v>768</v>
+        <v>742</v>
       </c>
       <c r="F7" t="s">
+        <v>742</v>
+      </c>
+      <c r="G7" t="s">
         <v>748</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>749</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="135" t="s">
-        <v>769</v>
+        <v>750</v>
       </c>
       <c r="B8" t="s">
-        <v>770</v>
+        <v>751</v>
       </c>
       <c r="E8" t="s">
-        <v>771</v>
+        <v>743</v>
       </c>
       <c r="F8" t="s">
+        <v>742</v>
+      </c>
+      <c r="G8" t="s">
         <v>759</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>761</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="135" t="s">
-        <v>772</v>
+        <v>752</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>211</v>
       </c>
       <c r="E9" t="s">
-        <v>773</v>
+        <v>742</v>
+      </c>
+      <c r="F9" t="s">
+        <v>742</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="135" t="s">
-        <v>774</v>
+        <v>753</v>
       </c>
       <c r="B10" t="s">
-        <v>775</v>
+        <v>754</v>
       </c>
       <c r="E10" t="s">
-        <v>776</v>
-      </c>
-      <c r="F10" s="85">
+        <v>742</v>
+      </c>
+      <c r="F10" t="s">
+        <v>742</v>
+      </c>
+      <c r="G10" s="85">
         <v>12530</v>
       </c>
-      <c r="G10" s="85">
+      <c r="H10" s="85">
         <v>525</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="135" t="s">
-        <v>777</v>
+        <v>755</v>
       </c>
       <c r="B11" t="s">
-        <v>775</v>
+        <v>754</v>
       </c>
       <c r="E11" t="s">
-        <v>778</v>
-      </c>
-      <c r="F11" s="85">
+        <v>742</v>
+      </c>
+      <c r="F11" t="s">
+        <v>742</v>
+      </c>
+      <c r="G11" s="85">
         <v>5360</v>
       </c>
-      <c r="G11" s="85">
+      <c r="H11" s="85">
         <v>464</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="135" t="s">
-        <v>779</v>
+        <v>756</v>
       </c>
       <c r="B12" t="s">
-        <v>775</v>
+        <v>754</v>
       </c>
       <c r="E12" t="s">
-        <v>780</v>
-      </c>
-      <c r="F12" s="85">
+        <v>742</v>
+      </c>
+      <c r="F12" t="s">
+        <v>742</v>
+      </c>
+      <c r="G12" s="85">
         <v>1340</v>
       </c>
-      <c r="G12" s="85">
+      <c r="H12" s="85">
         <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="136" t="s">
-        <v>781</v>
+        <v>757</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>210</v>
       </c>
       <c r="E13" t="s">
-        <v>782</v>
-      </c>
-      <c r="F13" s="85">
+        <v>742</v>
+      </c>
+      <c r="F13" t="s">
+        <v>742</v>
+      </c>
+      <c r="G13" s="85">
         <v>5127095</v>
       </c>
-      <c r="G13" s="85">
+      <c r="H13" s="85">
         <v>4604041</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="139" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="85">
-        <v>1</v>
-      </c>
-      <c r="G14" s="85">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{70A1E038-0C96-4A41-9912-DEEE86C5416F}"/>
+    <hyperlink ref="A1" location="Index!A1" display="index" xr:uid="{517959C2-4AED-4317-8F4E-F3B3E9646D4B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Modified Bus Matrix Sheet
</commit_message>
<xml_diff>
--- a/DW2022/Documentation/Design document.xlsx
+++ b/DW2022/Documentation/Design document.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Llewellyn\Desktop\DW2022_Repo\DW2022\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831D1975-757A-4EA6-B1E3-5EEDA9F3684D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417F7CD5-3728-4F25-ACC3-A0CE9BEB90AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -63,6 +63,7 @@
     <definedName name="the_date">'[1]Calendar Day'!$A$31</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -90,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1877" uniqueCount="825">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1877" uniqueCount="826">
   <si>
     <t>Source Files</t>
   </si>
@@ -2585,6 +2586,9 @@
   </si>
   <si>
     <t>Project Management Bubble Chart</t>
+  </si>
+  <si>
+    <t>Project_Status</t>
   </si>
 </sst>
 </file>
@@ -3274,6 +3278,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3291,18 +3307,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -5913,6 +5917,15 @@
             <a:t>Fact</a:t>
           </a:r>
         </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-ZA" sz="900"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-ZA" sz="900"/>
+            <a:t>One row added per timesheet submitted during a week</a:t>
+          </a:r>
+        </a:p>
       </dgm:t>
     </dgm:pt>
     <dgm:pt modelId="{57A736B5-626C-4E9D-BDFA-678EC89851E9}" type="parTrans" cxnId="{167F6348-8EF0-4AD6-9FB4-431EBF7C21FF}">
@@ -6083,7 +6096,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{3C89EE6D-C5E6-4A60-AF4F-1B8C5AE23421}" type="pres">
-      <dgm:prSet presAssocID="{F0E1DDDD-AEB7-4ADC-A709-7ADD329B80AC}" presName="centerShape" presStyleLbl="node0" presStyleIdx="0" presStyleCnt="1" custLinFactNeighborX="1161"/>
+      <dgm:prSet presAssocID="{F0E1DDDD-AEB7-4ADC-A709-7ADD329B80AC}" presName="centerShape" presStyleLbl="node0" presStyleIdx="0" presStyleCnt="1" custScaleX="152418" custScaleY="142811" custLinFactNeighborX="1161"/>
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{5487FA13-369F-4726-A0B2-57E018C98BED}" type="pres">
@@ -6111,7 +6124,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{C45628D1-3F4D-481A-AC4F-D94C30465E21}" type="pres">
-      <dgm:prSet presAssocID="{AD65B444-B9CD-400C-A09C-E61C6A021388}" presName="node" presStyleLbl="node1" presStyleIdx="1" presStyleCnt="3">
+      <dgm:prSet presAssocID="{AD65B444-B9CD-400C-A09C-E61C6A021388}" presName="node" presStyleLbl="node1" presStyleIdx="1" presStyleCnt="3" custRadScaleRad="122040" custRadScaleInc="-8597">
         <dgm:presLayoutVars>
           <dgm:bulletEnabled val="1"/>
         </dgm:presLayoutVars>
@@ -6127,7 +6140,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{BC69186D-43E7-4F50-8E24-158008589D07}" type="pres">
-      <dgm:prSet presAssocID="{24E4D073-C36A-4CF1-A642-3BC904CE82CE}" presName="node" presStyleLbl="node1" presStyleIdx="2" presStyleCnt="3">
+      <dgm:prSet presAssocID="{24E4D073-C36A-4CF1-A642-3BC904CE82CE}" presName="node" presStyleLbl="node1" presStyleIdx="2" presStyleCnt="3" custRadScaleRad="124474" custRadScaleInc="-4998">
         <dgm:presLayoutVars>
           <dgm:bulletEnabled val="1"/>
         </dgm:presLayoutVars>
@@ -6187,16 +6200,28 @@
       </dgm:t>
     </dgm:pt>
     <dgm:pt modelId="{1B70F922-C51B-4614-B3E6-00A343653E2F}">
-      <dgm:prSet phldrT="[Text]"/>
+      <dgm:prSet phldrT="[Text]" custT="1"/>
       <dgm:spPr/>
       <dgm:t>
         <a:bodyPr/>
         <a:lstStyle/>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ZA"/>
+            <a:rPr lang="en-ZA" sz="800"/>
             <a:t>Project Management Fact</a:t>
           </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-ZA" sz="800"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-ZA" sz="800"/>
+            <a:t>One row added per project worked on during a year</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-ZA" sz="600"/>
         </a:p>
       </dgm:t>
     </dgm:pt>
@@ -6437,7 +6462,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{4B1526E4-5669-4024-83B8-4A8B6E169241}" type="pres">
-      <dgm:prSet presAssocID="{1B70F922-C51B-4614-B3E6-00A343653E2F}" presName="centerShape" presStyleLbl="node0" presStyleIdx="0" presStyleCnt="1" custScaleX="88488" custScaleY="79950" custLinFactNeighborX="-273" custLinFactNeighborY="-10642"/>
+      <dgm:prSet presAssocID="{1B70F922-C51B-4614-B3E6-00A343653E2F}" presName="centerShape" presStyleLbl="node0" presStyleIdx="0" presStyleCnt="1" custScaleX="122959" custScaleY="120200" custLinFactNeighborX="-273" custLinFactNeighborY="1914"/>
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{2838AADE-7FDA-4D9A-957B-367ECF25EB2C}" type="pres">
@@ -6449,7 +6474,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{980338C9-76FC-44DF-A765-78EDBF0932A9}" type="pres">
-      <dgm:prSet presAssocID="{B9DAC63D-D6A5-4FDB-93F1-BFDBF49405E4}" presName="node" presStyleLbl="node1" presStyleIdx="0" presStyleCnt="5" custScaleX="67748" custScaleY="55461" custRadScaleRad="80011" custRadScaleInc="-2171">
+      <dgm:prSet presAssocID="{B9DAC63D-D6A5-4FDB-93F1-BFDBF49405E4}" presName="node" presStyleLbl="node1" presStyleIdx="0" presStyleCnt="5" custScaleX="67748" custScaleY="55461" custRadScaleRad="110771" custRadScaleInc="-1568">
         <dgm:presLayoutVars>
           <dgm:bulletEnabled val="1"/>
         </dgm:presLayoutVars>
@@ -6465,7 +6490,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{C64E4C62-DBF5-4441-B992-140CDE54B3A0}" type="pres">
-      <dgm:prSet presAssocID="{5DE650A2-71CC-41D6-99A0-6889253322A0}" presName="node" presStyleLbl="node1" presStyleIdx="1" presStyleCnt="5" custScaleX="57420" custScaleY="59701" custRadScaleRad="79183" custRadScaleInc="-22257">
+      <dgm:prSet presAssocID="{5DE650A2-71CC-41D6-99A0-6889253322A0}" presName="node" presStyleLbl="node1" presStyleIdx="1" presStyleCnt="5" custScaleX="57420" custScaleY="59701" custRadScaleRad="115950" custRadScaleInc="-39339">
         <dgm:presLayoutVars>
           <dgm:bulletEnabled val="1"/>
         </dgm:presLayoutVars>
@@ -6481,7 +6506,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{49732D0F-F12C-48ED-97D7-25F133515C4D}" type="pres">
-      <dgm:prSet presAssocID="{CA4608D4-F871-42B8-81FD-7FC78933A958}" presName="node" presStyleLbl="node1" presStyleIdx="2" presStyleCnt="5" custScaleX="72355" custScaleY="67748" custRadScaleRad="59450" custRadScaleInc="-35856">
+      <dgm:prSet presAssocID="{CA4608D4-F871-42B8-81FD-7FC78933A958}" presName="node" presStyleLbl="node1" presStyleIdx="2" presStyleCnt="5" custScaleX="72355" custScaleY="67748" custRadScaleRad="100740" custRadScaleInc="-33509">
         <dgm:presLayoutVars>
           <dgm:bulletEnabled val="1"/>
         </dgm:presLayoutVars>
@@ -6497,7 +6522,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{5C1E975B-6DBE-4512-AC63-CDD9CF929A8A}" type="pres">
-      <dgm:prSet presAssocID="{7678F76A-6399-4502-80A1-4554E5B9BC4C}" presName="node" presStyleLbl="node1" presStyleIdx="3" presStyleCnt="5" custScaleX="59301" custScaleY="58073" custRadScaleRad="53769" custRadScaleInc="50987">
+      <dgm:prSet presAssocID="{7678F76A-6399-4502-80A1-4554E5B9BC4C}" presName="node" presStyleLbl="node1" presStyleIdx="3" presStyleCnt="5" custScaleX="59301" custScaleY="58073" custRadScaleRad="105319" custRadScaleInc="37551">
         <dgm:presLayoutVars>
           <dgm:bulletEnabled val="1"/>
         </dgm:presLayoutVars>
@@ -6513,7 +6538,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{1396B6E6-142A-4DDF-8A4B-4A5D7095A85D}" type="pres">
-      <dgm:prSet presAssocID="{C2C01C8F-4848-4B16-8890-993C6C6DE454}" presName="node" presStyleLbl="node1" presStyleIdx="4" presStyleCnt="5" custScaleX="69207" custScaleY="66639" custRadScaleRad="83090" custRadScaleInc="30330">
+      <dgm:prSet presAssocID="{C2C01C8F-4848-4B16-8890-993C6C6DE454}" presName="node" presStyleLbl="node1" presStyleIdx="4" presStyleCnt="5" custScaleX="69207" custScaleY="66639" custRadScaleRad="108030" custRadScaleInc="52131">
         <dgm:presLayoutVars>
           <dgm:bulletEnabled val="1"/>
         </dgm:presLayoutVars>
@@ -7170,8 +7195,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="1849693" y="1209126"/>
-          <a:ext cx="928687" cy="928687"/>
+          <a:off x="1611632" y="1013459"/>
+          <a:ext cx="1404428" cy="1315906"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -7271,10 +7296,43 @@
             <a:t>Fact</a:t>
           </a:r>
         </a:p>
+        <a:p>
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="400050">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPct val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPct val="35000"/>
+            </a:spcAft>
+            <a:buNone/>
+          </a:pPr>
+          <a:endParaRPr lang="en-ZA" sz="900" kern="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="400050">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPct val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPct val="35000"/>
+            </a:spcAft>
+            <a:buNone/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-ZA" sz="900" kern="1200"/>
+            <a:t>One row added per timesheet submitted during a week</a:t>
+          </a:r>
+        </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="1985696" y="1345129"/>
-        <a:ext cx="656681" cy="656681"/>
+        <a:off x="1817306" y="1206169"/>
+        <a:ext cx="993080" cy="930486"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{5487FA13-369F-4726-A0B2-57E018C98BED}">
@@ -7284,8 +7342,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm rot="16155673">
-          <a:off x="2166822" y="1051465"/>
-          <a:ext cx="278859" cy="36562"/>
+          <a:off x="2264522" y="955052"/>
+          <a:ext cx="80640" cy="36276"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -7296,10 +7354,10 @@
           <a:pathLst>
             <a:path>
               <a:moveTo>
-                <a:pt x="0" y="18281"/>
+                <a:pt x="0" y="18138"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="278859" y="18281"/>
+                <a:pt x="80640" y="18138"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -7354,8 +7412,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="10800000">
-        <a:off x="2299281" y="1062775"/>
-        <a:ext cx="13942" cy="13942"/>
+        <a:off x="2302827" y="971174"/>
+        <a:ext cx="4032" cy="4032"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{44889C79-B9F1-436F-AEA0-10F07D494EE6}">
@@ -7365,8 +7423,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="1784866" y="1672"/>
-          <a:ext cx="1027202" cy="928687"/>
+          <a:off x="1788794" y="11472"/>
+          <a:ext cx="1019177" cy="921432"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -7465,8 +7523,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="1935296" y="137675"/>
-        <a:ext cx="726342" cy="656681"/>
+        <a:off x="1938049" y="146413"/>
+        <a:ext cx="720667" cy="651550"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{D8A36C47-6E0C-4953-A975-2B34002DA6FF}">
@@ -7475,9 +7533,9 @@
         <dsp:cNvSpPr/>
       </dsp:nvSpPr>
       <dsp:spPr>
-        <a:xfrm rot="1840729">
-          <a:off x="2695575" y="1957059"/>
-          <a:ext cx="254596" cy="36562"/>
+        <a:xfrm rot="1510261">
+          <a:off x="2928122" y="2008323"/>
+          <a:ext cx="282466" cy="36276"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -7488,10 +7546,10 @@
           <a:pathLst>
             <a:path>
               <a:moveTo>
-                <a:pt x="0" y="18281"/>
+                <a:pt x="0" y="18138"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="254596" y="18281"/>
+                <a:pt x="282466" y="18138"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -7546,8 +7604,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="2816509" y="1968976"/>
-        <a:ext cx="12729" cy="12729"/>
+        <a:off x="3062294" y="2019400"/>
+        <a:ext cx="14123" cy="14123"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{C45628D1-3F4D-481A-AC4F-D94C30465E21}">
@@ -7557,8 +7615,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="2867366" y="1812867"/>
-          <a:ext cx="928687" cy="928687"/>
+          <a:off x="3153429" y="1821767"/>
+          <a:ext cx="921432" cy="921432"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -7619,8 +7677,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="3003369" y="1948870"/>
-        <a:ext cx="656681" cy="656681"/>
+        <a:off x="3288370" y="1956708"/>
+        <a:ext cx="651550" cy="651550"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{73464EC0-510D-44AB-933F-E0AA350BE21E}">
@@ -7629,9 +7687,9 @@
         <dsp:cNvSpPr/>
       </dsp:nvSpPr>
       <dsp:spPr>
-        <a:xfrm rot="9039124">
-          <a:off x="1625585" y="1957059"/>
-          <a:ext cx="303155" cy="36562"/>
+        <a:xfrm rot="9268600">
+          <a:off x="1436916" y="2008922"/>
+          <a:ext cx="264160" cy="36276"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -7642,10 +7700,10 @@
           <a:pathLst>
             <a:path>
               <a:moveTo>
-                <a:pt x="0" y="18281"/>
+                <a:pt x="0" y="18138"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="303155" y="18281"/>
+                <a:pt x="264160" y="18138"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -7700,8 +7758,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="10800000">
-        <a:off x="1769584" y="1967762"/>
-        <a:ext cx="15157" cy="15157"/>
+        <a:off x="1562392" y="2020456"/>
+        <a:ext cx="13208" cy="13208"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{BC69186D-43E7-4F50-8E24-158008589D07}">
@@ -7711,8 +7769,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="775945" y="1812867"/>
-          <a:ext cx="928687" cy="928687"/>
+          <a:off x="573335" y="1821767"/>
+          <a:ext cx="921432" cy="921432"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -7773,8 +7831,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="911948" y="1948870"/>
-        <a:ext cx="656681" cy="656681"/>
+        <a:off x="708276" y="1956708"/>
+        <a:ext cx="651550" cy="651550"/>
       </dsp:txXfrm>
     </dsp:sp>
   </dsp:spTree>
@@ -7796,8 +7854,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="1891195" y="1029352"/>
-          <a:ext cx="831654" cy="751409"/>
+          <a:off x="1809642" y="1150526"/>
+          <a:ext cx="1146828" cy="1121095"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -7861,10 +7919,58 @@
             <a:t>Project Management Fact</a:t>
           </a:r>
         </a:p>
+        <a:p>
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="355600">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPct val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPct val="35000"/>
+            </a:spcAft>
+            <a:buNone/>
+          </a:pPr>
+          <a:endParaRPr lang="en-ZA" sz="800" kern="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="355600">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPct val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPct val="35000"/>
+            </a:spcAft>
+            <a:buNone/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-ZA" sz="800" kern="1200"/>
+            <a:t>One row added per project worked on during a year</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="355600">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPct val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPct val="35000"/>
+            </a:spcAft>
+            <a:buNone/>
+          </a:pPr>
+          <a:endParaRPr lang="en-ZA" sz="600" kern="1200"/>
+        </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="2012988" y="1139393"/>
-        <a:ext cx="588068" cy="531327"/>
+        <a:off x="1977591" y="1314707"/>
+        <a:ext cx="810930" cy="792733"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{2838AADE-7FDA-4D9A-957B-367ECF25EB2C}">
@@ -7873,9 +7979,9 @@
         <dsp:cNvSpPr/>
       </dsp:nvSpPr>
       <dsp:spPr>
-        <a:xfrm rot="16168072">
-          <a:off x="2262499" y="970211"/>
-          <a:ext cx="81311" cy="37001"/>
+        <a:xfrm rot="16183641">
+          <a:off x="2093095" y="846834"/>
+          <a:ext cx="571865" cy="35535"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -7886,10 +7992,10 @@
           <a:pathLst>
             <a:path>
               <a:moveTo>
-                <a:pt x="0" y="18500"/>
+                <a:pt x="0" y="17767"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="81311" y="18500"/>
+                <a:pt x="571865" y="17767"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -7944,8 +8050,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="10800000">
-        <a:off x="2301122" y="986679"/>
-        <a:ext cx="4065" cy="4065"/>
+        <a:off x="2364731" y="850305"/>
+        <a:ext cx="28593" cy="28593"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{980338C9-76FC-44DF-A765-78EDBF0932A9}">
@@ -7955,8 +8061,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="1981992" y="426815"/>
-          <a:ext cx="636729" cy="521249"/>
+          <a:off x="2060496" y="61394"/>
+          <a:ext cx="631879" cy="517280"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -8017,8 +8123,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="2075239" y="503150"/>
-        <a:ext cx="450235" cy="368579"/>
+        <a:off x="2153033" y="137148"/>
+        <a:ext cx="446805" cy="365772"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{E3EA2590-1296-49C3-BAF7-BBFF2DE63A07}">
@@ -8027,9 +8133,9 @@
         <dsp:cNvSpPr/>
       </dsp:nvSpPr>
       <dsp:spPr>
-        <a:xfrm rot="20962917">
-          <a:off x="2712403" y="1291138"/>
-          <a:ext cx="207189" cy="37001"/>
+        <a:xfrm rot="19584680">
+          <a:off x="2807444" y="1212890"/>
+          <a:ext cx="598012" cy="35535"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -8040,10 +8146,10 @@
           <a:pathLst>
             <a:path>
               <a:moveTo>
-                <a:pt x="0" y="18500"/>
+                <a:pt x="0" y="17767"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="207189" y="18500"/>
+                <a:pt x="598012" y="17767"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -8098,8 +8204,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="2810818" y="1304459"/>
-        <a:ext cx="10359" cy="10359"/>
+        <a:off x="3091500" y="1215707"/>
+        <a:ext cx="29900" cy="29900"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{C64E4C62-DBF5-4441-B992-140CDE54B3A0}">
@@ -8109,8 +8215,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="2913536" y="960218"/>
-          <a:ext cx="539661" cy="561099"/>
+          <a:off x="3313425" y="636956"/>
+          <a:ext cx="535551" cy="556826"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -8173,8 +8279,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="2992568" y="1042389"/>
-        <a:ext cx="381597" cy="396757"/>
+        <a:off x="3391855" y="718501"/>
+        <a:ext cx="378691" cy="393736"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{0FCD4A5D-2B20-4E6E-BF59-242521BC3F8B}">
@@ -8183,9 +8289,9 @@
         <dsp:cNvSpPr/>
       </dsp:nvSpPr>
       <dsp:spPr>
-        <a:xfrm rot="3184820">
-          <a:off x="2499018" y="1780610"/>
-          <a:ext cx="208159" cy="37001"/>
+        <a:xfrm rot="2404226">
+          <a:off x="2782325" y="2155939"/>
+          <a:ext cx="301403" cy="35535"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -8196,10 +8302,10 @@
           <a:pathLst>
             <a:path>
               <a:moveTo>
-                <a:pt x="0" y="18500"/>
+                <a:pt x="0" y="17767"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="208159" y="18500"/>
+                <a:pt x="301403" y="17767"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -8254,8 +8360,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="2597894" y="1793907"/>
-        <a:ext cx="10407" cy="10407"/>
+        <a:off x="2925491" y="2166172"/>
+        <a:ext cx="15070" cy="15070"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{49732D0F-F12C-48ED-97D7-25F133515C4D}">
@@ -8265,8 +8371,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="2521245" y="1824340"/>
-          <a:ext cx="680028" cy="636729"/>
+          <a:off x="2961932" y="2165923"/>
+          <a:ext cx="674849" cy="631879"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -8327,8 +8433,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="2620833" y="1917587"/>
-        <a:ext cx="480852" cy="450235"/>
+        <a:off x="3060761" y="2258460"/>
+        <a:ext cx="477191" cy="446805"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{8BF4EDA2-910D-46CB-9F48-E05EC525E760}">
@@ -8337,9 +8443,9 @@
         <dsp:cNvSpPr/>
       </dsp:nvSpPr>
       <dsp:spPr>
-        <a:xfrm rot="7761192">
-          <a:off x="1923802" y="1752629"/>
-          <a:ext cx="166048" cy="37001"/>
+        <a:xfrm rot="8456917">
+          <a:off x="1585418" y="2177664"/>
+          <a:ext cx="401201" cy="35535"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -8350,10 +8456,10 @@
           <a:pathLst>
             <a:path>
               <a:moveTo>
-                <a:pt x="0" y="18500"/>
+                <a:pt x="0" y="17767"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="166048" y="18500"/>
+                <a:pt x="401201" y="17767"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -8408,8 +8514,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="10800000">
-        <a:off x="2002675" y="1766979"/>
-        <a:ext cx="8302" cy="8302"/>
+        <a:off x="1775988" y="2185402"/>
+        <a:ext cx="20060" cy="20060"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{5C1E975B-6DBE-4512-AC63-CDD9CF929A8A}">
@@ -8419,8 +8525,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="1501022" y="1775210"/>
-          <a:ext cx="557340" cy="545798"/>
+          <a:off x="1140725" y="2223763"/>
+          <a:ext cx="553095" cy="541642"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -8481,8 +8587,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="1582643" y="1855140"/>
-        <a:ext cx="394098" cy="385938"/>
+        <a:off x="1221724" y="2303085"/>
+        <a:ext cx="391097" cy="382998"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{9D4692C8-D487-4537-B4A5-B19EA5D5686F}">
@@ -8491,9 +8597,9 @@
         <dsp:cNvSpPr/>
       </dsp:nvSpPr>
       <dsp:spPr>
-        <a:xfrm rot="11680168">
-          <a:off x="1735849" y="1259892"/>
-          <a:ext cx="174617" cy="37001"/>
+        <a:xfrm rot="13112157">
+          <a:off x="1539065" y="1199609"/>
+          <a:ext cx="448255" cy="35535"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -8504,10 +8610,10 @@
           <a:pathLst>
             <a:path>
               <a:moveTo>
-                <a:pt x="0" y="18500"/>
+                <a:pt x="0" y="17767"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="174617" y="18500"/>
+                <a:pt x="448255" y="17767"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -8562,8 +8668,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="10800000">
-        <a:off x="1818792" y="1274028"/>
-        <a:ext cx="8730" cy="8730"/>
+        <a:off x="1751986" y="1206170"/>
+        <a:ext cx="22412" cy="22412"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{1396B6E6-142A-4DDF-8A4B-4A5D7095A85D}">
@@ -8573,8 +8679,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="1099644" y="860977"/>
-          <a:ext cx="650441" cy="626306"/>
+          <a:off x="1016439" y="568901"/>
+          <a:ext cx="645487" cy="621536"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -8635,8 +8741,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="1194899" y="952697"/>
-        <a:ext cx="459931" cy="442866"/>
+        <a:off x="1110968" y="659923"/>
+        <a:ext cx="456429" cy="439492"/>
       </dsp:txXfrm>
     </dsp:sp>
   </dsp:spTree>
@@ -12506,15 +12612,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
+      <xdr:colOff>1040130</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:rowOff>68580</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>560070</xdr:colOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>575310</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15063,14 +15169,14 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="142" t="s">
+      <c r="A8" s="146" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
-      <c r="E8" s="142"/>
-      <c r="F8" s="142"/>
+      <c r="B8" s="146"/>
+      <c r="C8" s="146"/>
+      <c r="D8" s="146"/>
+      <c r="E8" s="146"/>
+      <c r="F8" s="146"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
@@ -15230,14 +15336,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="142" t="s">
+      <c r="A18" s="146" t="s">
         <v>485</v>
       </c>
-      <c r="B18" s="142"/>
-      <c r="C18" s="142"/>
-      <c r="D18" s="142"/>
-      <c r="E18" s="142"/>
-      <c r="F18" s="142"/>
+      <c r="B18" s="146"/>
+      <c r="C18" s="146"/>
+      <c r="D18" s="146"/>
+      <c r="E18" s="146"/>
+      <c r="F18" s="146"/>
     </row>
     <row r="19" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -15246,11 +15352,11 @@
       <c r="B19" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="141" t="s">
+      <c r="C19" s="145" t="s">
         <v>470</v>
       </c>
-      <c r="D19" s="141"/>
-      <c r="E19" s="141"/>
+      <c r="D19" s="145"/>
+      <c r="E19" s="145"/>
       <c r="F19" s="12"/>
     </row>
     <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -15276,14 +15382,14 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="143" t="s">
+      <c r="A23" s="147" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="143"/>
-      <c r="C23" s="143"/>
-      <c r="D23" s="143"/>
-      <c r="E23" s="143"/>
-      <c r="F23" s="143"/>
+      <c r="B23" s="147"/>
+      <c r="C23" s="147"/>
+      <c r="D23" s="147"/>
+      <c r="E23" s="147"/>
+      <c r="F23" s="147"/>
     </row>
     <row r="24" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
@@ -15292,11 +15398,11 @@
       <c r="B24" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="141" t="s">
+      <c r="C24" s="145" t="s">
         <v>482</v>
       </c>
-      <c r="D24" s="141"/>
-      <c r="E24" s="141"/>
+      <c r="D24" s="145"/>
+      <c r="E24" s="145"/>
       <c r="F24" s="8" t="s">
         <v>23</v>
       </c>
@@ -15344,14 +15450,14 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="143" t="s">
+      <c r="A29" s="147" t="s">
         <v>468</v>
       </c>
-      <c r="B29" s="143"/>
-      <c r="C29" s="143"/>
-      <c r="D29" s="143"/>
-      <c r="E29" s="143"/>
-      <c r="F29" s="143"/>
+      <c r="B29" s="147"/>
+      <c r="C29" s="147"/>
+      <c r="D29" s="147"/>
+      <c r="E29" s="147"/>
+      <c r="F29" s="147"/>
     </row>
     <row r="30" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
@@ -15360,11 +15466,11 @@
       <c r="B30" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="141" t="s">
+      <c r="C30" s="145" t="s">
         <v>470</v>
       </c>
-      <c r="D30" s="141"/>
-      <c r="E30" s="141"/>
+      <c r="D30" s="145"/>
+      <c r="E30" s="145"/>
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -17438,14 +17544,14 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="142" t="s">
+      <c r="A8" s="146" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
-      <c r="E8" s="142"/>
-      <c r="F8" s="142"/>
+      <c r="B8" s="146"/>
+      <c r="C8" s="146"/>
+      <c r="D8" s="146"/>
+      <c r="E8" s="146"/>
+      <c r="F8" s="146"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
@@ -17528,14 +17634,14 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="142" t="s">
+      <c r="A14" s="146" t="s">
         <v>485</v>
       </c>
-      <c r="B14" s="142"/>
-      <c r="C14" s="142"/>
-      <c r="D14" s="142"/>
-      <c r="E14" s="142"/>
-      <c r="F14" s="142"/>
+      <c r="B14" s="146"/>
+      <c r="C14" s="146"/>
+      <c r="D14" s="146"/>
+      <c r="E14" s="146"/>
+      <c r="F14" s="146"/>
     </row>
     <row r="15" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
@@ -17544,11 +17650,11 @@
       <c r="B15" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="141" t="s">
+      <c r="C15" s="145" t="s">
         <v>470</v>
       </c>
-      <c r="D15" s="141"/>
-      <c r="E15" s="141"/>
+      <c r="D15" s="145"/>
+      <c r="E15" s="145"/>
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -17563,14 +17669,14 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="143" t="s">
+      <c r="A20" s="147" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="143"/>
-      <c r="C20" s="143"/>
-      <c r="D20" s="143"/>
-      <c r="E20" s="143"/>
-      <c r="F20" s="143"/>
+      <c r="B20" s="147"/>
+      <c r="C20" s="147"/>
+      <c r="D20" s="147"/>
+      <c r="E20" s="147"/>
+      <c r="F20" s="147"/>
     </row>
     <row r="21" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -17579,11 +17685,11 @@
       <c r="B21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="141" t="s">
+      <c r="C21" s="145" t="s">
         <v>482</v>
       </c>
-      <c r="D21" s="141"/>
-      <c r="E21" s="141"/>
+      <c r="D21" s="145"/>
+      <c r="E21" s="145"/>
       <c r="F21" s="8" t="s">
         <v>23</v>
       </c>
@@ -17631,14 +17737,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="143" t="s">
+      <c r="A26" s="147" t="s">
         <v>468</v>
       </c>
-      <c r="B26" s="143"/>
-      <c r="C26" s="143"/>
-      <c r="D26" s="143"/>
-      <c r="E26" s="143"/>
-      <c r="F26" s="143"/>
+      <c r="B26" s="147"/>
+      <c r="C26" s="147"/>
+      <c r="D26" s="147"/>
+      <c r="E26" s="147"/>
+      <c r="F26" s="147"/>
     </row>
     <row r="27" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
@@ -17647,11 +17753,11 @@
       <c r="B27" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="141" t="s">
+      <c r="C27" s="145" t="s">
         <v>470</v>
       </c>
-      <c r="D27" s="141"/>
-      <c r="E27" s="141"/>
+      <c r="D27" s="145"/>
+      <c r="E27" s="145"/>
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -17769,10 +17875,10 @@
       <c r="F5" s="53"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="145" t="s">
+      <c r="A10" s="149" t="s">
         <v>497</v>
       </c>
-      <c r="B10" s="145"/>
+      <c r="B10" s="149"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
@@ -18766,7 +18872,7 @@
     <col min="9" max="9" width="15.5546875" style="29" customWidth="1"/>
     <col min="10" max="10" width="14" style="29" customWidth="1"/>
     <col min="11" max="11" width="14.6640625" style="29" customWidth="1"/>
-    <col min="12" max="12" width="12.21875" style="29" customWidth="1"/>
+    <col min="12" max="12" width="14.44140625" style="29" customWidth="1"/>
     <col min="13" max="13" width="7.88671875" style="29" bestFit="1" customWidth="1"/>
     <col min="14" max="16384" width="9.109375" style="29"/>
   </cols>
@@ -18789,19 +18895,19 @@
       <c r="H2" s="98" t="s">
         <v>553</v>
       </c>
-      <c r="I2" s="148" t="s">
+      <c r="I2" s="142" t="s">
         <v>806</v>
       </c>
-      <c r="J2" s="148" t="s">
+      <c r="J2" s="142" t="s">
         <v>807</v>
       </c>
-      <c r="K2" s="148" t="s">
+      <c r="K2" s="142" t="s">
         <v>810</v>
       </c>
-      <c r="L2" s="148" t="s">
-        <v>750</v>
-      </c>
-      <c r="M2" s="148" t="s">
+      <c r="L2" s="142" t="s">
+        <v>825</v>
+      </c>
+      <c r="M2" s="142" t="s">
         <v>808</v>
       </c>
     </row>
@@ -18908,7 +19014,7 @@
       <c r="D6" s="30" t="s">
         <v>818</v>
       </c>
-      <c r="E6" s="149" t="s">
+      <c r="E6" s="143" t="s">
         <v>819</v>
       </c>
       <c r="F6" s="30" t="s">
@@ -18935,7 +19041,7 @@
       <c r="D7" s="30" t="s">
         <v>818</v>
       </c>
-      <c r="E7" s="149" t="s">
+      <c r="E7" s="143" t="s">
         <v>820</v>
       </c>
       <c r="F7" s="30" t="s">
@@ -18956,14 +19062,14 @@
       <c r="N7" s="30"/>
     </row>
     <row r="9" spans="2:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B9" s="147"/>
-      <c r="D9" s="147" t="s">
+      <c r="B9" s="141"/>
+      <c r="D9" s="141" t="s">
         <v>290</v>
       </c>
-      <c r="G9" s="150" t="s">
+      <c r="G9" s="144" t="s">
         <v>823</v>
       </c>
-      <c r="K9" s="150" t="s">
+      <c r="K9" s="144" t="s">
         <v>824</v>
       </c>
     </row>
@@ -19039,7 +19145,7 @@
       <c r="F6" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="146" t="s">
+      <c r="J6" s="150" t="s">
         <v>467</v>
       </c>
     </row>
@@ -19056,7 +19162,7 @@
       <c r="F7" t="s">
         <v>95</v>
       </c>
-      <c r="J7" s="146"/>
+      <c r="J7" s="150"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -19068,7 +19174,7 @@
       <c r="F8" t="s">
         <v>93</v>
       </c>
-      <c r="J8" s="146"/>
+      <c r="J8" s="150"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -19080,7 +19186,7 @@
       <c r="F9" t="s">
         <v>462</v>
       </c>
-      <c r="J9" s="146"/>
+      <c r="J9" s="150"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -19092,7 +19198,7 @@
       <c r="F10" t="s">
         <v>463</v>
       </c>
-      <c r="J10" s="146"/>
+      <c r="J10" s="150"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -19104,7 +19210,7 @@
       <c r="F11" t="s">
         <v>89</v>
       </c>
-      <c r="J11" s="146"/>
+      <c r="J11" s="150"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -19119,7 +19225,7 @@
       <c r="F12" t="s">
         <v>86</v>
       </c>
-      <c r="J12" s="146"/>
+      <c r="J12" s="150"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -19131,7 +19237,7 @@
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="J13" s="146"/>
+      <c r="J13" s="150"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="122" t="s">
@@ -19510,14 +19616,14 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="142" t="s">
+      <c r="A7" s="146" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="142"/>
-      <c r="C7" s="142"/>
-      <c r="D7" s="142"/>
-      <c r="E7" s="142"/>
-      <c r="F7" s="142"/>
+      <c r="B7" s="146"/>
+      <c r="C7" s="146"/>
+      <c r="D7" s="146"/>
+      <c r="E7" s="146"/>
+      <c r="F7" s="146"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
@@ -19606,14 +19712,14 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="142" t="s">
+      <c r="A14" s="146" t="s">
         <v>485</v>
       </c>
-      <c r="B14" s="142"/>
-      <c r="C14" s="142"/>
-      <c r="D14" s="142"/>
-      <c r="E14" s="142"/>
-      <c r="F14" s="142"/>
+      <c r="B14" s="146"/>
+      <c r="C14" s="146"/>
+      <c r="D14" s="146"/>
+      <c r="E14" s="146"/>
+      <c r="F14" s="146"/>
     </row>
     <row r="15" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
@@ -19622,11 +19728,11 @@
       <c r="B15" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="141" t="s">
+      <c r="C15" s="145" t="s">
         <v>470</v>
       </c>
-      <c r="D15" s="141"/>
-      <c r="E15" s="141"/>
+      <c r="D15" s="145"/>
+      <c r="E15" s="145"/>
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -19638,14 +19744,14 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="143" t="s">
+      <c r="A20" s="147" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="143"/>
-      <c r="C20" s="143"/>
-      <c r="D20" s="143"/>
-      <c r="E20" s="143"/>
-      <c r="F20" s="143"/>
+      <c r="B20" s="147"/>
+      <c r="C20" s="147"/>
+      <c r="D20" s="147"/>
+      <c r="E20" s="147"/>
+      <c r="F20" s="147"/>
     </row>
     <row r="21" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -19654,11 +19760,11 @@
       <c r="B21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="141" t="s">
+      <c r="C21" s="145" t="s">
         <v>482</v>
       </c>
-      <c r="D21" s="141"/>
-      <c r="E21" s="141"/>
+      <c r="D21" s="145"/>
+      <c r="E21" s="145"/>
       <c r="F21" s="8" t="s">
         <v>23</v>
       </c>
@@ -19706,14 +19812,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="143" t="s">
+      <c r="A26" s="147" t="s">
         <v>468</v>
       </c>
-      <c r="B26" s="143"/>
-      <c r="C26" s="143"/>
-      <c r="D26" s="143"/>
-      <c r="E26" s="143"/>
-      <c r="F26" s="143"/>
+      <c r="B26" s="147"/>
+      <c r="C26" s="147"/>
+      <c r="D26" s="147"/>
+      <c r="E26" s="147"/>
+      <c r="F26" s="147"/>
     </row>
     <row r="27" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
@@ -19722,11 +19828,11 @@
       <c r="B27" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="141" t="s">
+      <c r="C27" s="145" t="s">
         <v>470</v>
       </c>
-      <c r="D27" s="141"/>
-      <c r="E27" s="141"/>
+      <c r="D27" s="145"/>
+      <c r="E27" s="145"/>
       <c r="F27" s="8"/>
     </row>
   </sheetData>
@@ -52428,16 +52534,16 @@
       <c r="A3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="144" t="s">
+      <c r="B3" s="148" t="s">
         <v>235</v>
       </c>
-      <c r="C3" s="144"/>
-      <c r="D3" s="144"/>
-      <c r="E3" s="144"/>
-      <c r="F3" s="144"/>
-      <c r="G3" s="144"/>
-      <c r="H3" s="144"/>
-      <c r="I3" s="144"/>
+      <c r="C3" s="148"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
+      <c r="G3" s="148"/>
+      <c r="H3" s="148"/>
+      <c r="I3" s="148"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="35" t="s">
@@ -53051,16 +53157,16 @@
       <c r="A3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="144" t="s">
+      <c r="B3" s="148" t="s">
         <v>409</v>
       </c>
-      <c r="C3" s="144"/>
-      <c r="D3" s="144"/>
-      <c r="E3" s="144"/>
-      <c r="F3" s="144"/>
-      <c r="G3" s="144"/>
-      <c r="H3" s="144"/>
-      <c r="I3" s="144"/>
+      <c r="C3" s="148"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
+      <c r="G3" s="148"/>
+      <c r="H3" s="148"/>
+      <c r="I3" s="148"/>
     </row>
     <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="35" t="s">

</xml_diff>

<commit_message>
Finalized corrections on Design document and dimensions
</commit_message>
<xml_diff>
--- a/DW2022/Documentation/Design document.xlsx
+++ b/DW2022/Documentation/Design document.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Llewellyn\Desktop\Honours Resources\DATA WAREHOUSING\DW2022_Repo\DW2022\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8C68D4-C36E-4557-BB43-74988165E0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDDF43A-F7EA-471A-BA2E-C79DAB4E9F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" firstSheet="27" activeTab="29" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -102,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2342" uniqueCount="917">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2408" uniqueCount="960">
   <si>
     <t>Source Files</t>
   </si>
@@ -2570,9 +2570,6 @@
     <t>Periodic Snapshot</t>
   </si>
   <si>
-    <t>One row for each employee that worked during that week</t>
-  </si>
-  <si>
     <t>One row for each project that have been worked on during that year</t>
   </si>
   <si>
@@ -2851,12 +2848,6 @@
     <t>External_Or_Internal</t>
   </si>
   <si>
-    <t>Total_Hours_Worked</t>
-  </si>
-  <si>
-    <t>The total number of hours the employee worked on a project when the timesheet is submitted per week</t>
-  </si>
-  <si>
     <t xml:space="preserve">Project status for every project. </t>
   </si>
   <si>
@@ -2866,15 +2857,156 @@
     <t>ID of the department the customer belongs to</t>
   </si>
   <si>
-    <t>Report_Date</t>
+    <t>One row for each employee that worked during that week per project</t>
   </si>
   <si>
     <t>X
-Report_Date
-Project_Request_Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One row for each employee timesheet event (when a timesheet is submitted) </t>
+Report_Date_Key
+Project_Request_Date_Key</t>
+  </si>
+  <si>
+    <t>Report_Date_Key</t>
+  </si>
+  <si>
+    <t>Project_Request_Date_Key</t>
+  </si>
+  <si>
+    <t>One row for each employee timesheet event (when a timesheet is submitted) per project</t>
+  </si>
+  <si>
+    <t>Service billing number of a project</t>
+  </si>
+  <si>
+    <t>Uniquely identifies each record submitted per timesheet per project</t>
+  </si>
+  <si>
+    <t>Annual_Project_Analysis_Cost_Key</t>
+  </si>
+  <si>
+    <t>Employee_TimeSheet_Key</t>
+  </si>
+  <si>
+    <t>Uniquely identifies each record for every year end</t>
+  </si>
+  <si>
+    <t>Current_Project_Status</t>
+  </si>
+  <si>
+    <t>Current_Customer_Name</t>
+  </si>
+  <si>
+    <t>*No Current Customer Name</t>
+  </si>
+  <si>
+    <t>*Unknown Current Customer Name</t>
+  </si>
+  <si>
+    <t>*Unknown Customer Name</t>
+  </si>
+  <si>
+    <t>Adam-Obenwienski</t>
+  </si>
+  <si>
+    <t>Current name of the customer</t>
+  </si>
+  <si>
+    <t>This will help with reporting to group together information over time for the same customer.</t>
+  </si>
+  <si>
+    <t>NB! No housekeeping columns in a dimension without any SCD fields</t>
+  </si>
+  <si>
+    <t>ID of Employee</t>
+  </si>
+  <si>
+    <t>Name of the Employee</t>
+  </si>
+  <si>
+    <t>Surname of the Employee</t>
+  </si>
+  <si>
+    <t>Year a timesheet was submitted</t>
+  </si>
+  <si>
+    <t>Week of the year as a numeric value a timesheet was submitted</t>
+  </si>
+  <si>
+    <t>Date of the Week End</t>
+  </si>
+  <si>
+    <t>ID of the project worked on</t>
+  </si>
+  <si>
+    <t>Employee that worked on the project</t>
+  </si>
+  <si>
+    <t>How many hours the employee worked on a project</t>
+  </si>
+  <si>
+    <t>ID of the Project</t>
+  </si>
+  <si>
+    <t>ID of the Customer</t>
+  </si>
+  <si>
+    <t>ID of a customer requesting the project</t>
+  </si>
+  <si>
+    <t>Category of the project</t>
+  </si>
+  <si>
+    <t>A description of the project being requested</t>
+  </si>
+  <si>
+    <t>Current status of the project</t>
+  </si>
+  <si>
+    <t>Labour Costs attached to the project</t>
+  </si>
+  <si>
+    <t>Material Costs attached to the project</t>
+  </si>
+  <si>
+    <t>Handling fees attached to the project</t>
+  </si>
+  <si>
+    <t>The service billing number of the project
+being requested</t>
+  </si>
+  <si>
+    <t>ID of the Customer Group</t>
+  </si>
+  <si>
+    <t>Name of the Customer Group</t>
+  </si>
+  <si>
+    <t>Is the Customer Group internal 
+or external?</t>
+  </si>
+  <si>
+    <t>ID of the Customer Department</t>
+  </si>
+  <si>
+    <t>Name of the Customer Department</t>
+  </si>
+  <si>
+    <t>ID of the Customer Group linked to
+the Customer Department</t>
+  </si>
+  <si>
+    <t>Name of the Customer</t>
+  </si>
+  <si>
+    <t>ID of Department Customer is assigned to</t>
+  </si>
+  <si>
+    <t>Name of the Contact Person</t>
+  </si>
+  <si>
+    <t>City or Town where customer lives</t>
+  </si>
+  <si>
+    <t>Postal Code of customer residence</t>
   </si>
 </sst>
 </file>
@@ -3283,7 +3415,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="204">
+  <cellXfs count="211">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3815,6 +3947,12 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3835,6 +3973,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -6789,7 +6942,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-ZA" sz="1200"/>
-            <a:t>Report_Date</a:t>
+            <a:t>Report_Date_Key</a:t>
           </a:r>
         </a:p>
       </dgm:t>
@@ -6945,6 +7098,13 @@
           <a:schemeClr val="accent4"/>
         </a:solidFill>
       </dgm:spPr>
+      <dgm:t>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-ZA"/>
+        </a:p>
+      </dgm:t>
     </dgm:pt>
     <dgm:pt modelId="{21706501-A09C-424A-B394-06DD0435B800}" type="parTrans" cxnId="{704B1FB8-7730-4177-8032-8DFD016F9632}">
       <dgm:prSet/>
@@ -6975,6 +7135,13 @@
           <a:schemeClr val="accent4"/>
         </a:solidFill>
       </dgm:spPr>
+      <dgm:t>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-ZA"/>
+        </a:p>
+      </dgm:t>
     </dgm:pt>
     <dgm:pt modelId="{BD238C88-CEBD-4C60-BFBA-C6D78C00EF21}" type="parTrans" cxnId="{5FD703B6-0150-4754-A06B-957ECE658F9C}">
       <dgm:prSet/>
@@ -7005,6 +7172,13 @@
           <a:schemeClr val="accent4"/>
         </a:solidFill>
       </dgm:spPr>
+      <dgm:t>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-ZA"/>
+        </a:p>
+      </dgm:t>
     </dgm:pt>
     <dgm:pt modelId="{6ECAC818-4381-4775-B60D-6E504593134D}" type="parTrans" cxnId="{C53109CE-FED1-4907-BB68-085EA2ADCC7F}">
       <dgm:prSet/>
@@ -7037,7 +7211,7 @@
         <a:p>
           <a:r>
             <a:rPr lang="en-ZA" sz="1200" baseline="0"/>
-            <a:t>Project_Request_Date</a:t>
+            <a:t>Project_Request_Date_Key</a:t>
           </a:r>
         </a:p>
       </dgm:t>
@@ -7088,7 +7262,7 @@
       <dgm:spPr/>
     </dgm:pt>
     <dgm:pt modelId="{980338C9-76FC-44DF-A765-78EDBF0932A9}" type="pres">
-      <dgm:prSet presAssocID="{B9DAC63D-D6A5-4FDB-93F1-BFDBF49405E4}" presName="node" presStyleLbl="node1" presStyleIdx="0" presStyleCnt="5" custScaleX="131210" custScaleY="124947" custRadScaleRad="163668" custRadScaleInc="97570">
+      <dgm:prSet presAssocID="{B9DAC63D-D6A5-4FDB-93F1-BFDBF49405E4}" presName="node" presStyleLbl="node1" presStyleIdx="0" presStyleCnt="5" custScaleX="140790" custScaleY="124947" custRadScaleRad="163668" custRadScaleInc="97570">
         <dgm:presLayoutVars>
           <dgm:bulletEnabled val="1"/>
         </dgm:presLayoutVars>
@@ -8596,9 +8770,9 @@
         <dsp:cNvSpPr/>
       </dsp:nvSpPr>
       <dsp:spPr>
-        <a:xfrm rot="19293940">
-          <a:off x="2816345" y="1154861"/>
-          <a:ext cx="341189" cy="47373"/>
+        <a:xfrm rot="19225782">
+          <a:off x="2812932" y="1164847"/>
+          <a:ext cx="268552" cy="47373"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -8612,7 +8786,7 @@
                 <a:pt x="0" y="23686"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="341189" y="23686"/>
+                <a:pt x="268552" y="23686"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -8667,8 +8841,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="2978410" y="1170017"/>
-        <a:ext cx="17059" cy="17059"/>
+        <a:off x="2940495" y="1181820"/>
+        <a:ext cx="13427" cy="13427"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{980338C9-76FC-44DF-A765-78EDBF0932A9}">
@@ -8678,8 +8852,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="2940801" y="-138896"/>
-          <a:ext cx="1551188" cy="1477146"/>
+          <a:off x="2827545" y="-138896"/>
+          <a:ext cx="1664444" cy="1477146"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -8735,13 +8909,13 @@
           </a:pPr>
           <a:r>
             <a:rPr lang="en-ZA" sz="1200" kern="1200"/>
-            <a:t>Report_Date</a:t>
+            <a:t>Report_Date_Key</a:t>
           </a:r>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="3167967" y="77427"/>
-        <a:ext cx="1096856" cy="1044500"/>
+        <a:off x="3071297" y="77427"/>
+        <a:ext cx="1176940" cy="1044500"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{E3EA2590-1296-49C3-BAF7-BBFF2DE63A07}">
@@ -9358,7 +9532,7 @@
           </a:pPr>
           <a:r>
             <a:rPr lang="en-ZA" sz="1200" kern="1200" baseline="0"/>
-            <a:t>Project_Request_Date</a:t>
+            <a:t>Project_Request_Date_Key</a:t>
           </a:r>
         </a:p>
       </dsp:txBody>
@@ -13852,12 +14026,12 @@
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
@@ -13877,7 +14051,7 @@
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C16" s="46" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
@@ -14098,16 +14272,16 @@
       <c r="A3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="200" t="s">
+      <c r="B3" s="202" t="s">
         <v>235</v>
       </c>
-      <c r="C3" s="200"/>
-      <c r="D3" s="200"/>
-      <c r="E3" s="200"/>
-      <c r="F3" s="200"/>
-      <c r="G3" s="200"/>
-      <c r="H3" s="200"/>
-      <c r="I3" s="200"/>
+      <c r="C3" s="202"/>
+      <c r="D3" s="202"/>
+      <c r="E3" s="202"/>
+      <c r="F3" s="202"/>
+      <c r="G3" s="202"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="202"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -14730,16 +14904,16 @@
       <c r="A3" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="200" t="s">
-        <v>877</v>
-      </c>
-      <c r="C3" s="200"/>
-      <c r="D3" s="200"/>
-      <c r="E3" s="200"/>
-      <c r="F3" s="200"/>
-      <c r="G3" s="200"/>
-      <c r="H3" s="200"/>
-      <c r="I3" s="200"/>
+      <c r="B3" s="202" t="s">
+        <v>876</v>
+      </c>
+      <c r="C3" s="202"/>
+      <c r="D3" s="202"/>
+      <c r="E3" s="202"/>
+      <c r="F3" s="202"/>
+      <c r="G3" s="202"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="202"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -14772,7 +14946,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="147" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B6" s="148" t="s">
         <v>20</v>
@@ -14823,13 +14997,13 @@
         <v>36</v>
       </c>
       <c r="C8" s="166" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="E8" s="176">
         <v>2</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="G8" s="75" t="s">
         <v>765</v>
@@ -14846,13 +15020,13 @@
         <v>767</v>
       </c>
       <c r="C9" s="166" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="E9" s="176">
         <v>2</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="G9" s="75" t="s">
         <v>768</v>
@@ -14863,13 +15037,13 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="147" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="B10" s="148" t="s">
         <v>57</v>
       </c>
       <c r="C10" s="147" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="D10" s="150"/>
       <c r="E10" s="177">
@@ -14887,25 +15061,25 @@
     </row>
     <row r="11" spans="1:9" s="165" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="165" t="s">
-        <v>821</v>
+        <v>921</v>
       </c>
       <c r="B11" s="148" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="166" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="E11" s="48">
         <v>1</v>
       </c>
       <c r="F11" s="37" t="s">
+        <v>843</v>
+      </c>
+      <c r="G11" s="75" t="s">
         <v>844</v>
       </c>
-      <c r="G11" s="75" t="s">
-        <v>845</v>
-      </c>
       <c r="H11" s="147" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="12" spans="1:9" s="33" customFormat="1" x14ac:dyDescent="0.3">
@@ -15106,16 +15280,16 @@
       <c r="A3" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="200" t="s">
-        <v>911</v>
-      </c>
-      <c r="C3" s="200"/>
-      <c r="D3" s="200"/>
-      <c r="E3" s="200"/>
-      <c r="F3" s="200"/>
-      <c r="G3" s="200"/>
-      <c r="H3" s="200"/>
-      <c r="I3" s="200"/>
+      <c r="B3" s="202" t="s">
+        <v>908</v>
+      </c>
+      <c r="C3" s="202"/>
+      <c r="D3" s="202"/>
+      <c r="E3" s="202"/>
+      <c r="F3" s="202"/>
+      <c r="G3" s="202"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="202"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -15148,7 +15322,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="178" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B6" s="179" t="s">
         <v>20</v>
@@ -15170,13 +15344,13 @@
     </row>
     <row r="7" spans="1:9" s="165" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="165" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B7" s="179" t="s">
         <v>36</v>
       </c>
       <c r="C7" s="166" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="D7" s="163" t="s">
         <v>131</v>
@@ -15185,13 +15359,13 @@
         <v>56</v>
       </c>
       <c r="F7" s="37" t="s">
+        <v>843</v>
+      </c>
+      <c r="G7" s="75" t="s">
         <v>844</v>
       </c>
-      <c r="G7" s="75" t="s">
-        <v>845</v>
-      </c>
       <c r="H7" s="178" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="165" customFormat="1" x14ac:dyDescent="0.3">
@@ -15203,137 +15377,31 @@
       <c r="H8" s="178"/>
     </row>
     <row r="9" spans="1:9" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
-        <v>139</v>
-      </c>
-      <c r="B9" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" s="170" t="s">
-        <v>140</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9" s="34">
-        <v>1</v>
-      </c>
-      <c r="G9" s="34">
-        <v>1</v>
-      </c>
-      <c r="H9" s="72">
-        <v>43101</v>
-      </c>
-      <c r="I9" s="33" t="s">
-        <v>141</v>
-      </c>
+      <c r="A9" s="208" t="s">
+        <v>929</v>
+      </c>
+      <c r="C9" s="170"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="72"/>
     </row>
     <row r="10" spans="1:9" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="B10" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="170" t="s">
-        <v>143</v>
-      </c>
-      <c r="E10" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="34">
-        <v>401768</v>
-      </c>
-      <c r="G10" s="34">
-        <v>401768</v>
-      </c>
-      <c r="H10" s="72">
-        <v>401404</v>
-      </c>
-      <c r="I10" s="33" t="s">
-        <v>141</v>
-      </c>
+      <c r="C10" s="170"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="72"/>
     </row>
     <row r="11" spans="1:9" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="33" t="s">
-        <v>144</v>
-      </c>
-      <c r="B11" s="33" t="s">
-        <v>145</v>
-      </c>
-      <c r="C11" s="170" t="s">
-        <v>146</v>
-      </c>
-      <c r="E11" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="33">
-        <v>1</v>
-      </c>
-      <c r="G11" s="33">
-        <v>1</v>
-      </c>
-      <c r="H11" s="178">
-        <v>1</v>
-      </c>
-      <c r="I11" s="33" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" s="33" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="33" t="s">
-        <v>148</v>
-      </c>
-      <c r="B12" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="170" t="s">
-        <v>149</v>
-      </c>
-      <c r="E12" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="G12" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="H12" s="178" t="s">
-        <v>150</v>
-      </c>
-      <c r="I12" s="33" t="s">
-        <v>141</v>
-      </c>
+      <c r="C11" s="170"/>
+      <c r="H11" s="178"/>
+    </row>
+    <row r="12" spans="1:9" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="170"/>
+      <c r="H12" s="178"/>
     </row>
     <row r="13" spans="1:9" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="170" t="s">
-        <v>147</v>
-      </c>
-      <c r="D13" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="E13" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="33">
-        <v>0</v>
-      </c>
-      <c r="G13" s="33">
-        <v>0</v>
-      </c>
-      <c r="H13" s="33">
-        <v>1</v>
-      </c>
-      <c r="I13" s="98" t="s">
-        <v>573</v>
-      </c>
+      <c r="C13" s="170"/>
+      <c r="I13" s="98"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -15341,7 +15409,6 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{CD3449D9-FB3E-4CDC-9A8F-AA4EC5796156}"/>
-    <hyperlink ref="I13" location="'Process Metadata'!A25" display="Import_Batch_Process_Task" xr:uid="{950B268C-FB55-4991-9940-E773BF176175}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -15390,7 +15457,7 @@
         <v>127</v>
       </c>
       <c r="B2" s="95" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="C2" s="47" t="s">
         <v>128</v>
@@ -15400,16 +15467,16 @@
       <c r="A3" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="200" t="s">
-        <v>871</v>
-      </c>
-      <c r="C3" s="200"/>
-      <c r="D3" s="200"/>
-      <c r="E3" s="200"/>
-      <c r="F3" s="200"/>
-      <c r="G3" s="200"/>
-      <c r="H3" s="200"/>
-      <c r="I3" s="200"/>
+      <c r="B3" s="202" t="s">
+        <v>870</v>
+      </c>
+      <c r="C3" s="202"/>
+      <c r="D3" s="202"/>
+      <c r="E3" s="202"/>
+      <c r="F3" s="202"/>
+      <c r="G3" s="202"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="202"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -15442,13 +15509,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="184" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B6" s="185" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="186" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="D6" s="178" t="s">
         <v>55</v>
@@ -15470,7 +15537,7 @@
         <v>61</v>
       </c>
       <c r="C7" s="189" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="D7" s="163" t="s">
         <v>131</v>
@@ -15481,19 +15548,19 @@
       <c r="F7" s="96"/>
       <c r="G7" s="96"/>
       <c r="H7" s="189" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="I7" s="163"/>
     </row>
     <row r="8" spans="1:9" s="165" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="190" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="B8" s="191" t="s">
         <v>36</v>
       </c>
       <c r="C8" s="153" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E8" s="69">
         <v>2</v>
@@ -15501,7 +15568,7 @@
       <c r="F8" s="37"/>
       <c r="G8" s="37"/>
       <c r="H8" s="153" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="165" customFormat="1" x14ac:dyDescent="0.3">
@@ -15512,7 +15579,7 @@
         <v>36</v>
       </c>
       <c r="C9" s="153" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="E9" s="69">
         <v>2</v>
@@ -15520,18 +15587,18 @@
       <c r="F9" s="37"/>
       <c r="G9" s="37"/>
       <c r="H9" s="153" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="165" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="190" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="B10" s="192" t="s">
         <v>659</v>
       </c>
       <c r="C10" s="153" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="E10" s="69">
         <v>2</v>
@@ -15539,7 +15606,7 @@
       <c r="F10" s="37"/>
       <c r="G10" s="37"/>
       <c r="H10" s="153" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="165" customFormat="1" x14ac:dyDescent="0.3">
@@ -15805,7 +15872,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="20.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42.33203125" style="136" customWidth="1"/>
@@ -15852,16 +15919,16 @@
       <c r="A3" s="138" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="201" t="s">
-        <v>892</v>
-      </c>
-      <c r="C3" s="201"/>
-      <c r="D3" s="201"/>
-      <c r="E3" s="201"/>
-      <c r="F3" s="201"/>
-      <c r="G3" s="201"/>
-      <c r="H3" s="201"/>
-      <c r="I3" s="201"/>
+      <c r="B3" s="203" t="s">
+        <v>891</v>
+      </c>
+      <c r="C3" s="203"/>
+      <c r="D3" s="203"/>
+      <c r="E3" s="203"/>
+      <c r="F3" s="203"/>
+      <c r="G3" s="203"/>
+      <c r="H3" s="203"/>
+      <c r="I3" s="203"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -15894,7 +15961,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="145" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B6" s="146" t="s">
         <v>20</v>
@@ -15934,7 +16001,7 @@
       <c r="F7" s="96"/>
       <c r="G7" s="96"/>
       <c r="H7" s="95" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="I7" s="163"/>
     </row>
@@ -15946,17 +16013,17 @@
         <v>659</v>
       </c>
       <c r="C8" s="166" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="D8" s="165"/>
       <c r="E8" s="69">
         <v>2</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="G8" s="75" t="s">
-        <v>662</v>
+        <v>925</v>
       </c>
       <c r="H8" s="75" t="s">
         <v>640</v>
@@ -15965,301 +16032,301 @@
     </row>
     <row r="9" spans="1:9" s="140" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="165" t="s">
-        <v>849</v>
-      </c>
-      <c r="B9" s="146" t="s">
+        <v>922</v>
+      </c>
+      <c r="B9" s="198" t="s">
+        <v>659</v>
+      </c>
+      <c r="C9" s="166" t="s">
+        <v>927</v>
+      </c>
+      <c r="D9" s="165"/>
+      <c r="E9" s="48">
+        <v>1</v>
+      </c>
+      <c r="F9" s="37" t="s">
+        <v>923</v>
+      </c>
+      <c r="G9" s="75" t="s">
+        <v>924</v>
+      </c>
+      <c r="H9" s="75" t="s">
+        <v>926</v>
+      </c>
+      <c r="I9" s="165" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="140" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="165" t="s">
+        <v>848</v>
+      </c>
+      <c r="B10" s="146" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="166" t="s">
-        <v>851</v>
-      </c>
-      <c r="D9" s="165"/>
-      <c r="E9" s="69">
-        <v>2</v>
-      </c>
-      <c r="F9" s="37" t="s">
-        <v>854</v>
-      </c>
-      <c r="G9" s="75" t="s">
-        <v>663</v>
-      </c>
-      <c r="H9" s="75" t="s">
-        <v>641</v>
-      </c>
-      <c r="I9" s="165"/>
-    </row>
-    <row r="10" spans="1:9" s="140" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="153" t="s">
-        <v>630</v>
-      </c>
-      <c r="B10" s="75" t="s">
-        <v>659</v>
-      </c>
-      <c r="C10" s="153" t="s">
-        <v>880</v>
+      <c r="C10" s="166" t="s">
+        <v>850</v>
       </c>
       <c r="D10" s="165"/>
       <c r="E10" s="69">
         <v>2</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>885</v>
-      </c>
-      <c r="G10" s="37" t="s">
-        <v>664</v>
+        <v>853</v>
+      </c>
+      <c r="G10" s="75" t="s">
+        <v>663</v>
       </c>
       <c r="H10" s="75" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="I10" s="165"/>
     </row>
-    <row r="11" spans="1:9" s="134" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" s="140" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="153" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B11" s="75" t="s">
         <v>659</v>
       </c>
       <c r="C11" s="153" t="s">
-        <v>881</v>
-      </c>
-      <c r="D11" s="33"/>
+        <v>879</v>
+      </c>
+      <c r="D11" s="165"/>
       <c r="E11" s="69">
         <v>2</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>669</v>
+        <v>884</v>
       </c>
       <c r="G11" s="37" t="s">
-        <v>665</v>
-      </c>
-      <c r="H11" s="72"/>
-      <c r="I11" s="33"/>
+        <v>664</v>
+      </c>
+      <c r="H11" s="75" t="s">
+        <v>642</v>
+      </c>
+      <c r="I11" s="165"/>
     </row>
     <row r="12" spans="1:9" s="134" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="153" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B12" s="75" t="s">
-        <v>36</v>
+        <v>659</v>
       </c>
       <c r="C12" s="153" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="D12" s="33"/>
       <c r="E12" s="69">
         <v>2</v>
       </c>
-      <c r="F12" s="167" t="s">
-        <v>886</v>
-      </c>
-      <c r="G12" s="167" t="s">
-        <v>666</v>
-      </c>
-      <c r="H12" s="72" t="s">
-        <v>643</v>
-      </c>
+      <c r="F12" s="37" t="s">
+        <v>669</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>665</v>
+      </c>
+      <c r="H12" s="72"/>
       <c r="I12" s="33"/>
     </row>
     <row r="13" spans="1:9" s="134" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="153" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B13" s="75" t="s">
-        <v>660</v>
+        <v>36</v>
       </c>
       <c r="C13" s="153" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="D13" s="33"/>
       <c r="E13" s="69">
         <v>2</v>
       </c>
-      <c r="F13" s="168" t="s">
-        <v>667</v>
-      </c>
-      <c r="G13" s="168" t="s">
-        <v>667</v>
-      </c>
-      <c r="H13" s="145">
-        <v>1200</v>
+      <c r="F13" s="167" t="s">
+        <v>885</v>
+      </c>
+      <c r="G13" s="167" t="s">
+        <v>666</v>
+      </c>
+      <c r="H13" s="72" t="s">
+        <v>643</v>
       </c>
       <c r="I13" s="33"/>
     </row>
-    <row r="14" spans="1:9" s="134" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" s="134" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="153" t="s">
-        <v>878</v>
+        <v>633</v>
       </c>
       <c r="B14" s="75" t="s">
-        <v>686</v>
+        <v>660</v>
       </c>
       <c r="C14" s="153" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="D14" s="33"/>
       <c r="E14" s="69">
         <v>2</v>
       </c>
       <c r="F14" s="168" t="s">
-        <v>887</v>
+        <v>667</v>
       </c>
       <c r="G14" s="168" t="s">
-        <v>888</v>
-      </c>
-      <c r="H14" s="146" t="s">
-        <v>889</v>
+        <v>667</v>
+      </c>
+      <c r="H14" s="145">
+        <v>1200</v>
       </c>
       <c r="I14" s="33"/>
     </row>
     <row r="15" spans="1:9" s="134" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="153" t="s">
-        <v>912</v>
+        <v>877</v>
       </c>
       <c r="B15" s="75" t="s">
-        <v>66</v>
+        <v>686</v>
       </c>
       <c r="C15" s="153" t="s">
-        <v>898</v>
+        <v>883</v>
       </c>
       <c r="D15" s="33"/>
       <c r="E15" s="69">
         <v>2</v>
       </c>
       <c r="F15" s="168" t="s">
-        <v>899</v>
+        <v>886</v>
       </c>
       <c r="G15" s="168" t="s">
-        <v>900</v>
-      </c>
-      <c r="H15" s="75" t="s">
-        <v>679</v>
+        <v>887</v>
+      </c>
+      <c r="H15" s="146" t="s">
+        <v>888</v>
       </c>
       <c r="I15" s="33"/>
     </row>
-    <row r="16" spans="1:9" s="134" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" s="134" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="153" t="s">
-        <v>901</v>
+        <v>909</v>
       </c>
       <c r="B16" s="75" t="s">
         <v>66</v>
       </c>
       <c r="C16" s="153" t="s">
-        <v>913</v>
+        <v>897</v>
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="69">
         <v>2</v>
       </c>
       <c r="F16" s="168" t="s">
-        <v>903</v>
+        <v>898</v>
       </c>
       <c r="G16" s="168" t="s">
-        <v>904</v>
-      </c>
-      <c r="H16" t="s">
-        <v>637</v>
+        <v>899</v>
+      </c>
+      <c r="H16" s="75" t="s">
+        <v>679</v>
       </c>
       <c r="I16" s="33"/>
     </row>
-    <row r="17" spans="1:9" s="134" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" s="134" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="153" t="s">
-        <v>879</v>
+        <v>900</v>
       </c>
       <c r="B17" s="75" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="C17" s="153" t="s">
-        <v>902</v>
+        <v>910</v>
       </c>
       <c r="D17" s="33"/>
       <c r="E17" s="69">
         <v>2</v>
       </c>
       <c r="F17" s="168" t="s">
-        <v>887</v>
+        <v>902</v>
       </c>
       <c r="G17" s="168" t="s">
-        <v>888</v>
-      </c>
-      <c r="H17" s="168" t="s">
-        <v>691</v>
-      </c>
-      <c r="I17" s="98"/>
+        <v>903</v>
+      </c>
+      <c r="H17" t="s">
+        <v>637</v>
+      </c>
+      <c r="I17" s="33"/>
     </row>
     <row r="18" spans="1:9" s="134" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="169" t="s">
-        <v>908</v>
+      <c r="A18" s="153" t="s">
+        <v>878</v>
       </c>
       <c r="B18" s="75" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18" s="169" t="s">
-        <v>894</v>
+        <v>36</v>
+      </c>
+      <c r="C18" s="153" t="s">
+        <v>901</v>
       </c>
       <c r="D18" s="33"/>
       <c r="E18" s="69">
         <v>2</v>
       </c>
       <c r="F18" s="168" t="s">
+        <v>886</v>
+      </c>
+      <c r="G18" s="168" t="s">
+        <v>887</v>
+      </c>
+      <c r="H18" s="168" t="s">
+        <v>691</v>
+      </c>
+      <c r="I18" s="98"/>
+    </row>
+    <row r="19" spans="1:9" s="134" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="169" t="s">
+        <v>907</v>
+      </c>
+      <c r="B19" s="75" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="169" t="s">
+        <v>893</v>
+      </c>
+      <c r="D19" s="33"/>
+      <c r="E19" s="69">
+        <v>2</v>
+      </c>
+      <c r="F19" s="168" t="s">
         <v>661</v>
       </c>
-      <c r="G18" s="168" t="s">
+      <c r="G19" s="168" t="s">
         <v>661</v>
       </c>
-      <c r="H18" s="168" t="s">
+      <c r="H19" s="168" t="s">
         <v>694</v>
       </c>
-      <c r="I18" s="98"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="33" t="s">
-        <v>139</v>
-      </c>
-      <c r="B19" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="C19" s="170" t="s">
-        <v>140</v>
-      </c>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="34">
-        <v>1</v>
-      </c>
-      <c r="G19" s="34">
-        <v>1</v>
-      </c>
-      <c r="H19" s="171">
-        <v>43101</v>
-      </c>
-      <c r="I19" s="33" t="s">
-        <v>141</v>
-      </c>
+      <c r="I19" s="98"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="33" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B20" s="33" t="s">
         <v>57</v>
       </c>
       <c r="C20" s="170" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D20" s="33"/>
       <c r="E20" s="33" t="s">
         <v>56</v>
       </c>
       <c r="F20" s="34">
-        <v>401768</v>
+        <v>1</v>
       </c>
       <c r="G20" s="34">
-        <v>401768</v>
+        <v>1</v>
       </c>
       <c r="H20" s="171">
-        <v>401404</v>
+        <v>43101</v>
       </c>
       <c r="I20" s="33" t="s">
         <v>141</v>
@@ -16267,97 +16334,113 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="33" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>145</v>
+        <v>57</v>
       </c>
       <c r="C21" s="170" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D21" s="33"/>
       <c r="E21" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="F21" s="33">
-        <v>1</v>
-      </c>
-      <c r="G21" s="33">
-        <v>1</v>
-      </c>
-      <c r="H21" s="172">
-        <v>1</v>
+      <c r="F21" s="34">
+        <v>401768</v>
+      </c>
+      <c r="G21" s="34">
+        <v>401768</v>
+      </c>
+      <c r="H21" s="171">
+        <v>401404</v>
       </c>
       <c r="I21" s="33" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="33" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>66</v>
+        <v>145</v>
       </c>
       <c r="C22" s="170" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D22" s="33"/>
       <c r="E22" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="F22" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="G22" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="H22" s="172" t="s">
-        <v>150</v>
+      <c r="F22" s="33">
+        <v>1</v>
+      </c>
+      <c r="G22" s="33">
+        <v>1</v>
+      </c>
+      <c r="H22" s="172">
+        <v>1</v>
       </c>
       <c r="I22" s="33" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="33" t="s">
-        <v>19</v>
+        <v>148</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="C23" s="170" t="s">
-        <v>147</v>
-      </c>
-      <c r="D23" s="33" t="s">
-        <v>98</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="D23" s="33"/>
       <c r="E23" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="F23" s="33">
+      <c r="F23" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="G23" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="H23" s="172" t="s">
+        <v>150</v>
+      </c>
+      <c r="I23" s="33" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="170" t="s">
+        <v>147</v>
+      </c>
+      <c r="D24" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>56</v>
+      </c>
+      <c r="F24" s="33">
         <v>0</v>
       </c>
-      <c r="G23" s="33">
+      <c r="G24" s="33">
         <v>0</v>
       </c>
-      <c r="H23" s="173">
+      <c r="H24" s="173">
         <v>1</v>
       </c>
-      <c r="I23" s="98" t="s">
+      <c r="I24" s="98" t="s">
         <v>573</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="134"/>
-      <c r="B24" s="134"/>
-      <c r="C24" s="135"/>
-      <c r="D24" s="134"/>
-      <c r="E24" s="134"/>
-      <c r="F24" s="134"/>
-      <c r="G24" s="134"/>
-      <c r="H24" s="144"/>
-      <c r="I24" s="134"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="134"/>
@@ -16367,6 +16450,7 @@
       <c r="E25" s="134"/>
       <c r="F25" s="134"/>
       <c r="G25" s="134"/>
+      <c r="H25" s="144"/>
       <c r="I25" s="134"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -16377,8 +16461,18 @@
       <c r="E26" s="134"/>
       <c r="F26" s="134"/>
       <c r="G26" s="134"/>
-      <c r="H26" s="134"/>
-      <c r="I26" s="137"/>
+      <c r="I26" s="134"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="134"/>
+      <c r="B27" s="134"/>
+      <c r="C27" s="135"/>
+      <c r="D27" s="134"/>
+      <c r="E27" s="134"/>
+      <c r="F27" s="134"/>
+      <c r="G27" s="134"/>
+      <c r="H27" s="134"/>
+      <c r="I27" s="137"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -16387,7 +16481,7 @@
   <phoneticPr fontId="19" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{BDFE1917-7BEB-4B2B-ADC4-70EB3929B98C}"/>
-    <hyperlink ref="I23" location="'Process Metadata'!A25" display="Import_Batch_Process_Task" xr:uid="{E2A21F73-57A4-432D-9FFB-58EFDE717546}"/>
+    <hyperlink ref="I24" location="'Process Metadata'!A25" display="Import_Batch_Process_Task" xr:uid="{E2A21F73-57A4-432D-9FFB-58EFDE717546}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -16438,16 +16532,16 @@
       <c r="A3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="200" t="s">
+      <c r="B3" s="202" t="s">
         <v>409</v>
       </c>
-      <c r="C3" s="200"/>
-      <c r="D3" s="200"/>
-      <c r="E3" s="200"/>
-      <c r="F3" s="200"/>
-      <c r="G3" s="200"/>
-      <c r="H3" s="200"/>
-      <c r="I3" s="200"/>
+      <c r="C3" s="202"/>
+      <c r="D3" s="202"/>
+      <c r="E3" s="202"/>
+      <c r="F3" s="202"/>
+      <c r="G3" s="202"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="202"/>
     </row>
     <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -16937,7 +17031,7 @@
   <cols>
     <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" customWidth="1"/>
-    <col min="3" max="3" width="10.88671875" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -16978,14 +17072,16 @@
         <v>218</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>705</v>
       </c>
       <c r="B3" t="s">
         <v>209</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>930</v>
+      </c>
       <c r="D3" t="s">
         <v>345</v>
       </c>
@@ -17009,7 +17105,9 @@
       <c r="B4" t="s">
         <v>210</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="2" t="s">
+        <v>931</v>
+      </c>
       <c r="E4" t="s">
         <v>155</v>
       </c>
@@ -17023,14 +17121,16 @@
         <v>710</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>711</v>
       </c>
       <c r="B5" t="s">
         <v>210</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>932</v>
+      </c>
       <c r="E5" t="s">
         <v>155</v>
       </c>
@@ -17090,17 +17190,19 @@
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" style="75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" style="75" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" style="75" customWidth="1"/>
+    <col min="4" max="4" width="11" style="75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" style="75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.88671875" style="75"/>
+    <col min="7" max="8" width="10.6640625" style="75" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="75" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="75"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="98" t="s">
         <v>5</v>
       </c>
     </row>
@@ -17133,21 +17235,23 @@
         <v>218</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="210" t="s">
         <v>713</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" t="s">
+      <c r="C3" s="47" t="s">
+        <v>933</v>
+      </c>
+      <c r="D3" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="75" t="s">
         <v>155</v>
       </c>
       <c r="G3" s="75">
@@ -17157,18 +17261,20 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="210" t="s">
         <v>714</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="E4" t="s">
+      <c r="C4" s="47" t="s">
+        <v>934</v>
+      </c>
+      <c r="E4" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="75" t="s">
         <v>345</v>
       </c>
       <c r="G4" s="75">
@@ -17179,20 +17285,22 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="210" t="s">
         <v>715</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" t="s">
+      <c r="C5" s="47" t="s">
+        <v>935</v>
+      </c>
+      <c r="D5" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="75" t="s">
         <v>345</v>
       </c>
       <c r="G5" s="118">
@@ -17202,69 +17310,78 @@
         <v>43791</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="210" t="s">
         <v>716</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="75" t="s">
         <v>717</v>
       </c>
-      <c r="D6" t="s">
+      <c r="C6" s="47" t="s">
+        <v>936</v>
+      </c>
+      <c r="D6" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="75" t="s">
         <v>718</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="75" t="s">
         <v>719</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
+    <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="210" t="s">
         <v>720</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="75" t="s">
         <v>209</v>
       </c>
-      <c r="D7" t="s">
+      <c r="C7" s="47" t="s">
+        <v>937</v>
+      </c>
+      <c r="D7" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="75" t="s">
         <v>721</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="75" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
+    <row r="8" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="210" t="s">
         <v>723</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="75" t="s">
         <v>724</v>
       </c>
-      <c r="E8" t="s">
+      <c r="C8" s="47" t="s">
+        <v>938</v>
+      </c>
+      <c r="E8" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="75" t="s">
         <v>345</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="75">
         <v>0.5</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="75">
         <v>6</v>
       </c>
     </row>
@@ -17286,7 +17403,7 @@
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.5546875" customWidth="1"/>
     <col min="6" max="6" width="11.5546875" customWidth="1"/>
@@ -17339,6 +17456,9 @@
       <c r="B4" t="s">
         <v>209</v>
       </c>
+      <c r="C4" t="s">
+        <v>939</v>
+      </c>
       <c r="D4" t="s">
         <v>740</v>
       </c>
@@ -17362,6 +17482,9 @@
       <c r="B5" t="s">
         <v>57</v>
       </c>
+      <c r="C5" t="s">
+        <v>906</v>
+      </c>
       <c r="E5" t="s">
         <v>741</v>
       </c>
@@ -17382,6 +17505,9 @@
       <c r="B6" t="s">
         <v>209</v>
       </c>
+      <c r="C6" t="s">
+        <v>941</v>
+      </c>
       <c r="E6" t="s">
         <v>741</v>
       </c>
@@ -17402,6 +17528,9 @@
       <c r="B7" t="s">
         <v>210</v>
       </c>
+      <c r="C7" t="s">
+        <v>942</v>
+      </c>
       <c r="E7" t="s">
         <v>740</v>
       </c>
@@ -17422,6 +17551,9 @@
       <c r="B8" t="s">
         <v>749</v>
       </c>
+      <c r="C8" t="s">
+        <v>943</v>
+      </c>
       <c r="E8" t="s">
         <v>741</v>
       </c>
@@ -17442,6 +17574,9 @@
       <c r="B9" t="s">
         <v>210</v>
       </c>
+      <c r="C9" t="s">
+        <v>944</v>
+      </c>
       <c r="E9" t="s">
         <v>740</v>
       </c>
@@ -17456,6 +17591,9 @@
       <c r="B10" t="s">
         <v>752</v>
       </c>
+      <c r="C10" t="s">
+        <v>945</v>
+      </c>
       <c r="E10" t="s">
         <v>740</v>
       </c>
@@ -17476,6 +17614,9 @@
       <c r="B11" t="s">
         <v>752</v>
       </c>
+      <c r="C11" t="s">
+        <v>946</v>
+      </c>
       <c r="E11" t="s">
         <v>740</v>
       </c>
@@ -17496,6 +17637,9 @@
       <c r="B12" t="s">
         <v>752</v>
       </c>
+      <c r="C12" t="s">
+        <v>947</v>
+      </c>
       <c r="E12" t="s">
         <v>740</v>
       </c>
@@ -17509,12 +17653,15 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="125" t="s">
         <v>755</v>
       </c>
       <c r="B13" t="s">
         <v>209</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>948</v>
       </c>
       <c r="E13" t="s">
         <v>740</v>
@@ -17810,7 +17957,7 @@
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.44140625" bestFit="1" customWidth="1"/>
@@ -17860,6 +18007,9 @@
       <c r="B4" t="s">
         <v>677</v>
       </c>
+      <c r="C4" t="s">
+        <v>949</v>
+      </c>
       <c r="D4" t="s">
         <v>345</v>
       </c>
@@ -17883,6 +18033,9 @@
       <c r="B5" t="s">
         <v>647</v>
       </c>
+      <c r="C5" t="s">
+        <v>950</v>
+      </c>
       <c r="E5" t="s">
         <v>155</v>
       </c>
@@ -17896,12 +18049,15 @@
         <v>693</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>690</v>
       </c>
       <c r="B6" t="s">
         <v>677</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>951</v>
       </c>
       <c r="E6" t="s">
         <v>155</v>
@@ -17934,7 +18090,7 @@
   <cols>
     <col min="1" max="1" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.109375" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.33203125" customWidth="1"/>
     <col min="6" max="6" width="15.44140625" bestFit="1" customWidth="1"/>
@@ -17984,6 +18140,9 @@
       <c r="B4" t="s">
         <v>645</v>
       </c>
+      <c r="C4" t="s">
+        <v>952</v>
+      </c>
       <c r="D4" t="s">
         <v>345</v>
       </c>
@@ -18007,6 +18166,9 @@
       <c r="B5" t="s">
         <v>676</v>
       </c>
+      <c r="C5" t="s">
+        <v>953</v>
+      </c>
       <c r="E5" t="s">
         <v>155</v>
       </c>
@@ -18020,12 +18182,15 @@
         <v>681</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>675</v>
       </c>
       <c r="B6" t="s">
         <v>677</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>954</v>
       </c>
       <c r="E6" t="s">
         <v>155</v>
@@ -18058,7 +18223,7 @@
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.109375" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.33203125" customWidth="1"/>
     <col min="6" max="6" width="15.44140625" bestFit="1" customWidth="1"/>
@@ -18108,7 +18273,9 @@
       <c r="B4" s="115" t="s">
         <v>645</v>
       </c>
-      <c r="C4" s="115"/>
+      <c r="C4" s="115" t="s">
+        <v>940</v>
+      </c>
       <c r="D4" s="115" t="s">
         <v>345</v>
       </c>
@@ -18132,7 +18299,9 @@
       <c r="B5" s="115" t="s">
         <v>645</v>
       </c>
-      <c r="C5" s="115"/>
+      <c r="C5" s="115" t="s">
+        <v>956</v>
+      </c>
       <c r="D5" s="115"/>
       <c r="E5" s="115" t="s">
         <v>155</v>
@@ -18154,7 +18323,9 @@
       <c r="B6" s="115" t="s">
         <v>646</v>
       </c>
-      <c r="C6" s="115"/>
+      <c r="C6" s="115" t="s">
+        <v>955</v>
+      </c>
       <c r="D6" s="115"/>
       <c r="E6" s="115" t="s">
         <v>155</v>
@@ -18176,7 +18347,9 @@
       <c r="B7" s="115" t="s">
         <v>647</v>
       </c>
-      <c r="C7" s="115"/>
+      <c r="C7" s="115" t="s">
+        <v>957</v>
+      </c>
       <c r="D7" s="115"/>
       <c r="E7" s="115" t="s">
         <v>155</v>
@@ -18198,7 +18371,9 @@
       <c r="B8" s="115" t="s">
         <v>646</v>
       </c>
-      <c r="C8" s="115"/>
+      <c r="C8" s="115" t="s">
+        <v>879</v>
+      </c>
       <c r="D8" s="115"/>
       <c r="E8" s="115" t="s">
         <v>345</v>
@@ -18217,7 +18392,9 @@
       <c r="B9" s="115" t="s">
         <v>646</v>
       </c>
-      <c r="C9" s="115"/>
+      <c r="C9" s="115" t="s">
+        <v>880</v>
+      </c>
       <c r="D9" s="115"/>
       <c r="E9" s="115" t="s">
         <v>345</v>
@@ -18234,7 +18411,9 @@
       <c r="B10" s="115" t="s">
         <v>647</v>
       </c>
-      <c r="C10" s="115"/>
+      <c r="C10" s="115" t="s">
+        <v>958</v>
+      </c>
       <c r="D10" s="115"/>
       <c r="E10" s="115" t="s">
         <v>345</v>
@@ -18253,7 +18432,9 @@
       <c r="B11" s="115" t="s">
         <v>648</v>
       </c>
-      <c r="C11" s="115"/>
+      <c r="C11" s="115" t="s">
+        <v>959</v>
+      </c>
       <c r="D11" s="115"/>
       <c r="E11" s="115" t="s">
         <v>345</v>
@@ -18803,14 +18984,14 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="198" t="s">
+      <c r="A8" s="200" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="198"/>
-      <c r="C8" s="198"/>
-      <c r="D8" s="198"/>
-      <c r="E8" s="198"/>
-      <c r="F8" s="198"/>
+      <c r="B8" s="200"/>
+      <c r="C8" s="200"/>
+      <c r="D8" s="200"/>
+      <c r="E8" s="200"/>
+      <c r="F8" s="200"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
@@ -18970,14 +19151,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="198" t="s">
+      <c r="A18" s="200" t="s">
         <v>485</v>
       </c>
-      <c r="B18" s="198"/>
-      <c r="C18" s="198"/>
-      <c r="D18" s="198"/>
-      <c r="E18" s="198"/>
-      <c r="F18" s="198"/>
+      <c r="B18" s="200"/>
+      <c r="C18" s="200"/>
+      <c r="D18" s="200"/>
+      <c r="E18" s="200"/>
+      <c r="F18" s="200"/>
     </row>
     <row r="19" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
@@ -18986,11 +19167,11 @@
       <c r="B19" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="197" t="s">
+      <c r="C19" s="199" t="s">
         <v>470</v>
       </c>
-      <c r="D19" s="197"/>
-      <c r="E19" s="197"/>
+      <c r="D19" s="199"/>
+      <c r="E19" s="199"/>
       <c r="F19" s="11"/>
     </row>
     <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -19016,14 +19197,14 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="199" t="s">
+      <c r="A23" s="201" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="199"/>
-      <c r="C23" s="199"/>
-      <c r="D23" s="199"/>
-      <c r="E23" s="199"/>
-      <c r="F23" s="199"/>
+      <c r="B23" s="201"/>
+      <c r="C23" s="201"/>
+      <c r="D23" s="201"/>
+      <c r="E23" s="201"/>
+      <c r="F23" s="201"/>
     </row>
     <row r="24" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
@@ -19032,11 +19213,11 @@
       <c r="B24" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="197" t="s">
+      <c r="C24" s="199" t="s">
         <v>482</v>
       </c>
-      <c r="D24" s="197"/>
-      <c r="E24" s="197"/>
+      <c r="D24" s="199"/>
+      <c r="E24" s="199"/>
       <c r="F24" s="8" t="s">
         <v>23</v>
       </c>
@@ -19084,14 +19265,14 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="199" t="s">
+      <c r="A29" s="201" t="s">
         <v>468</v>
       </c>
-      <c r="B29" s="199"/>
-      <c r="C29" s="199"/>
-      <c r="D29" s="199"/>
-      <c r="E29" s="199"/>
-      <c r="F29" s="199"/>
+      <c r="B29" s="201"/>
+      <c r="C29" s="201"/>
+      <c r="D29" s="201"/>
+      <c r="E29" s="201"/>
+      <c r="F29" s="201"/>
     </row>
     <row r="30" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
@@ -19100,11 +19281,11 @@
       <c r="B30" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="197" t="s">
+      <c r="C30" s="199" t="s">
         <v>470</v>
       </c>
-      <c r="D30" s="197"/>
-      <c r="E30" s="197"/>
+      <c r="D30" s="199"/>
+      <c r="E30" s="199"/>
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -19156,30 +19337,33 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="73.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="44.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="73.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="44.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="75"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D1" s="75"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C2" s="75"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D2" s="75"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
@@ -19190,19 +19374,22 @@
         <v>494</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>725</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="115" t="s">
         <v>651</v>
       </c>
@@ -19212,20 +19399,23 @@
       <c r="C4" t="s">
         <v>155</v>
       </c>
-      <c r="D4" s="116" t="s">
+      <c r="D4" s="115" t="s">
+        <v>940</v>
+      </c>
+      <c r="E4" s="116" t="s">
         <v>661</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>634</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>635</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="115" t="s">
         <v>652</v>
       </c>
@@ -19235,17 +19425,20 @@
       <c r="C5" t="s">
         <v>155</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="115" t="s">
+        <v>956</v>
+      </c>
+      <c r="E5" t="s">
         <v>134</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>668</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="115" t="s">
         <v>653</v>
       </c>
@@ -19255,17 +19448,20 @@
       <c r="C6" t="s">
         <v>155</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="115" t="s">
+        <v>955</v>
+      </c>
+      <c r="E6" t="s">
         <v>662</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>640</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="115" t="s">
         <v>654</v>
       </c>
@@ -19275,17 +19471,20 @@
       <c r="C7" t="s">
         <v>155</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="115" t="s">
+        <v>957</v>
+      </c>
+      <c r="E7" t="s">
         <v>663</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>641</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="115" t="s">
         <v>655</v>
       </c>
@@ -19295,17 +19494,20 @@
       <c r="C8" t="s">
         <v>155</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="115" t="s">
+        <v>879</v>
+      </c>
+      <c r="E8" t="s">
         <v>664</v>
       </c>
-      <c r="E8" s="115" t="s">
+      <c r="F8" s="115" t="s">
         <v>642</v>
       </c>
-      <c r="F8" s="115" t="s">
+      <c r="G8" s="115" t="s">
         <v>664</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="115" t="s">
         <v>656</v>
       </c>
@@ -19315,20 +19517,23 @@
       <c r="C9" t="s">
         <v>155</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="115" t="s">
+        <v>880</v>
+      </c>
+      <c r="E9" t="s">
         <v>665</v>
       </c>
-      <c r="E9" s="115" t="s">
+      <c r="F9" s="115" t="s">
         <v>669</v>
       </c>
-      <c r="F9" s="115" t="s">
+      <c r="G9" s="115" t="s">
         <v>664</v>
       </c>
-      <c r="G9" s="115" t="s">
+      <c r="H9" s="115" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="115" t="s">
         <v>657</v>
       </c>
@@ -19338,17 +19543,20 @@
       <c r="C10" t="s">
         <v>155</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="115" t="s">
+        <v>958</v>
+      </c>
+      <c r="E10" t="s">
         <v>666</v>
       </c>
-      <c r="E10" s="115" t="s">
+      <c r="F10" s="115" t="s">
         <v>643</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>666</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="115" t="s">
         <v>658</v>
       </c>
@@ -19358,17 +19566,20 @@
       <c r="C11" t="s">
         <v>155</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="115" t="s">
+        <v>959</v>
+      </c>
+      <c r="E11" t="s">
         <v>667</v>
       </c>
-      <c r="E11" s="117">
+      <c r="F11" s="117">
         <v>1200</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>667</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="115" t="s">
         <v>19</v>
       </c>
@@ -19378,13 +19589,16 @@
       <c r="C12" t="s">
         <v>155</v>
       </c>
-      <c r="E12" s="75">
-        <v>1</v>
+      <c r="D12" s="209" t="s">
+        <v>257</v>
       </c>
       <c r="F12" s="75">
         <v>1</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="75">
+        <v>1</v>
+      </c>
+      <c r="H12" t="s">
         <v>672</v>
       </c>
     </row>
@@ -19402,31 +19616,34 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="44.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="44.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="75"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D1" s="75"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C2" s="75"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D2" s="75"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
@@ -19437,19 +19654,22 @@
         <v>494</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>725</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>683</v>
       </c>
@@ -19460,19 +19680,22 @@
         <v>155</v>
       </c>
       <c r="D4" t="s">
+        <v>952</v>
+      </c>
+      <c r="E4" t="s">
         <v>661</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>637</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>680</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>684</v>
       </c>
@@ -19483,16 +19706,19 @@
         <v>155</v>
       </c>
       <c r="D5" t="s">
+        <v>953</v>
+      </c>
+      <c r="E5" t="s">
         <v>687</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>678</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>681</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>685</v>
       </c>
@@ -19502,17 +19728,20 @@
       <c r="C6" t="s">
         <v>155</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
+        <v>954</v>
+      </c>
+      <c r="E6" t="s">
         <v>134</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>679</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>682</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="115" t="s">
         <v>19</v>
       </c>
@@ -19522,13 +19751,16 @@
       <c r="C7" t="s">
         <v>155</v>
       </c>
-      <c r="E7" s="75">
-        <v>1</v>
+      <c r="D7" s="209" t="s">
+        <v>257</v>
       </c>
       <c r="F7" s="75">
         <v>1</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="75">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
         <v>672</v>
       </c>
     </row>
@@ -19545,30 +19777,33 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="83.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.88671875" customWidth="1"/>
+    <col min="5" max="5" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="83.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="75"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D1" s="75"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C2" s="75"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D2" s="75"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
@@ -19579,19 +19814,22 @@
         <v>494</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>725</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>705</v>
       </c>
@@ -19599,20 +19837,23 @@
         <v>61</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
+        <v>930</v>
+      </c>
+      <c r="E4" t="s">
         <v>661</v>
       </c>
-      <c r="E4" s="75" t="s">
+      <c r="F4" s="75" t="s">
         <v>706</v>
       </c>
-      <c r="F4" s="75" t="s">
+      <c r="G4" s="75" t="s">
         <v>707</v>
       </c>
-      <c r="G4" s="119" t="s">
+      <c r="H4" s="119" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>708</v>
       </c>
@@ -19620,18 +19861,21 @@
         <v>36</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" t="s">
+      <c r="D5" s="2" t="s">
+        <v>931</v>
+      </c>
+      <c r="E5" t="s">
         <v>733</v>
       </c>
-      <c r="E5" s="75" t="s">
+      <c r="F5" s="75" t="s">
         <v>709</v>
       </c>
-      <c r="F5" s="75" t="s">
+      <c r="G5" s="75" t="s">
         <v>710</v>
       </c>
-      <c r="G5" s="78"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" s="78"/>
+    </row>
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>711</v>
       </c>
@@ -19639,20 +19883,23 @@
         <v>36</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
+        <v>932</v>
+      </c>
+      <c r="E6" t="s">
         <v>734</v>
       </c>
-      <c r="E6" s="75" t="s">
+      <c r="F6" s="75" t="s">
         <v>709</v>
       </c>
-      <c r="F6" s="75" t="s">
+      <c r="G6" s="75" t="s">
         <v>712</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>730</v>
       </c>
@@ -19662,44 +19909,52 @@
       <c r="C7" s="75" t="s">
         <v>731</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="75">
-        <v>1</v>
-      </c>
+      <c r="D7" s="209" t="s">
+        <v>257</v>
+      </c>
+      <c r="E7" s="44"/>
       <c r="F7" s="75">
         <v>1</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="75">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
         <v>732</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="9"/>
       <c r="C8" s="2"/>
-      <c r="E8" s="75"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D8" s="2"/>
+      <c r="F8" s="75"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="9"/>
       <c r="C9" s="2"/>
-      <c r="E9" s="75"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D9" s="2"/>
+      <c r="F9" s="75"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="9"/>
       <c r="C10" s="2"/>
-      <c r="E10" s="75"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D10" s="2"/>
+      <c r="F10" s="75"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="9"/>
       <c r="C11" s="2"/>
-      <c r="E11" s="75"/>
+      <c r="D11" s="2"/>
       <c r="F11" s="75"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G11" s="75"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="9"/>
       <c r="C12" s="75"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="75"/>
+      <c r="D12" s="75"/>
+      <c r="E12" s="2"/>
       <c r="F12" s="75"/>
+      <c r="G12" s="75"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -19720,7 +19975,7 @@
     <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="55.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="42.109375" bestFit="1" customWidth="1"/>
@@ -19776,6 +20031,9 @@
       <c r="B4" t="s">
         <v>61</v>
       </c>
+      <c r="D4" t="s">
+        <v>939</v>
+      </c>
       <c r="E4" t="s">
         <v>661</v>
       </c>
@@ -19793,6 +20051,9 @@
       <c r="B5" t="s">
         <v>57</v>
       </c>
+      <c r="D5" t="s">
+        <v>906</v>
+      </c>
       <c r="E5" s="118">
         <v>43872</v>
       </c>
@@ -19810,6 +20071,9 @@
       <c r="B6" t="s">
         <v>61</v>
       </c>
+      <c r="D6" t="s">
+        <v>941</v>
+      </c>
       <c r="E6" t="s">
         <v>134</v>
       </c>
@@ -19827,6 +20091,9 @@
       <c r="B7" t="s">
         <v>36</v>
       </c>
+      <c r="D7" t="s">
+        <v>942</v>
+      </c>
       <c r="E7" t="s">
         <v>765</v>
       </c>
@@ -19844,6 +20111,9 @@
       <c r="B8" t="s">
         <v>767</v>
       </c>
+      <c r="D8" t="s">
+        <v>943</v>
+      </c>
       <c r="E8" t="s">
         <v>768</v>
       </c>
@@ -19861,6 +20131,9 @@
       <c r="B9" t="s">
         <v>36</v>
       </c>
+      <c r="D9" t="s">
+        <v>944</v>
+      </c>
       <c r="E9" t="s">
         <v>770</v>
       </c>
@@ -19872,6 +20145,9 @@
       <c r="B10" t="s">
         <v>772</v>
       </c>
+      <c r="D10" t="s">
+        <v>945</v>
+      </c>
       <c r="E10" t="s">
         <v>325</v>
       </c>
@@ -19889,6 +20165,9 @@
       <c r="B11" t="s">
         <v>772</v>
       </c>
+      <c r="D11" t="s">
+        <v>946</v>
+      </c>
       <c r="E11" t="s">
         <v>325</v>
       </c>
@@ -19906,6 +20185,9 @@
       <c r="B12" t="s">
         <v>772</v>
       </c>
+      <c r="D12" t="s">
+        <v>947</v>
+      </c>
       <c r="E12" t="s">
         <v>325</v>
       </c>
@@ -19916,13 +20198,16 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="125" t="s">
         <v>775</v>
       </c>
       <c r="B13" t="s">
         <v>61</v>
       </c>
+      <c r="D13" s="2" t="s">
+        <v>948</v>
+      </c>
       <c r="E13" t="s">
         <v>776</v>
       </c>
@@ -19933,12 +20218,15 @@
         <v>4604041</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="128" t="s">
         <v>19</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
+      </c>
+      <c r="D14" s="209" t="s">
+        <v>257</v>
       </c>
       <c r="F14" s="75">
         <v>1</v>
@@ -19960,29 +20248,32 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5546875" customWidth="1"/>
+    <col min="5" max="5" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="75"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D1" s="75"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C2" s="75"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D2" s="75"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
@@ -19993,19 +20284,22 @@
         <v>494</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>725</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>713</v>
       </c>
@@ -20013,20 +20307,23 @@
         <v>20</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
+        <v>933</v>
+      </c>
+      <c r="E4" t="s">
         <v>661</v>
-      </c>
-      <c r="E4" s="75">
-        <v>2019</v>
       </c>
       <c r="F4" s="75">
         <v>2019</v>
       </c>
-      <c r="G4" s="119" t="s">
+      <c r="G4" s="75">
+        <v>2019</v>
+      </c>
+      <c r="H4" s="119" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>714</v>
       </c>
@@ -20034,18 +20331,21 @@
         <v>20</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="75">
+      <c r="D5" s="2" t="s">
+        <v>934</v>
+      </c>
+      <c r="E5" s="75">
         <v>0</v>
       </c>
-      <c r="E5" s="75">
+      <c r="F5" s="75">
         <v>36</v>
       </c>
-      <c r="F5" s="75">
+      <c r="G5" s="75">
         <v>47</v>
       </c>
-      <c r="G5" s="78"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" s="78"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>715</v>
       </c>
@@ -20053,17 +20353,20 @@
         <v>57</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="118">
+      <c r="D6" s="2" t="s">
+        <v>935</v>
+      </c>
+      <c r="E6" s="118">
         <v>43872</v>
       </c>
-      <c r="E6" s="118">
+      <c r="F6" s="118">
         <v>43714</v>
       </c>
-      <c r="F6" s="118">
+      <c r="G6" s="118">
         <v>43791</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>716</v>
       </c>
@@ -20072,50 +20375,59 @@
       </c>
       <c r="C7" s="75"/>
       <c r="D7" s="2" t="s">
+        <v>936</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>728</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>718</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>719</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>720</v>
       </c>
       <c r="B8" t="s">
         <v>61</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2" t="s">
+        <v>937</v>
+      </c>
+      <c r="E8" t="s">
         <v>729</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>721</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>723</v>
       </c>
       <c r="B9" t="s">
         <v>724</v>
       </c>
-      <c r="D9" s="75" t="s">
+      <c r="D9" s="2" t="s">
+        <v>938</v>
+      </c>
+      <c r="E9" s="75" t="s">
         <v>325</v>
       </c>
-      <c r="E9" s="75">
+      <c r="F9" s="75">
         <v>0.5</v>
       </c>
-      <c r="F9" s="75">
+      <c r="G9" s="75">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>730</v>
       </c>
@@ -20125,14 +20437,17 @@
       <c r="C10" s="75" t="s">
         <v>731</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="75">
-        <v>1</v>
-      </c>
+      <c r="D10" s="209" t="s">
+        <v>257</v>
+      </c>
+      <c r="E10" s="2"/>
       <c r="F10" s="75">
         <v>1</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="75">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
         <v>732</v>
       </c>
     </row>
@@ -20195,7 +20510,7 @@
         <v>809</v>
       </c>
       <c r="L2" s="133" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -20250,7 +20565,7 @@
         <v>705</v>
       </c>
       <c r="J4" s="20" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="K4" s="20" t="s">
         <v>739</v>
@@ -20294,10 +20609,10 @@
         <v>124</v>
       </c>
       <c r="E6" s="131" t="s">
-        <v>816</v>
+        <v>911</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="I6" s="20" t="s">
         <v>44</v>
@@ -20313,16 +20628,16 @@
         <v>813</v>
       </c>
       <c r="C7" s="142" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="D7" s="20" t="s">
         <v>815</v>
       </c>
       <c r="E7" s="131" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
       <c r="J7" s="20" t="s">
         <v>44</v>
@@ -20341,10 +20656,10 @@
         <v>290</v>
       </c>
       <c r="G9" s="132" t="s">
+        <v>818</v>
+      </c>
+      <c r="K9" s="132" t="s">
         <v>819</v>
-      </c>
-      <c r="K9" s="132" t="s">
-        <v>820</v>
       </c>
     </row>
   </sheetData>
@@ -20373,30 +20688,33 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.5546875" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="44.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.44140625" customWidth="1"/>
+    <col min="6" max="6" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="44.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="75"/>
       <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C2" s="75"/>
       <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
@@ -20410,16 +20728,19 @@
         <v>725</v>
       </c>
       <c r="E3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>695</v>
       </c>
@@ -20430,16 +20751,19 @@
         <v>661</v>
       </c>
       <c r="E4" t="s">
+        <v>949</v>
+      </c>
+      <c r="F4" t="s">
         <v>679</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>682</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>696</v>
       </c>
@@ -20450,16 +20774,16 @@
         <v>661</v>
       </c>
       <c r="E5" t="s">
+        <v>950</v>
+      </c>
+      <c r="F5" t="s">
         <v>691</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>693</v>
       </c>
-      <c r="G5" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>697</v>
       </c>
@@ -20469,30 +20793,33 @@
       <c r="D6" s="116" t="s">
         <v>661</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
+        <v>951</v>
+      </c>
+      <c r="F6" t="s">
         <v>692</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>694</v>
       </c>
-      <c r="G6" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="115" t="s">
         <v>19</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="75">
-        <v>1</v>
+      <c r="E7" s="44" t="s">
+        <v>257</v>
       </c>
       <c r="F7" s="75">
         <v>1</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="75">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
         <v>672</v>
       </c>
     </row>
@@ -21139,14 +21466,14 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="198" t="s">
+      <c r="A8" s="200" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="198"/>
-      <c r="C8" s="198"/>
-      <c r="D8" s="198"/>
-      <c r="E8" s="198"/>
-      <c r="F8" s="198"/>
+      <c r="B8" s="200"/>
+      <c r="C8" s="200"/>
+      <c r="D8" s="200"/>
+      <c r="E8" s="200"/>
+      <c r="F8" s="200"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
@@ -21229,14 +21556,14 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="198" t="s">
+      <c r="A14" s="200" t="s">
         <v>485</v>
       </c>
-      <c r="B14" s="198"/>
-      <c r="C14" s="198"/>
-      <c r="D14" s="198"/>
-      <c r="E14" s="198"/>
-      <c r="F14" s="198"/>
+      <c r="B14" s="200"/>
+      <c r="C14" s="200"/>
+      <c r="D14" s="200"/>
+      <c r="E14" s="200"/>
+      <c r="F14" s="200"/>
     </row>
     <row r="15" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
@@ -21245,11 +21572,11 @@
       <c r="B15" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="197" t="s">
+      <c r="C15" s="199" t="s">
         <v>470</v>
       </c>
-      <c r="D15" s="197"/>
-      <c r="E15" s="197"/>
+      <c r="D15" s="199"/>
+      <c r="E15" s="199"/>
       <c r="F15" s="11"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -21264,14 +21591,14 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="199" t="s">
+      <c r="A20" s="201" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="199"/>
-      <c r="C20" s="199"/>
-      <c r="D20" s="199"/>
-      <c r="E20" s="199"/>
-      <c r="F20" s="199"/>
+      <c r="B20" s="201"/>
+      <c r="C20" s="201"/>
+      <c r="D20" s="201"/>
+      <c r="E20" s="201"/>
+      <c r="F20" s="201"/>
     </row>
     <row r="21" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -21280,11 +21607,11 @@
       <c r="B21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="197" t="s">
+      <c r="C21" s="199" t="s">
         <v>482</v>
       </c>
-      <c r="D21" s="197"/>
-      <c r="E21" s="197"/>
+      <c r="D21" s="199"/>
+      <c r="E21" s="199"/>
       <c r="F21" s="8" t="s">
         <v>23</v>
       </c>
@@ -21332,14 +21659,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="199" t="s">
+      <c r="A26" s="201" t="s">
         <v>468</v>
       </c>
-      <c r="B26" s="199"/>
-      <c r="C26" s="199"/>
-      <c r="D26" s="199"/>
-      <c r="E26" s="199"/>
-      <c r="F26" s="199"/>
+      <c r="B26" s="201"/>
+      <c r="C26" s="201"/>
+      <c r="D26" s="201"/>
+      <c r="E26" s="201"/>
+      <c r="F26" s="201"/>
     </row>
     <row r="27" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
@@ -21348,11 +21675,11 @@
       <c r="B27" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="197" t="s">
+      <c r="C27" s="199" t="s">
         <v>470</v>
       </c>
-      <c r="D27" s="197"/>
-      <c r="E27" s="197"/>
+      <c r="D27" s="199"/>
+      <c r="E27" s="199"/>
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -21470,10 +21797,10 @@
       <c r="F5" s="43"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="202" t="s">
+      <c r="A10" s="204" t="s">
         <v>497</v>
       </c>
-      <c r="B10" s="202"/>
+      <c r="B10" s="204"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
@@ -22505,7 +22832,7 @@
       <c r="F6" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="203" t="s">
+      <c r="J6" s="205" t="s">
         <v>467</v>
       </c>
     </row>
@@ -22522,7 +22849,7 @@
       <c r="F7" t="s">
         <v>95</v>
       </c>
-      <c r="J7" s="203"/>
+      <c r="J7" s="205"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -22534,7 +22861,7 @@
       <c r="F8" t="s">
         <v>93</v>
       </c>
-      <c r="J8" s="203"/>
+      <c r="J8" s="205"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -22546,7 +22873,7 @@
       <c r="F9" t="s">
         <v>462</v>
       </c>
-      <c r="J9" s="203"/>
+      <c r="J9" s="205"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -22558,7 +22885,7 @@
       <c r="F10" t="s">
         <v>463</v>
       </c>
-      <c r="J10" s="203"/>
+      <c r="J10" s="205"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -22570,7 +22897,7 @@
       <c r="F11" t="s">
         <v>89</v>
       </c>
-      <c r="J11" s="203"/>
+      <c r="J11" s="205"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -22585,7 +22912,7 @@
       <c r="F12" t="s">
         <v>86</v>
       </c>
-      <c r="J12" s="203"/>
+      <c r="J12" s="205"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -22597,7 +22924,7 @@
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="J13" s="203"/>
+      <c r="J13" s="205"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="111" t="s">
@@ -22976,14 +23303,14 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="198" t="s">
+      <c r="A7" s="200" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="198"/>
-      <c r="C7" s="198"/>
-      <c r="D7" s="198"/>
-      <c r="E7" s="198"/>
-      <c r="F7" s="198"/>
+      <c r="B7" s="200"/>
+      <c r="C7" s="200"/>
+      <c r="D7" s="200"/>
+      <c r="E7" s="200"/>
+      <c r="F7" s="200"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
@@ -23072,14 +23399,14 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="198" t="s">
+      <c r="A14" s="200" t="s">
         <v>485</v>
       </c>
-      <c r="B14" s="198"/>
-      <c r="C14" s="198"/>
-      <c r="D14" s="198"/>
-      <c r="E14" s="198"/>
-      <c r="F14" s="198"/>
+      <c r="B14" s="200"/>
+      <c r="C14" s="200"/>
+      <c r="D14" s="200"/>
+      <c r="E14" s="200"/>
+      <c r="F14" s="200"/>
     </row>
     <row r="15" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
@@ -23088,11 +23415,11 @@
       <c r="B15" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="197" t="s">
+      <c r="C15" s="199" t="s">
         <v>470</v>
       </c>
-      <c r="D15" s="197"/>
-      <c r="E15" s="197"/>
+      <c r="D15" s="199"/>
+      <c r="E15" s="199"/>
       <c r="F15" s="11"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -23104,14 +23431,14 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="199" t="s">
+      <c r="A20" s="201" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="199"/>
-      <c r="C20" s="199"/>
-      <c r="D20" s="199"/>
-      <c r="E20" s="199"/>
-      <c r="F20" s="199"/>
+      <c r="B20" s="201"/>
+      <c r="C20" s="201"/>
+      <c r="D20" s="201"/>
+      <c r="E20" s="201"/>
+      <c r="F20" s="201"/>
     </row>
     <row r="21" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -23120,11 +23447,11 @@
       <c r="B21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="197" t="s">
+      <c r="C21" s="199" t="s">
         <v>482</v>
       </c>
-      <c r="D21" s="197"/>
-      <c r="E21" s="197"/>
+      <c r="D21" s="199"/>
+      <c r="E21" s="199"/>
       <c r="F21" s="8" t="s">
         <v>23</v>
       </c>
@@ -23172,14 +23499,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="199" t="s">
+      <c r="A26" s="201" t="s">
         <v>468</v>
       </c>
-      <c r="B26" s="199"/>
-      <c r="C26" s="199"/>
-      <c r="D26" s="199"/>
-      <c r="E26" s="199"/>
-      <c r="F26" s="199"/>
+      <c r="B26" s="201"/>
+      <c r="C26" s="201"/>
+      <c r="D26" s="201"/>
+      <c r="E26" s="201"/>
+      <c r="F26" s="201"/>
     </row>
     <row r="27" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
@@ -23188,11 +23515,11 @@
       <c r="B27" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="197" t="s">
+      <c r="C27" s="199" t="s">
         <v>470</v>
       </c>
-      <c r="D27" s="197"/>
-      <c r="E27" s="197"/>
+      <c r="D27" s="199"/>
+      <c r="E27" s="199"/>
       <c r="F27" s="8"/>
     </row>
   </sheetData>
@@ -23718,7 +24045,7 @@
         <v>45</v>
       </c>
       <c r="B3" s="178" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -23750,32 +24077,33 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="153" t="s">
-        <v>890</v>
-      </c>
-      <c r="B6" s="153" t="s">
+    <row r="6" spans="1:9" s="197" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="206" t="s">
+        <v>919</v>
+      </c>
+      <c r="B6" s="206" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="95" t="s">
+      <c r="C6" s="206" t="s">
         <v>155</v>
       </c>
-      <c r="D6" s="153" t="s">
-        <v>865</v>
-      </c>
-      <c r="E6" s="162" t="s">
-        <v>98</v>
-      </c>
-      <c r="F6" s="98" t="s">
-        <v>806</v>
-      </c>
-      <c r="G6" s="153">
-        <v>1</v>
+      <c r="D6" s="206" t="s">
+        <v>868</v>
+      </c>
+      <c r="E6" s="207" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="206"/>
+      <c r="G6" s="206">
+        <v>112</v>
+      </c>
+      <c r="H6" s="206" t="s">
+        <v>917</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="153" t="s">
-        <v>897</v>
+        <v>889</v>
       </c>
       <c r="B7" s="153" t="s">
         <v>20</v>
@@ -23784,21 +24112,21 @@
         <v>155</v>
       </c>
       <c r="D7" s="153" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="E7" s="162" t="s">
         <v>98</v>
       </c>
       <c r="F7" s="98" t="s">
-        <v>43</v>
+        <v>806</v>
       </c>
       <c r="G7" s="153">
-        <v>20200124</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" s="95" customFormat="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="153" t="s">
-        <v>824</v>
+        <v>896</v>
       </c>
       <c r="B8" s="153" t="s">
         <v>20</v>
@@ -23807,38 +24135,44 @@
         <v>155</v>
       </c>
       <c r="D8" s="153" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="E8" s="162" t="s">
         <v>98</v>
       </c>
-      <c r="F8" s="180" t="s">
+      <c r="F8" s="98" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="153">
+        <v>20200124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="95" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="153" t="s">
+        <v>823</v>
+      </c>
+      <c r="B9" s="153" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="95" t="s">
+        <v>155</v>
+      </c>
+      <c r="D9" s="153" t="s">
+        <v>866</v>
+      </c>
+      <c r="E9" s="162" t="s">
+        <v>98</v>
+      </c>
+      <c r="F9" s="180" t="s">
         <v>809</v>
       </c>
-      <c r="G8" s="153">
+      <c r="G9" s="153">
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="54" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="153" t="s">
-        <v>855</v>
-      </c>
-      <c r="B9" s="153" t="s">
-        <v>772</v>
-      </c>
-      <c r="C9" s="95" t="s">
-        <v>345</v>
-      </c>
-      <c r="D9" s="153" t="s">
-        <v>868</v>
-      </c>
-      <c r="G9" s="153">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" s="54" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="169" t="s">
-        <v>909</v>
+    <row r="10" spans="1:9" s="54" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="153" t="s">
+        <v>854</v>
       </c>
       <c r="B10" s="153" t="s">
         <v>772</v>
@@ -23847,10 +24181,10 @@
         <v>345</v>
       </c>
       <c r="D10" s="153" t="s">
-        <v>910</v>
-      </c>
-      <c r="G10" s="169">
-        <v>45</v>
+        <v>867</v>
+      </c>
+      <c r="G10" s="153">
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="54" customFormat="1" x14ac:dyDescent="0.3">
@@ -23985,9 +24319,9 @@
   <hyperlinks>
     <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{8402A49E-D3E0-4037-920F-B02CE895AE24}"/>
     <hyperlink ref="F12" location="'Process Metadata'!A25" display="Import_Batch_Process_Task" xr:uid="{711F08C5-5B7C-4423-B885-52AEFB576C7B}"/>
-    <hyperlink ref="F6" location="Employee_Dimension!A1" display="Employee" xr:uid="{6286886C-F575-44C3-BBC7-C293215BC447}"/>
-    <hyperlink ref="F8" location="Project!A1" display="Project" xr:uid="{62B6770D-6301-4F22-9A86-2C8046C4CD99}"/>
-    <hyperlink ref="F7" location="Date!A1" display="Date" xr:uid="{2499E08C-7C05-4603-A891-7093F76F9D53}"/>
+    <hyperlink ref="F7" location="Employee_Dimension!A1" display="Employee" xr:uid="{6286886C-F575-44C3-BBC7-C293215BC447}"/>
+    <hyperlink ref="F9" location="Project!A1" display="Project" xr:uid="{62B6770D-6301-4F22-9A86-2C8046C4CD99}"/>
+    <hyperlink ref="F8" location="Date!A1" display="Date" xr:uid="{2499E08C-7C05-4603-A891-7093F76F9D53}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23998,7 +24332,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultColWidth="21.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50.109375" style="145" customWidth="1"/>
@@ -24022,7 +24356,7 @@
         <v>127</v>
       </c>
       <c r="B2" s="95" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -24030,7 +24364,7 @@
         <v>45</v>
       </c>
       <c r="B3" s="145" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -24062,35 +24396,33 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="145" t="s">
-        <v>914</v>
-      </c>
-      <c r="B6" s="146" t="s">
+    <row r="6" spans="1:8" s="197" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="206" t="s">
+        <v>918</v>
+      </c>
+      <c r="B6" s="206" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="145" t="s">
+      <c r="C6" s="206" t="s">
         <v>155</v>
       </c>
-      <c r="D6" s="149" t="s">
-        <v>822</v>
-      </c>
-      <c r="E6" s="95" t="s">
-        <v>98</v>
-      </c>
-      <c r="F6" s="98" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" s="145">
-        <v>20190125</v>
-      </c>
-      <c r="H6" s="145" t="s">
-        <v>344</v>
+      <c r="D6" s="206" t="s">
+        <v>868</v>
+      </c>
+      <c r="E6" s="207" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="206"/>
+      <c r="G6" s="206">
+        <v>341</v>
+      </c>
+      <c r="H6" s="206" t="s">
+        <v>920</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="145" t="s">
-        <v>906</v>
+        <v>913</v>
       </c>
       <c r="B7" s="146" t="s">
         <v>20</v>
@@ -24098,8 +24430,8 @@
       <c r="C7" s="145" t="s">
         <v>155</v>
       </c>
-      <c r="D7" s="150" t="s">
-        <v>823</v>
+      <c r="D7" s="149" t="s">
+        <v>821</v>
       </c>
       <c r="E7" s="95" t="s">
         <v>98</v>
@@ -24110,10 +24442,13 @@
       <c r="G7" s="145">
         <v>20190125</v>
       </c>
+      <c r="H7" s="145" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="145" t="s">
-        <v>824</v>
+        <v>914</v>
       </c>
       <c r="B8" s="146" t="s">
         <v>20</v>
@@ -24122,21 +24457,21 @@
         <v>155</v>
       </c>
       <c r="D8" s="150" t="s">
-        <v>876</v>
+        <v>822</v>
       </c>
       <c r="E8" s="95" t="s">
         <v>98</v>
       </c>
-      <c r="F8" s="151" t="s">
-        <v>875</v>
-      </c>
-      <c r="G8" s="145" t="s">
-        <v>742</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" s="95" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="152" t="s">
-        <v>896</v>
+      <c r="F8" s="98" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="145">
+        <v>20190125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="145" t="s">
+        <v>823</v>
       </c>
       <c r="B9" s="146" t="s">
         <v>20</v>
@@ -24144,22 +24479,22 @@
       <c r="C9" s="145" t="s">
         <v>155</v>
       </c>
-      <c r="D9" s="152" t="s">
-        <v>839</v>
+      <c r="D9" s="150" t="s">
+        <v>875</v>
       </c>
       <c r="E9" s="95" t="s">
         <v>98</v>
       </c>
-      <c r="F9" s="98" t="s">
+      <c r="F9" s="151" t="s">
         <v>874</v>
       </c>
-      <c r="G9" s="152" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G9" s="145" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="95" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="152" t="s">
-        <v>838</v>
+        <v>895</v>
       </c>
       <c r="B10" s="146" t="s">
         <v>20</v>
@@ -24168,62 +24503,65 @@
         <v>155</v>
       </c>
       <c r="D10" s="152" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="E10" s="95" t="s">
         <v>98</v>
       </c>
       <c r="F10" s="98" t="s">
-        <v>821</v>
-      </c>
-      <c r="G10" s="75" t="s">
-        <v>841</v>
-      </c>
-      <c r="H10" s="152"/>
+        <v>873</v>
+      </c>
+      <c r="G10" s="152" t="s">
+        <v>634</v>
+      </c>
     </row>
     <row r="11" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="54" t="s">
-        <v>826</v>
-      </c>
-      <c r="B11" s="153" t="s">
-        <v>772</v>
-      </c>
-      <c r="C11" s="54" t="s">
-        <v>345</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>827</v>
-      </c>
-      <c r="G11" s="155">
-        <v>12530</v>
-      </c>
-      <c r="H11" s="54" t="s">
-        <v>831</v>
-      </c>
+      <c r="A11" s="152" t="s">
+        <v>837</v>
+      </c>
+      <c r="B11" s="146" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="145" t="s">
+        <v>155</v>
+      </c>
+      <c r="D11" s="152" t="s">
+        <v>839</v>
+      </c>
+      <c r="E11" s="95" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" s="98" t="s">
+        <v>820</v>
+      </c>
+      <c r="G11" s="75" t="s">
+        <v>840</v>
+      </c>
+      <c r="H11" s="152"/>
     </row>
     <row r="12" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="54" t="s">
-        <v>828</v>
-      </c>
-      <c r="B12" s="153" t="s">
-        <v>772</v>
-      </c>
-      <c r="C12" s="54" t="s">
-        <v>345</v>
-      </c>
-      <c r="D12" s="154" t="s">
-        <v>829</v>
-      </c>
-      <c r="G12" s="155">
-        <v>5360</v>
-      </c>
-      <c r="H12" s="54" t="s">
-        <v>830</v>
-      </c>
+      <c r="A12" s="152" t="s">
+        <v>755</v>
+      </c>
+      <c r="B12" s="198" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="197" t="s">
+        <v>155</v>
+      </c>
+      <c r="D12" s="152" t="s">
+        <v>916</v>
+      </c>
+      <c r="E12" s="95"/>
+      <c r="F12" s="98"/>
+      <c r="G12" s="75">
+        <v>5127095</v>
+      </c>
+      <c r="H12" s="152"/>
     </row>
     <row r="13" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="54" t="s">
-        <v>832</v>
+        <v>825</v>
       </c>
       <c r="B13" s="153" t="s">
         <v>772</v>
@@ -24232,18 +24570,18 @@
         <v>345</v>
       </c>
       <c r="D13" s="154" t="s">
-        <v>833</v>
+        <v>826</v>
       </c>
       <c r="G13" s="155">
-        <v>1340</v>
+        <v>12530</v>
       </c>
       <c r="H13" s="54" t="s">
-        <v>834</v>
+        <v>830</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="54" t="s">
-        <v>835</v>
+        <v>827</v>
       </c>
       <c r="B14" s="153" t="s">
         <v>772</v>
@@ -24252,84 +24590,124 @@
         <v>345</v>
       </c>
       <c r="D14" s="154" t="s">
+        <v>828</v>
+      </c>
+      <c r="G14" s="155">
+        <v>5360</v>
+      </c>
+      <c r="H14" s="54" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="54" t="s">
+        <v>831</v>
+      </c>
+      <c r="B15" s="153" t="s">
+        <v>772</v>
+      </c>
+      <c r="C15" s="54" t="s">
+        <v>345</v>
+      </c>
+      <c r="D15" s="154" t="s">
+        <v>832</v>
+      </c>
+      <c r="G15" s="155">
+        <v>1340</v>
+      </c>
+      <c r="H15" s="54" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="54" t="s">
+        <v>834</v>
+      </c>
+      <c r="B16" s="153" t="s">
+        <v>772</v>
+      </c>
+      <c r="C16" s="54" t="s">
+        <v>345</v>
+      </c>
+      <c r="D16" s="154" t="s">
+        <v>835</v>
+      </c>
+      <c r="G16" s="54">
+        <f>SUM(G13:G15)</f>
+        <v>19230</v>
+      </c>
+      <c r="H16" s="54" t="s">
         <v>836</v>
       </c>
-      <c r="G14" s="54">
-        <f>SUM(G11:G13)</f>
-        <v>19230</v>
-      </c>
-      <c r="H14" s="54" t="s">
-        <v>837</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" s="62" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="62" t="s">
+    </row>
+    <row r="17" spans="1:8" s="62" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="62" t="s">
         <v>148</v>
       </c>
-      <c r="B15" s="62" t="s">
+      <c r="B17" s="62" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="62" t="s">
+      <c r="C17" s="62" t="s">
         <v>155</v>
       </c>
-      <c r="D15" s="156" t="s">
+      <c r="D17" s="156" t="s">
         <v>572</v>
       </c>
-      <c r="G15" s="62" t="s">
+      <c r="G17" s="62" t="s">
         <v>150</v>
       </c>
-      <c r="H15" s="62" t="s">
+      <c r="H17" s="62" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="62" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="62" t="s">
+    <row r="18" spans="1:8" s="62" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="62" t="s">
+      <c r="B18" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="62" t="s">
+      <c r="C18" s="62" t="s">
         <v>155</v>
       </c>
-      <c r="D16" s="156" t="s">
+      <c r="D18" s="156" t="s">
         <v>147</v>
       </c>
-      <c r="F16" s="98" t="s">
+      <c r="F18" s="98" t="s">
         <v>30</v>
       </c>
-      <c r="G16" s="62">
+      <c r="G18" s="62">
         <v>1</v>
       </c>
-      <c r="H16" s="62" t="s">
+      <c r="H18" s="62" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="17" spans="1:6" s="62" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="156"/>
-      <c r="F17" s="98"/>
-    </row>
-    <row r="18" spans="1:6" s="62" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D18" s="156"/>
-      <c r="F18" s="98"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="95" t="s">
+    <row r="19" spans="1:8" s="62" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="156"/>
+      <c r="F19" s="98"/>
+    </row>
+    <row r="20" spans="1:8" s="62" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D20" s="156"/>
+      <c r="F20" s="98"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="95" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="20" spans="1:6" s="157" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D20" s="158"/>
+    <row r="22" spans="1:8" s="157" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D22" s="158"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="Index!A1" display="Index" xr:uid="{FA15B678-0793-4DFD-9F5C-81B4068420A4}"/>
-    <hyperlink ref="F6" location="Date!A1" display="Date" xr:uid="{E762CFFA-CCDD-49D8-A7EA-6CD06C0933E8}"/>
-    <hyperlink ref="F16" location="'Process Metadata'!A25" display="Import_Batch_Process_Task" xr:uid="{B5D440B5-0249-4B6C-84A6-F36698C87CFD}"/>
-    <hyperlink ref="F7" location="Date!A1" display="Date" xr:uid="{71F31C74-0A03-4B30-9D99-0E3629062544}"/>
-    <hyperlink ref="F8" location="Project!A1" display="Projects" xr:uid="{E1BB4138-E373-478E-A2A8-1CD348A831E4}"/>
-    <hyperlink ref="F9" location="Customer!A1" display="Customers" xr:uid="{56D25DE4-CC5C-4C9F-98B0-894AF3FCC88D}"/>
-    <hyperlink ref="F10" location="Project_Status!A1" display="Project_Status" xr:uid="{A55BCE96-86F0-434F-A6FF-8004377BA56E}"/>
+    <hyperlink ref="F7" location="Date!A1" display="Date" xr:uid="{E762CFFA-CCDD-49D8-A7EA-6CD06C0933E8}"/>
+    <hyperlink ref="F18" location="'Process Metadata'!A25" display="Import_Batch_Process_Task" xr:uid="{B5D440B5-0249-4B6C-84A6-F36698C87CFD}"/>
+    <hyperlink ref="F8" location="Date!A1" display="Date" xr:uid="{71F31C74-0A03-4B30-9D99-0E3629062544}"/>
+    <hyperlink ref="F9" location="Project!A1" display="Projects" xr:uid="{E1BB4138-E373-478E-A2A8-1CD348A831E4}"/>
+    <hyperlink ref="F10" location="Customer!A1" display="Customers" xr:uid="{56D25DE4-CC5C-4C9F-98B0-894AF3FCC88D}"/>
+    <hyperlink ref="F11" location="Project_Status!A1" display="Project_Status" xr:uid="{A55BCE96-86F0-434F-A6FF-8004377BA56E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -24512,7 +24890,7 @@
     </row>
     <row r="9" spans="1:11" s="145" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="153" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B9" s="153" t="s">
         <v>20</v>
@@ -24521,7 +24899,7 @@
         <v>345</v>
       </c>
       <c r="D9" s="153" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="E9" s="162"/>
       <c r="F9" s="98"/>
@@ -24609,13 +24987,13 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="75" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B13" s="47" t="s">
         <v>57</v>
       </c>
       <c r="D13" s="47" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G13" s="75" t="s">
         <v>56</v>
@@ -24685,10 +25063,10 @@
         <v>76</v>
       </c>
       <c r="H2" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="I2" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -64948,7 +65326,7 @@
     </row>
     <row r="1091" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1091">
-        <f t="shared" ref="A1091:A1154" si="136">YEAR(B1091)*10000+MONTH(B1091)*100+DAY(B1091)</f>
+        <f t="shared" ref="A1091:A1100" si="136">YEAR(B1091)*10000+MONTH(B1091)*100+DAY(B1091)</f>
         <v>20221223</v>
       </c>
       <c r="B1091" s="193">
@@ -64992,7 +65370,7 @@
         <v>44919</v>
       </c>
       <c r="C1092" s="196" t="str">
-        <f t="shared" ref="C1092:C1155" si="143">TEXT(B1092,"dd MMMM YYYY")</f>
+        <f t="shared" ref="C1092:C1099" si="143">TEXT(B1092,"dd MMMM YYYY")</f>
         <v>24 December 2022</v>
       </c>
       <c r="D1092">

</xml_diff>

<commit_message>
Modified grain of Employee_TimeSheet_Fact
</commit_message>
<xml_diff>
--- a/DW2022/Documentation/Design document.xlsx
+++ b/DW2022/Documentation/Design document.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Llewellyn\Desktop\Honours Resources\DATA WAREHOUSING\DW2022_Repo\DW2022\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDDF43A-F7EA-471A-BA2E-C79DAB4E9F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575CE688-A57D-4CA7-A10F-B11809BA6B45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" firstSheet="27" activeTab="29" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" tabRatio="887" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -2857,9 +2857,6 @@
     <t>ID of the department the customer belongs to</t>
   </si>
   <si>
-    <t>One row for each employee that worked during that week per project</t>
-  </si>
-  <si>
     <t>X
 Report_Date_Key
 Project_Request_Date_Key</t>
@@ -2871,9 +2868,6 @@
     <t>Project_Request_Date_Key</t>
   </si>
   <si>
-    <t>One row for each employee timesheet event (when a timesheet is submitted) per project</t>
-  </si>
-  <si>
     <t>Service billing number of a project</t>
   </si>
   <si>
@@ -3007,6 +3001,12 @@
   </si>
   <si>
     <t>Postal Code of customer residence</t>
+  </si>
+  <si>
+    <t>One row per employee per week that worked on a project and syubmitted a time sheet</t>
+  </si>
+  <si>
+    <t>*Unknown Customer Group Name</t>
   </si>
 </sst>
 </file>
@@ -3953,6 +3953,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3973,21 +3988,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -14272,16 +14272,16 @@
       <c r="A3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="202" t="s">
+      <c r="B3" s="207" t="s">
         <v>235</v>
       </c>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="202"/>
-      <c r="G3" s="202"/>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
+      <c r="C3" s="207"/>
+      <c r="D3" s="207"/>
+      <c r="E3" s="207"/>
+      <c r="F3" s="207"/>
+      <c r="G3" s="207"/>
+      <c r="H3" s="207"/>
+      <c r="I3" s="207"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -14904,16 +14904,16 @@
       <c r="A3" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="202" t="s">
+      <c r="B3" s="207" t="s">
         <v>876</v>
       </c>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="202"/>
-      <c r="G3" s="202"/>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
+      <c r="C3" s="207"/>
+      <c r="D3" s="207"/>
+      <c r="E3" s="207"/>
+      <c r="F3" s="207"/>
+      <c r="G3" s="207"/>
+      <c r="H3" s="207"/>
+      <c r="I3" s="207"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -15061,7 +15061,7 @@
     </row>
     <row r="11" spans="1:9" s="165" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="165" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="B11" s="148" t="s">
         <v>36</v>
@@ -15280,16 +15280,16 @@
       <c r="A3" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="202" t="s">
+      <c r="B3" s="207" t="s">
         <v>908</v>
       </c>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="202"/>
-      <c r="G3" s="202"/>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
+      <c r="C3" s="207"/>
+      <c r="D3" s="207"/>
+      <c r="E3" s="207"/>
+      <c r="F3" s="207"/>
+      <c r="G3" s="207"/>
+      <c r="H3" s="207"/>
+      <c r="I3" s="207"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -15377,8 +15377,8 @@
       <c r="H8" s="178"/>
     </row>
     <row r="9" spans="1:9" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="208" t="s">
-        <v>929</v>
+      <c r="A9" s="201" t="s">
+        <v>927</v>
       </c>
       <c r="C9" s="170"/>
       <c r="F9" s="34"/>
@@ -15467,16 +15467,16 @@
       <c r="A3" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="202" t="s">
+      <c r="B3" s="207" t="s">
         <v>870</v>
       </c>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="202"/>
-      <c r="G3" s="202"/>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
+      <c r="C3" s="207"/>
+      <c r="D3" s="207"/>
+      <c r="E3" s="207"/>
+      <c r="F3" s="207"/>
+      <c r="G3" s="207"/>
+      <c r="H3" s="207"/>
+      <c r="I3" s="207"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -15919,16 +15919,16 @@
       <c r="A3" s="138" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="203" t="s">
+      <c r="B3" s="208" t="s">
         <v>891</v>
       </c>
-      <c r="C3" s="203"/>
-      <c r="D3" s="203"/>
-      <c r="E3" s="203"/>
-      <c r="F3" s="203"/>
-      <c r="G3" s="203"/>
-      <c r="H3" s="203"/>
-      <c r="I3" s="203"/>
+      <c r="C3" s="208"/>
+      <c r="D3" s="208"/>
+      <c r="E3" s="208"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="208"/>
+      <c r="H3" s="208"/>
+      <c r="I3" s="208"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -16023,7 +16023,7 @@
         <v>852</v>
       </c>
       <c r="G8" s="75" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H8" s="75" t="s">
         <v>640</v>
@@ -16032,29 +16032,29 @@
     </row>
     <row r="9" spans="1:9" s="140" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="165" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="B9" s="198" t="s">
         <v>659</v>
       </c>
       <c r="C9" s="166" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
       <c r="D9" s="165"/>
       <c r="E9" s="48">
         <v>1</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="G9" s="75" t="s">
+        <v>922</v>
+      </c>
+      <c r="H9" s="75" t="s">
         <v>924</v>
       </c>
-      <c r="H9" s="75" t="s">
+      <c r="I9" s="165" t="s">
         <v>926</v>
-      </c>
-      <c r="I9" s="165" t="s">
-        <v>928</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="140" customFormat="1" x14ac:dyDescent="0.3">
@@ -16532,16 +16532,16 @@
       <c r="A3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="202" t="s">
+      <c r="B3" s="207" t="s">
         <v>409</v>
       </c>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="202"/>
-      <c r="G3" s="202"/>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
+      <c r="C3" s="207"/>
+      <c r="D3" s="207"/>
+      <c r="E3" s="207"/>
+      <c r="F3" s="207"/>
+      <c r="G3" s="207"/>
+      <c r="H3" s="207"/>
+      <c r="I3" s="207"/>
     </row>
     <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -17080,7 +17080,7 @@
         <v>209</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="D3" t="s">
         <v>345</v>
@@ -17106,7 +17106,7 @@
         <v>210</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="E4" t="s">
         <v>155</v>
@@ -17129,7 +17129,7 @@
         <v>210</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="E5" t="s">
         <v>155</v>
@@ -17236,14 +17236,14 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="210" t="s">
+      <c r="A3" s="203" t="s">
         <v>713</v>
       </c>
       <c r="B3" s="75" t="s">
         <v>20</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="D3" s="75" t="s">
         <v>345</v>
@@ -17262,14 +17262,14 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="210" t="s">
+      <c r="A4" s="203" t="s">
         <v>714</v>
       </c>
       <c r="B4" s="75" t="s">
         <v>20</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="E4" s="75" t="s">
         <v>155</v>
@@ -17285,14 +17285,14 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="210" t="s">
+      <c r="A5" s="203" t="s">
         <v>715</v>
       </c>
       <c r="B5" s="75" t="s">
         <v>57</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="D5" s="75" t="s">
         <v>345</v>
@@ -17311,14 +17311,14 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="210" t="s">
+      <c r="A6" s="203" t="s">
         <v>716</v>
       </c>
       <c r="B6" s="75" t="s">
         <v>717</v>
       </c>
       <c r="C6" s="47" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="D6" s="75" t="s">
         <v>345</v>
@@ -17337,14 +17337,14 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="210" t="s">
+      <c r="A7" s="203" t="s">
         <v>720</v>
       </c>
       <c r="B7" s="75" t="s">
         <v>209</v>
       </c>
       <c r="C7" s="47" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="D7" s="75" t="s">
         <v>345</v>
@@ -17363,14 +17363,14 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="210" t="s">
+      <c r="A8" s="203" t="s">
         <v>723</v>
       </c>
       <c r="B8" s="75" t="s">
         <v>724</v>
       </c>
       <c r="C8" s="47" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E8" s="75" t="s">
         <v>345</v>
@@ -17457,7 +17457,7 @@
         <v>209</v>
       </c>
       <c r="C4" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="D4" t="s">
         <v>740</v>
@@ -17506,7 +17506,7 @@
         <v>209</v>
       </c>
       <c r="C6" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="E6" t="s">
         <v>741</v>
@@ -17529,7 +17529,7 @@
         <v>210</v>
       </c>
       <c r="C7" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="E7" t="s">
         <v>740</v>
@@ -17552,7 +17552,7 @@
         <v>749</v>
       </c>
       <c r="C8" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="E8" t="s">
         <v>741</v>
@@ -17575,7 +17575,7 @@
         <v>210</v>
       </c>
       <c r="C9" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="E9" t="s">
         <v>740</v>
@@ -17592,7 +17592,7 @@
         <v>752</v>
       </c>
       <c r="C10" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="E10" t="s">
         <v>740</v>
@@ -17615,7 +17615,7 @@
         <v>752</v>
       </c>
       <c r="C11" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="E11" t="s">
         <v>740</v>
@@ -17638,7 +17638,7 @@
         <v>752</v>
       </c>
       <c r="C12" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="E12" t="s">
         <v>740</v>
@@ -17661,7 +17661,7 @@
         <v>209</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="E13" t="s">
         <v>740</v>
@@ -18008,7 +18008,7 @@
         <v>677</v>
       </c>
       <c r="C4" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="D4" t="s">
         <v>345</v>
@@ -18034,7 +18034,7 @@
         <v>647</v>
       </c>
       <c r="C5" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="E5" t="s">
         <v>155</v>
@@ -18057,7 +18057,7 @@
         <v>677</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="E6" t="s">
         <v>155</v>
@@ -18141,7 +18141,7 @@
         <v>645</v>
       </c>
       <c r="C4" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="D4" t="s">
         <v>345</v>
@@ -18167,7 +18167,7 @@
         <v>676</v>
       </c>
       <c r="C5" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="E5" t="s">
         <v>155</v>
@@ -18190,7 +18190,7 @@
         <v>677</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="E6" t="s">
         <v>155</v>
@@ -18274,7 +18274,7 @@
         <v>645</v>
       </c>
       <c r="C4" s="115" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="D4" s="115" t="s">
         <v>345</v>
@@ -18300,7 +18300,7 @@
         <v>645</v>
       </c>
       <c r="C5" s="115" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="D5" s="115"/>
       <c r="E5" s="115" t="s">
@@ -18324,7 +18324,7 @@
         <v>646</v>
       </c>
       <c r="C6" s="115" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="D6" s="115"/>
       <c r="E6" s="115" t="s">
@@ -18348,7 +18348,7 @@
         <v>647</v>
       </c>
       <c r="C7" s="115" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="D7" s="115"/>
       <c r="E7" s="115" t="s">
@@ -18412,7 +18412,7 @@
         <v>647</v>
       </c>
       <c r="C10" s="115" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="D10" s="115"/>
       <c r="E10" s="115" t="s">
@@ -18433,7 +18433,7 @@
         <v>648</v>
       </c>
       <c r="C11" s="115" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="D11" s="115"/>
       <c r="E11" s="115" t="s">
@@ -18984,14 +18984,14 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="200" t="s">
+      <c r="A8" s="205" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="200"/>
-      <c r="C8" s="200"/>
-      <c r="D8" s="200"/>
-      <c r="E8" s="200"/>
-      <c r="F8" s="200"/>
+      <c r="B8" s="205"/>
+      <c r="C8" s="205"/>
+      <c r="D8" s="205"/>
+      <c r="E8" s="205"/>
+      <c r="F8" s="205"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
@@ -19151,14 +19151,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="200" t="s">
+      <c r="A18" s="205" t="s">
         <v>485</v>
       </c>
-      <c r="B18" s="200"/>
-      <c r="C18" s="200"/>
-      <c r="D18" s="200"/>
-      <c r="E18" s="200"/>
-      <c r="F18" s="200"/>
+      <c r="B18" s="205"/>
+      <c r="C18" s="205"/>
+      <c r="D18" s="205"/>
+      <c r="E18" s="205"/>
+      <c r="F18" s="205"/>
     </row>
     <row r="19" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
@@ -19167,11 +19167,11 @@
       <c r="B19" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="199" t="s">
+      <c r="C19" s="204" t="s">
         <v>470</v>
       </c>
-      <c r="D19" s="199"/>
-      <c r="E19" s="199"/>
+      <c r="D19" s="204"/>
+      <c r="E19" s="204"/>
       <c r="F19" s="11"/>
     </row>
     <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -19197,14 +19197,14 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="201" t="s">
+      <c r="A23" s="206" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="201"/>
-      <c r="C23" s="201"/>
-      <c r="D23" s="201"/>
-      <c r="E23" s="201"/>
-      <c r="F23" s="201"/>
+      <c r="B23" s="206"/>
+      <c r="C23" s="206"/>
+      <c r="D23" s="206"/>
+      <c r="E23" s="206"/>
+      <c r="F23" s="206"/>
     </row>
     <row r="24" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
@@ -19213,11 +19213,11 @@
       <c r="B24" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="199" t="s">
+      <c r="C24" s="204" t="s">
         <v>482</v>
       </c>
-      <c r="D24" s="199"/>
-      <c r="E24" s="199"/>
+      <c r="D24" s="204"/>
+      <c r="E24" s="204"/>
       <c r="F24" s="8" t="s">
         <v>23</v>
       </c>
@@ -19265,14 +19265,14 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="201" t="s">
+      <c r="A29" s="206" t="s">
         <v>468</v>
       </c>
-      <c r="B29" s="201"/>
-      <c r="C29" s="201"/>
-      <c r="D29" s="201"/>
-      <c r="E29" s="201"/>
-      <c r="F29" s="201"/>
+      <c r="B29" s="206"/>
+      <c r="C29" s="206"/>
+      <c r="D29" s="206"/>
+      <c r="E29" s="206"/>
+      <c r="F29" s="206"/>
     </row>
     <row r="30" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
@@ -19281,11 +19281,11 @@
       <c r="B30" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="199" t="s">
+      <c r="C30" s="204" t="s">
         <v>470</v>
       </c>
-      <c r="D30" s="199"/>
-      <c r="E30" s="199"/>
+      <c r="D30" s="204"/>
+      <c r="E30" s="204"/>
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -19400,7 +19400,7 @@
         <v>155</v>
       </c>
       <c r="D4" s="115" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="E4" s="116" t="s">
         <v>661</v>
@@ -19426,7 +19426,7 @@
         <v>155</v>
       </c>
       <c r="D5" s="115" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="E5" t="s">
         <v>134</v>
@@ -19449,7 +19449,7 @@
         <v>155</v>
       </c>
       <c r="D6" s="115" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="E6" t="s">
         <v>662</v>
@@ -19472,7 +19472,7 @@
         <v>155</v>
       </c>
       <c r="D7" s="115" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="E7" t="s">
         <v>663</v>
@@ -19544,7 +19544,7 @@
         <v>155</v>
       </c>
       <c r="D10" s="115" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="E10" t="s">
         <v>666</v>
@@ -19567,7 +19567,7 @@
         <v>155</v>
       </c>
       <c r="D11" s="115" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="E11" t="s">
         <v>667</v>
@@ -19589,7 +19589,7 @@
       <c r="C12" t="s">
         <v>155</v>
       </c>
-      <c r="D12" s="209" t="s">
+      <c r="D12" s="202" t="s">
         <v>257</v>
       </c>
       <c r="F12" s="75">
@@ -19680,7 +19680,7 @@
         <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="E4" t="s">
         <v>661</v>
@@ -19706,7 +19706,7 @@
         <v>155</v>
       </c>
       <c r="D5" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="E5" t="s">
         <v>687</v>
@@ -19729,7 +19729,7 @@
         <v>155</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="E6" t="s">
         <v>134</v>
@@ -19751,7 +19751,7 @@
       <c r="C7" t="s">
         <v>155</v>
       </c>
-      <c r="D7" s="209" t="s">
+      <c r="D7" s="202" t="s">
         <v>257</v>
       </c>
       <c r="F7" s="75">
@@ -19838,7 +19838,7 @@
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="E4" t="s">
         <v>661</v>
@@ -19862,7 +19862,7 @@
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="E5" t="s">
         <v>733</v>
@@ -19884,7 +19884,7 @@
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="E6" t="s">
         <v>734</v>
@@ -19909,7 +19909,7 @@
       <c r="C7" s="75" t="s">
         <v>731</v>
       </c>
-      <c r="D7" s="209" t="s">
+      <c r="D7" s="202" t="s">
         <v>257</v>
       </c>
       <c r="E7" s="44"/>
@@ -20032,7 +20032,7 @@
         <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="E4" t="s">
         <v>661</v>
@@ -20072,7 +20072,7 @@
         <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="E6" t="s">
         <v>134</v>
@@ -20092,7 +20092,7 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="E7" t="s">
         <v>765</v>
@@ -20112,7 +20112,7 @@
         <v>767</v>
       </c>
       <c r="D8" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="E8" t="s">
         <v>768</v>
@@ -20132,7 +20132,7 @@
         <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="E9" t="s">
         <v>770</v>
@@ -20146,7 +20146,7 @@
         <v>772</v>
       </c>
       <c r="D10" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="E10" t="s">
         <v>325</v>
@@ -20166,7 +20166,7 @@
         <v>772</v>
       </c>
       <c r="D11" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="E11" t="s">
         <v>325</v>
@@ -20186,7 +20186,7 @@
         <v>772</v>
       </c>
       <c r="D12" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="E12" t="s">
         <v>325</v>
@@ -20206,7 +20206,7 @@
         <v>61</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="E13" t="s">
         <v>776</v>
@@ -20225,7 +20225,7 @@
       <c r="B14" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="209" t="s">
+      <c r="D14" s="202" t="s">
         <v>257</v>
       </c>
       <c r="F14" s="75">
@@ -20308,7 +20308,7 @@
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="E4" t="s">
         <v>661</v>
@@ -20332,7 +20332,7 @@
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="E5" s="75">
         <v>0</v>
@@ -20354,7 +20354,7 @@
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="E6" s="118">
         <v>43872</v>
@@ -20375,7 +20375,7 @@
       </c>
       <c r="C7" s="75"/>
       <c r="D7" s="2" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>728</v>
@@ -20395,7 +20395,7 @@
         <v>61</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="E8" t="s">
         <v>729</v>
@@ -20415,7 +20415,7 @@
         <v>724</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E9" s="75" t="s">
         <v>325</v>
@@ -20437,7 +20437,7 @@
       <c r="C10" s="75" t="s">
         <v>731</v>
       </c>
-      <c r="D10" s="209" t="s">
+      <c r="D10" s="202" t="s">
         <v>257</v>
       </c>
       <c r="E10" s="2"/>
@@ -20598,7 +20598,7 @@
       </c>
       <c r="L5" s="20"/>
     </row>
-    <row r="6" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
         <v>812</v>
       </c>
@@ -20609,7 +20609,7 @@
         <v>124</v>
       </c>
       <c r="E6" s="131" t="s">
-        <v>911</v>
+        <v>958</v>
       </c>
       <c r="F6" s="20" t="s">
         <v>817</v>
@@ -20637,7 +20637,7 @@
         <v>816</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="J7" s="20" t="s">
         <v>44</v>
@@ -20694,7 +20694,7 @@
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" customWidth="1"/>
+    <col min="4" max="4" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.44140625" customWidth="1"/>
     <col min="6" max="6" width="19.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29.109375" bestFit="1" customWidth="1"/>
@@ -20751,7 +20751,7 @@
         <v>661</v>
       </c>
       <c r="E4" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="F4" t="s">
         <v>679</v>
@@ -20771,10 +20771,10 @@
         <v>36</v>
       </c>
       <c r="D5" s="116" t="s">
-        <v>661</v>
+        <v>959</v>
       </c>
       <c r="E5" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="F5" t="s">
         <v>691</v>
@@ -20791,10 +20791,10 @@
         <v>66</v>
       </c>
       <c r="D6" s="116" t="s">
-        <v>661</v>
+        <v>134</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="F6" t="s">
         <v>692</v>
@@ -21466,14 +21466,14 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="200" t="s">
+      <c r="A8" s="205" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="200"/>
-      <c r="C8" s="200"/>
-      <c r="D8" s="200"/>
-      <c r="E8" s="200"/>
-      <c r="F8" s="200"/>
+      <c r="B8" s="205"/>
+      <c r="C8" s="205"/>
+      <c r="D8" s="205"/>
+      <c r="E8" s="205"/>
+      <c r="F8" s="205"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
@@ -21556,14 +21556,14 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="200" t="s">
+      <c r="A14" s="205" t="s">
         <v>485</v>
       </c>
-      <c r="B14" s="200"/>
-      <c r="C14" s="200"/>
-      <c r="D14" s="200"/>
-      <c r="E14" s="200"/>
-      <c r="F14" s="200"/>
+      <c r="B14" s="205"/>
+      <c r="C14" s="205"/>
+      <c r="D14" s="205"/>
+      <c r="E14" s="205"/>
+      <c r="F14" s="205"/>
     </row>
     <row r="15" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
@@ -21572,11 +21572,11 @@
       <c r="B15" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="199" t="s">
+      <c r="C15" s="204" t="s">
         <v>470</v>
       </c>
-      <c r="D15" s="199"/>
-      <c r="E15" s="199"/>
+      <c r="D15" s="204"/>
+      <c r="E15" s="204"/>
       <c r="F15" s="11"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -21591,14 +21591,14 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="201" t="s">
+      <c r="A20" s="206" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="201"/>
-      <c r="C20" s="201"/>
-      <c r="D20" s="201"/>
-      <c r="E20" s="201"/>
-      <c r="F20" s="201"/>
+      <c r="B20" s="206"/>
+      <c r="C20" s="206"/>
+      <c r="D20" s="206"/>
+      <c r="E20" s="206"/>
+      <c r="F20" s="206"/>
     </row>
     <row r="21" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -21607,11 +21607,11 @@
       <c r="B21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="199" t="s">
+      <c r="C21" s="204" t="s">
         <v>482</v>
       </c>
-      <c r="D21" s="199"/>
-      <c r="E21" s="199"/>
+      <c r="D21" s="204"/>
+      <c r="E21" s="204"/>
       <c r="F21" s="8" t="s">
         <v>23</v>
       </c>
@@ -21659,14 +21659,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="201" t="s">
+      <c r="A26" s="206" t="s">
         <v>468</v>
       </c>
-      <c r="B26" s="201"/>
-      <c r="C26" s="201"/>
-      <c r="D26" s="201"/>
-      <c r="E26" s="201"/>
-      <c r="F26" s="201"/>
+      <c r="B26" s="206"/>
+      <c r="C26" s="206"/>
+      <c r="D26" s="206"/>
+      <c r="E26" s="206"/>
+      <c r="F26" s="206"/>
     </row>
     <row r="27" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
@@ -21675,11 +21675,11 @@
       <c r="B27" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="199" t="s">
+      <c r="C27" s="204" t="s">
         <v>470</v>
       </c>
-      <c r="D27" s="199"/>
-      <c r="E27" s="199"/>
+      <c r="D27" s="204"/>
+      <c r="E27" s="204"/>
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -21797,10 +21797,10 @@
       <c r="F5" s="43"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="204" t="s">
+      <c r="A10" s="209" t="s">
         <v>497</v>
       </c>
-      <c r="B10" s="204"/>
+      <c r="B10" s="209"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
@@ -22832,7 +22832,7 @@
       <c r="F6" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="205" t="s">
+      <c r="J6" s="210" t="s">
         <v>467</v>
       </c>
     </row>
@@ -22849,7 +22849,7 @@
       <c r="F7" t="s">
         <v>95</v>
       </c>
-      <c r="J7" s="205"/>
+      <c r="J7" s="210"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -22861,7 +22861,7 @@
       <c r="F8" t="s">
         <v>93</v>
       </c>
-      <c r="J8" s="205"/>
+      <c r="J8" s="210"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -22873,7 +22873,7 @@
       <c r="F9" t="s">
         <v>462</v>
       </c>
-      <c r="J9" s="205"/>
+      <c r="J9" s="210"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -22885,7 +22885,7 @@
       <c r="F10" t="s">
         <v>463</v>
       </c>
-      <c r="J10" s="205"/>
+      <c r="J10" s="210"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -22897,7 +22897,7 @@
       <c r="F11" t="s">
         <v>89</v>
       </c>
-      <c r="J11" s="205"/>
+      <c r="J11" s="210"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -22912,7 +22912,7 @@
       <c r="F12" t="s">
         <v>86</v>
       </c>
-      <c r="J12" s="205"/>
+      <c r="J12" s="210"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -22924,7 +22924,7 @@
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="J13" s="205"/>
+      <c r="J13" s="210"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="111" t="s">
@@ -23303,14 +23303,14 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="200" t="s">
+      <c r="A7" s="205" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="200"/>
-      <c r="C7" s="200"/>
-      <c r="D7" s="200"/>
-      <c r="E7" s="200"/>
-      <c r="F7" s="200"/>
+      <c r="B7" s="205"/>
+      <c r="C7" s="205"/>
+      <c r="D7" s="205"/>
+      <c r="E7" s="205"/>
+      <c r="F7" s="205"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
@@ -23399,14 +23399,14 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="200" t="s">
+      <c r="A14" s="205" t="s">
         <v>485</v>
       </c>
-      <c r="B14" s="200"/>
-      <c r="C14" s="200"/>
-      <c r="D14" s="200"/>
-      <c r="E14" s="200"/>
-      <c r="F14" s="200"/>
+      <c r="B14" s="205"/>
+      <c r="C14" s="205"/>
+      <c r="D14" s="205"/>
+      <c r="E14" s="205"/>
+      <c r="F14" s="205"/>
     </row>
     <row r="15" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
@@ -23415,11 +23415,11 @@
       <c r="B15" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="199" t="s">
+      <c r="C15" s="204" t="s">
         <v>470</v>
       </c>
-      <c r="D15" s="199"/>
-      <c r="E15" s="199"/>
+      <c r="D15" s="204"/>
+      <c r="E15" s="204"/>
       <c r="F15" s="11"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -23431,14 +23431,14 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="201" t="s">
+      <c r="A20" s="206" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="201"/>
-      <c r="C20" s="201"/>
-      <c r="D20" s="201"/>
-      <c r="E20" s="201"/>
-      <c r="F20" s="201"/>
+      <c r="B20" s="206"/>
+      <c r="C20" s="206"/>
+      <c r="D20" s="206"/>
+      <c r="E20" s="206"/>
+      <c r="F20" s="206"/>
     </row>
     <row r="21" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -23447,11 +23447,11 @@
       <c r="B21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="199" t="s">
+      <c r="C21" s="204" t="s">
         <v>482</v>
       </c>
-      <c r="D21" s="199"/>
-      <c r="E21" s="199"/>
+      <c r="D21" s="204"/>
+      <c r="E21" s="204"/>
       <c r="F21" s="8" t="s">
         <v>23</v>
       </c>
@@ -23499,14 +23499,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="201" t="s">
+      <c r="A26" s="206" t="s">
         <v>468</v>
       </c>
-      <c r="B26" s="201"/>
-      <c r="C26" s="201"/>
-      <c r="D26" s="201"/>
-      <c r="E26" s="201"/>
-      <c r="F26" s="201"/>
+      <c r="B26" s="206"/>
+      <c r="C26" s="206"/>
+      <c r="D26" s="206"/>
+      <c r="E26" s="206"/>
+      <c r="F26" s="206"/>
     </row>
     <row r="27" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
@@ -23515,11 +23515,11 @@
       <c r="B27" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="199" t="s">
+      <c r="C27" s="204" t="s">
         <v>470</v>
       </c>
-      <c r="D27" s="199"/>
-      <c r="E27" s="199"/>
+      <c r="D27" s="204"/>
+      <c r="E27" s="204"/>
       <c r="F27" s="8"/>
     </row>
   </sheetData>
@@ -24045,7 +24045,7 @@
         <v>45</v>
       </c>
       <c r="B3" s="178" t="s">
-        <v>915</v>
+        <v>958</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -24078,27 +24078,27 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="197" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="206" t="s">
-        <v>919</v>
-      </c>
-      <c r="B6" s="206" t="s">
+      <c r="A6" s="199" t="s">
+        <v>917</v>
+      </c>
+      <c r="B6" s="199" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="206" t="s">
+      <c r="C6" s="199" t="s">
         <v>155</v>
       </c>
-      <c r="D6" s="206" t="s">
+      <c r="D6" s="199" t="s">
         <v>868</v>
       </c>
-      <c r="E6" s="207" t="s">
+      <c r="E6" s="200" t="s">
         <v>55</v>
       </c>
-      <c r="F6" s="206"/>
-      <c r="G6" s="206">
+      <c r="F6" s="199"/>
+      <c r="G6" s="199">
         <v>112</v>
       </c>
-      <c r="H6" s="206" t="s">
-        <v>917</v>
+      <c r="H6" s="199" t="s">
+        <v>915</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -24397,32 +24397,32 @@
       </c>
     </row>
     <row r="6" spans="1:8" s="197" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="206" t="s">
+      <c r="A6" s="199" t="s">
+        <v>916</v>
+      </c>
+      <c r="B6" s="199" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="199" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="199" t="s">
+        <v>868</v>
+      </c>
+      <c r="E6" s="200" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="199"/>
+      <c r="G6" s="199">
+        <v>341</v>
+      </c>
+      <c r="H6" s="199" t="s">
         <v>918</v>
-      </c>
-      <c r="B6" s="206" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="206" t="s">
-        <v>155</v>
-      </c>
-      <c r="D6" s="206" t="s">
-        <v>868</v>
-      </c>
-      <c r="E6" s="207" t="s">
-        <v>55</v>
-      </c>
-      <c r="F6" s="206"/>
-      <c r="G6" s="206">
-        <v>341</v>
-      </c>
-      <c r="H6" s="206" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="145" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B7" s="146" t="s">
         <v>20</v>
@@ -24448,7 +24448,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="145" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B8" s="146" t="s">
         <v>20</v>
@@ -24550,7 +24550,7 @@
         <v>155</v>
       </c>
       <c r="D12" s="152" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="E12" s="95"/>
       <c r="F12" s="98"/>

</xml_diff>